<commit_message>
currently working but is not dynamic and not fitting with other sets. Will need modifications
</commit_message>
<xml_diff>
--- a/Expected Value and Cost Ratio Calculator Pokemon/excelDocs/scarletAndViolet151/pokemon_data.xlsx
+++ b/Expected Value and Cost Ratio Calculator Pokemon/excelDocs/scarletAndViolet151/pokemon_data.xlsx
@@ -3,14 +3,14 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="1350" yWindow="2325" windowWidth="21600" windowHeight="11385" tabRatio="797" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-27375" yWindow="90" windowWidth="25260" windowHeight="11385" tabRatio="797" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Data'!$A$1:$N$210</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Data'!$A$1:$K$210</definedName>
   </definedNames>
   <calcPr calcId="181029" fullCalcOnLoad="1"/>
 </workbook>
@@ -21,7 +21,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -41,10 +41,15 @@
       <sz val="11"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -53,16 +58,36 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFD9D9D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00D9D9D9"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -90,7 +115,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -114,6 +139,18 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -481,7 +518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N1263"/>
+  <dimension ref="A1:K1263"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39.6" customWidth="1" min="1" max="1"/>
@@ -493,9 +530,6 @@
     <col width="33.5703125" customWidth="1" min="7" max="8"/>
     <col width="32.42578125" customWidth="1" min="9" max="10"/>
     <col width="39.42578125" customWidth="1" min="11" max="11"/>
-    <col width="16.85546875" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="6" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -554,21 +588,6 @@
           <t>Current Market Price of ETB Promo Card</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>EV Component</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Total EV</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>EVR</t>
-        </is>
-      </c>
     </row>
     <row r="2" ht="17.25" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
@@ -585,21 +604,21 @@
         <v>46</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06</v>
       </c>
       <c r="E2" s="3" t="n">
         <v>0.15</v>
       </c>
       <c r="F2" s="3">
-        <f>IF(B2="common", 4, IF(B2="uncommon", 3, IF(B2="rare", 1.22, 1)))</f>
+        <f>IF(B2="common", 4, IF(B2="uncommon", 3, IF(B2="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
       <c r="G2">
-        <f>SUMPRODUCT(F2:F210, D2:D210/ C2:C210)</f>
+        <f>SUM(H2:H10)</f>
         <v/>
       </c>
       <c r="H2">
-        <f>SUMPRODUCT((B2:B210="Common") * D2:D210 * F2:F210 / C2:C210)</f>
+        <f>SUMPRODUCT((B2:B217="Common") * D2:D217 * F2:F217 / C2:C217)</f>
         <v/>
       </c>
       <c r="I2" s="3" t="n">
@@ -627,21 +646,17 @@
         <v>21</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>0.16</v>
+        <v>0.2</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>0.7</v>
+        <v>0.55</v>
       </c>
       <c r="F3" s="3">
-        <f>IF(B3="common", 4, IF(B3="uncommon", 3, IF(B3="rare", 1.22, 1)))</f>
-        <v/>
-      </c>
-      <c r="G3">
-        <f>SUM(H2:H9)</f>
+        <f>IF(B3="common", 4, IF(B3="uncommon", 3, IF(B3="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
       <c r="H3">
-        <f>SUMPRODUCT((B2:B210="Uncommon") * D2:D210 * F2:F210 / C2:C210)</f>
+        <f>SUMPRODUCT((B2:B217="Uncommon") * D2:D217 * F2:F217 / C2:C217)</f>
         <v/>
       </c>
     </row>
@@ -660,11 +675,11 @@
         <v>90</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>0.74</v>
+        <v>1.12</v>
       </c>
       <c r="E4" s="3" t="inlineStr"/>
       <c r="F4" s="3">
-        <f>IF(B4="common", 4, IF(B4="uncommon", 3, IF(B4="rare", 1.22, 1)))</f>
+        <f>IF(B4="common", 4, IF(B4="uncommon", 3, IF(B4="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
       <c r="H4">
@@ -687,15 +702,15 @@
         <v>248</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>7.64</v>
+        <v>7.46</v>
       </c>
       <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="3">
-        <f>IF(B5="common", 4, IF(B5="uncommon", 3, IF(B5="rare", 1.22, 1)))</f>
+        <f>IF(B5="common", 4, IF(B5="uncommon", 3, IF(B5="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
       <c r="H5">
-        <f>SUMPRODUCT((B2:B210="Double Rare") * D2:D210 * F2:F210 / C2:C210)</f>
+        <f>SUMPRODUCT((B2:B217="Double Rare") * D2:D217 * F2:F217 / C2:C217)</f>
         <v/>
       </c>
     </row>
@@ -714,11 +729,11 @@
         <v>225</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>39.98</v>
+        <v>43.34</v>
       </c>
       <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="3">
-        <f>IF(B6="common", 4, IF(B6="uncommon", 3, IF(B6="rare", 1.22, 1)))</f>
+        <f>IF(B6="common", 4, IF(B6="uncommon", 3, IF(B6="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
       <c r="H6">
@@ -741,17 +756,17 @@
         <v>46</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>0.1</v>
+        <v>0.08</v>
       </c>
       <c r="E7" s="3" t="n">
         <v>0.64</v>
       </c>
       <c r="F7" s="3">
-        <f>IF(B7="common", 4, IF(B7="uncommon", 3, IF(B7="rare", 1.22, 1)))</f>
+        <f>IF(B7="common", 4, IF(B7="uncommon", 3, IF(B7="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
       <c r="H7">
-        <f>SUMPRODUCT((B2:B210="Illustration Rare") * D2:D210 * F2:F210 / C2:C210)</f>
+        <f>SUMPRODUCT((B2:B217="Illustration Rare") * D2:D217 * F2:F217 / C2:C217)</f>
         <v/>
       </c>
     </row>
@@ -770,17 +785,17 @@
         <v>46</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>0.1</v>
+        <v>0.12</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>1.39</v>
+        <v>1.06</v>
       </c>
       <c r="F8" s="3">
-        <f>IF(B8="common", 4, IF(B8="uncommon", 3, IF(B8="rare", 1.22, 1)))</f>
+        <f>IF(B8="common", 4, IF(B8="uncommon", 3, IF(B8="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
       <c r="H8">
-        <f>SUMPRODUCT((B2:B210="Special Illustration Rare") * D2:D210 * F2:F210 / C2:C210)</f>
+        <f>SUMPRODUCT((B2:B217="Special Illustration Rare") * D2:D217 * F2:F217 / C2:C217)</f>
         <v/>
       </c>
     </row>
@@ -799,17 +814,17 @@
         <v>46</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>0.1</v>
+        <v>0.11</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>0.64</v>
+        <v>0.65</v>
       </c>
       <c r="F9" s="3">
-        <f>IF(B9="common", 4, IF(B9="uncommon", 3, IF(B9="rare", 1.22, 1)))</f>
+        <f>IF(B9="common", 4, IF(B9="uncommon", 3, IF(B9="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
       <c r="H9">
-        <f>SUMPRODUCT((B2:B210="Ultra Rare") * D2:D210 * F2:F210 / C2:C210)</f>
+        <f>SUMPRODUCT((B2:B217="Ultra Rare") * D2:D217 * F2:F217 / C2:C217)</f>
         <v/>
       </c>
     </row>
@@ -828,11 +843,15 @@
         <v>90</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>0.8</v>
+        <v>0.76</v>
       </c>
       <c r="E10" s="3" t="inlineStr"/>
       <c r="F10" s="3">
-        <f>IF(B10="common", 4, IF(B10="uncommon", 3, IF(B10="rare", 1.22, 1)))</f>
+        <f>IF(B10="common", 4, IF(B10="uncommon", 3, IF(B10="rare", 1.74127216869152, 1)))</f>
+        <v/>
+      </c>
+      <c r="H10">
+        <f>1.88 * SUMPRODUCT((C2:C217&lt;&gt;"") * (E2:E217&lt;&gt;"") * (E2:E217 / C2:C217))</f>
         <v/>
       </c>
     </row>
@@ -851,11 +870,11 @@
         <v>248</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>5.46</v>
+        <v>4.89</v>
       </c>
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="3">
-        <f>IF(B11="common", 4, IF(B11="uncommon", 3, IF(B11="rare", 1.22, 1)))</f>
+        <f>IF(B11="common", 4, IF(B11="uncommon", 3, IF(B11="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -874,13 +893,13 @@
         <v>33</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>0.09</v>
+        <v>0.11</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>0.15</v>
+        <v>0.18</v>
       </c>
       <c r="F12" s="3">
-        <f>IF(B12="common", 4, IF(B12="uncommon", 3, IF(B12="rare", 1.22, 1)))</f>
+        <f>IF(B12="common", 4, IF(B12="uncommon", 3, IF(B12="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -899,13 +918,13 @@
         <v>21</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>0.23</v>
+        <v>0.2</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>0.88</v>
+        <v>0.74</v>
       </c>
       <c r="F13" s="3">
-        <f>IF(B13="common", 4, IF(B13="uncommon", 3, IF(B13="rare", 1.22, 1)))</f>
+        <f>IF(B13="common", 4, IF(B13="uncommon", 3, IF(B13="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -924,11 +943,11 @@
         <v>154</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>5.36</v>
+        <v>4.95</v>
       </c>
       <c r="E14" s="3" t="inlineStr"/>
       <c r="F14" s="3">
-        <f>IF(B14="common", 4, IF(B14="uncommon", 3, IF(B14="rare", 1.22, 1)))</f>
+        <f>IF(B14="common", 4, IF(B14="uncommon", 3, IF(B14="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -947,13 +966,13 @@
         <v>21</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>0.14</v>
+        <v>0.16</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>0.7</v>
+        <v>0.75</v>
       </c>
       <c r="F15" s="3">
-        <f>IF(B15="common", 4, IF(B15="uncommon", 3, IF(B15="rare", 1.22, 1)))</f>
+        <f>IF(B15="common", 4, IF(B15="uncommon", 3, IF(B15="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -972,13 +991,13 @@
         <v>46</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>0.06</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="E16" s="3" t="n">
         <v>0.14</v>
       </c>
       <c r="F16" s="3">
-        <f>IF(B16="common", 4, IF(B16="uncommon", 3, IF(B16="rare", 1.22, 1)))</f>
+        <f>IF(B16="common", 4, IF(B16="uncommon", 3, IF(B16="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -997,13 +1016,13 @@
         <v>33</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>0.12</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>1.25</v>
+        <v>1.12</v>
       </c>
       <c r="F17" s="3">
-        <f>IF(B17="common", 4, IF(B17="uncommon", 3, IF(B17="rare", 1.22, 1)))</f>
+        <f>IF(B17="common", 4, IF(B17="uncommon", 3, IF(B17="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -1022,13 +1041,13 @@
         <v>33</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>0.1</v>
+        <v>0.12</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>0.45</v>
+        <v>0.44</v>
       </c>
       <c r="F18" s="3">
-        <f>IF(B18="common", 4, IF(B18="uncommon", 3, IF(B18="rare", 1.22, 1)))</f>
+        <f>IF(B18="common", 4, IF(B18="uncommon", 3, IF(B18="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -1047,11 +1066,11 @@
         <v>248</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>2.77</v>
+        <v>3.05</v>
       </c>
       <c r="E19" s="3" t="inlineStr"/>
       <c r="F19" s="3">
-        <f>IF(B19="common", 4, IF(B19="uncommon", 3, IF(B19="rare", 1.22, 1)))</f>
+        <f>IF(B19="common", 4, IF(B19="uncommon", 3, IF(B19="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -1070,11 +1089,11 @@
         <v>90</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>0.66</v>
+        <v>1.18</v>
       </c>
       <c r="E20" s="3" t="inlineStr"/>
       <c r="F20" s="3">
-        <f>IF(B20="common", 4, IF(B20="uncommon", 3, IF(B20="rare", 1.22, 1)))</f>
+        <f>IF(B20="common", 4, IF(B20="uncommon", 3, IF(B20="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -1093,11 +1112,11 @@
         <v>248</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>14.54</v>
+        <v>14.89</v>
       </c>
       <c r="E21" s="3" t="inlineStr"/>
       <c r="F21" s="3">
-        <f>IF(B21="common", 4, IF(B21="uncommon", 3, IF(B21="rare", 1.22, 1)))</f>
+        <f>IF(B21="common", 4, IF(B21="uncommon", 3, IF(B21="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -1116,11 +1135,11 @@
         <v>225</v>
       </c>
       <c r="D22" s="3" t="n">
-        <v>70.20999999999999</v>
+        <v>73.55</v>
       </c>
       <c r="E22" s="3" t="inlineStr"/>
       <c r="F22" s="3">
-        <f>IF(B22="common", 4, IF(B22="uncommon", 3, IF(B22="rare", 1.22, 1)))</f>
+        <f>IF(B22="common", 4, IF(B22="uncommon", 3, IF(B22="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -1139,13 +1158,13 @@
         <v>46</v>
       </c>
       <c r="D23" s="3" t="n">
-        <v>0.12</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="E23" s="3" t="n">
-        <v>0.2</v>
+        <v>0.24</v>
       </c>
       <c r="F23" s="3">
-        <f>IF(B23="common", 4, IF(B23="uncommon", 3, IF(B23="rare", 1.22, 1)))</f>
+        <f>IF(B23="common", 4, IF(B23="uncommon", 3, IF(B23="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -1164,11 +1183,11 @@
         <v>188</v>
       </c>
       <c r="D24" s="3" t="n">
-        <v>37.17</v>
+        <v>37.52</v>
       </c>
       <c r="E24" s="3" t="inlineStr"/>
       <c r="F24" s="3">
-        <f>IF(B24="common", 4, IF(B24="uncommon", 3, IF(B24="rare", 1.22, 1)))</f>
+        <f>IF(B24="common", 4, IF(B24="uncommon", 3, IF(B24="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -1187,13 +1206,13 @@
         <v>33</v>
       </c>
       <c r="D25" s="3" t="n">
-        <v>0.06</v>
+        <v>0.1</v>
       </c>
       <c r="E25" s="3" t="n">
-        <v>0.18</v>
+        <v>0.16</v>
       </c>
       <c r="F25" s="3">
-        <f>IF(B25="common", 4, IF(B25="uncommon", 3, IF(B25="rare", 1.22, 1)))</f>
+        <f>IF(B25="common", 4, IF(B25="uncommon", 3, IF(B25="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -1212,13 +1231,13 @@
         <v>46</v>
       </c>
       <c r="D26" s="3" t="n">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="E26" s="3" t="n">
-        <v>0.13</v>
+        <v>0.21</v>
       </c>
       <c r="F26" s="3">
-        <f>IF(B26="common", 4, IF(B26="uncommon", 3, IF(B26="rare", 1.22, 1)))</f>
+        <f>IF(B26="common", 4, IF(B26="uncommon", 3, IF(B26="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -1237,11 +1256,11 @@
         <v>188</v>
       </c>
       <c r="D27" s="3" t="n">
-        <v>9.66</v>
+        <v>9.56</v>
       </c>
       <c r="E27" s="3" t="inlineStr"/>
       <c r="F27" s="3">
-        <f>IF(B27="common", 4, IF(B27="uncommon", 3, IF(B27="rare", 1.22, 1)))</f>
+        <f>IF(B27="common", 4, IF(B27="uncommon", 3, IF(B27="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -1260,13 +1279,13 @@
         <v>21</v>
       </c>
       <c r="D28" s="3" t="n">
-        <v>0.17</v>
+        <v>0.15</v>
       </c>
       <c r="E28" s="3" t="n">
-        <v>0.86</v>
+        <v>0.65</v>
       </c>
       <c r="F28" s="3">
-        <f>IF(B28="common", 4, IF(B28="uncommon", 3, IF(B28="rare", 1.22, 1)))</f>
+        <f>IF(B28="common", 4, IF(B28="uncommon", 3, IF(B28="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -1285,11 +1304,11 @@
         <v>90</v>
       </c>
       <c r="D29" s="3" t="n">
-        <v>4.54</v>
+        <v>4.71</v>
       </c>
       <c r="E29" s="3" t="inlineStr"/>
       <c r="F29" s="3">
-        <f>IF(B29="common", 4, IF(B29="uncommon", 3, IF(B29="rare", 1.22, 1)))</f>
+        <f>IF(B29="common", 4, IF(B29="uncommon", 3, IF(B29="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -1308,11 +1327,11 @@
         <v>248</v>
       </c>
       <c r="D30" s="3" t="n">
-        <v>29.54</v>
+        <v>31.27</v>
       </c>
       <c r="E30" s="3" t="inlineStr"/>
       <c r="F30" s="3">
-        <f>IF(B30="common", 4, IF(B30="uncommon", 3, IF(B30="rare", 1.22, 1)))</f>
+        <f>IF(B30="common", 4, IF(B30="uncommon", 3, IF(B30="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -1331,11 +1350,11 @@
         <v>225</v>
       </c>
       <c r="D31" s="3" t="n">
-        <v>210.03</v>
+        <v>210.14</v>
       </c>
       <c r="E31" s="3" t="inlineStr"/>
       <c r="F31" s="3">
-        <f>IF(B31="common", 4, IF(B31="uncommon", 3, IF(B31="rare", 1.22, 1)))</f>
+        <f>IF(B31="common", 4, IF(B31="uncommon", 3, IF(B31="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -1354,13 +1373,13 @@
         <v>46</v>
       </c>
       <c r="D32" s="3" t="n">
-        <v>0.1</v>
+        <v>0.08</v>
       </c>
       <c r="E32" s="3" t="n">
         <v>0.19</v>
       </c>
       <c r="F32" s="3">
-        <f>IF(B32="common", 4, IF(B32="uncommon", 3, IF(B32="rare", 1.22, 1)))</f>
+        <f>IF(B32="common", 4, IF(B32="uncommon", 3, IF(B32="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -1379,11 +1398,11 @@
         <v>188</v>
       </c>
       <c r="D33" s="3" t="n">
-        <v>46.71</v>
+        <v>52.06</v>
       </c>
       <c r="E33" s="3" t="inlineStr"/>
       <c r="F33" s="3">
-        <f>IF(B33="common", 4, IF(B33="uncommon", 3, IF(B33="rare", 1.22, 1)))</f>
+        <f>IF(B33="common", 4, IF(B33="uncommon", 3, IF(B33="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -1405,10 +1424,10 @@
         <v>0.1</v>
       </c>
       <c r="E34" s="3" t="n">
-        <v>0.2</v>
+        <v>0.23</v>
       </c>
       <c r="F34" s="3">
-        <f>IF(B34="common", 4, IF(B34="uncommon", 3, IF(B34="rare", 1.22, 1)))</f>
+        <f>IF(B34="common", 4, IF(B34="uncommon", 3, IF(B34="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -1427,11 +1446,11 @@
         <v>188</v>
       </c>
       <c r="D35" s="3" t="n">
-        <v>32.96</v>
+        <v>34.86</v>
       </c>
       <c r="E35" s="3" t="inlineStr"/>
       <c r="F35" s="3">
-        <f>IF(B35="common", 4, IF(B35="uncommon", 3, IF(B35="rare", 1.22, 1)))</f>
+        <f>IF(B35="common", 4, IF(B35="uncommon", 3, IF(B35="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -1450,13 +1469,13 @@
         <v>33</v>
       </c>
       <c r="D36" s="3" t="n">
-        <v>0.06</v>
+        <v>0.08</v>
       </c>
       <c r="E36" s="3" t="n">
-        <v>0.17</v>
+        <v>0.19</v>
       </c>
       <c r="F36" s="3">
-        <f>IF(B36="common", 4, IF(B36="uncommon", 3, IF(B36="rare", 1.22, 1)))</f>
+        <f>IF(B36="common", 4, IF(B36="uncommon", 3, IF(B36="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -1475,13 +1494,13 @@
         <v>46</v>
       </c>
       <c r="D37" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.08</v>
       </c>
       <c r="E37" s="3" t="n">
-        <v>0.14</v>
+        <v>0.16</v>
       </c>
       <c r="F37" s="3">
-        <f>IF(B37="common", 4, IF(B37="uncommon", 3, IF(B37="rare", 1.22, 1)))</f>
+        <f>IF(B37="common", 4, IF(B37="uncommon", 3, IF(B37="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -1500,13 +1519,13 @@
         <v>33</v>
       </c>
       <c r="D38" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.08</v>
       </c>
       <c r="E38" s="3" t="n">
-        <v>0.17</v>
+        <v>0.15</v>
       </c>
       <c r="F38" s="3">
-        <f>IF(B38="common", 4, IF(B38="uncommon", 3, IF(B38="rare", 1.22, 1)))</f>
+        <f>IF(B38="common", 4, IF(B38="uncommon", 3, IF(B38="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -1525,13 +1544,13 @@
         <v>46</v>
       </c>
       <c r="D39" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.11</v>
       </c>
       <c r="E39" s="3" t="n">
-        <v>0.18</v>
+        <v>0.14</v>
       </c>
       <c r="F39" s="3">
-        <f>IF(B39="common", 4, IF(B39="uncommon", 3, IF(B39="rare", 1.22, 1)))</f>
+        <f>IF(B39="common", 4, IF(B39="uncommon", 3, IF(B39="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -1550,13 +1569,13 @@
         <v>33</v>
       </c>
       <c r="D40" s="3" t="n">
-        <v>0.08</v>
+        <v>0.1</v>
       </c>
       <c r="E40" s="3" t="n">
-        <v>0.61</v>
+        <v>0.59</v>
       </c>
       <c r="F40" s="3">
-        <f>IF(B40="common", 4, IF(B40="uncommon", 3, IF(B40="rare", 1.22, 1)))</f>
+        <f>IF(B40="common", 4, IF(B40="uncommon", 3, IF(B40="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -1578,10 +1597,10 @@
         <v>0.09</v>
       </c>
       <c r="E41" s="3" t="n">
-        <v>0.48</v>
+        <v>0.43</v>
       </c>
       <c r="F41" s="3">
-        <f>IF(B41="common", 4, IF(B41="uncommon", 3, IF(B41="rare", 1.22, 1)))</f>
+        <f>IF(B41="common", 4, IF(B41="uncommon", 3, IF(B41="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -1600,11 +1619,11 @@
         <v>248</v>
       </c>
       <c r="D42" s="3" t="n">
-        <v>3.42</v>
+        <v>4.04</v>
       </c>
       <c r="E42" s="3" t="inlineStr"/>
       <c r="F42" s="3">
-        <f>IF(B42="common", 4, IF(B42="uncommon", 3, IF(B42="rare", 1.22, 1)))</f>
+        <f>IF(B42="common", 4, IF(B42="uncommon", 3, IF(B42="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -1626,10 +1645,10 @@
         <v>0.06</v>
       </c>
       <c r="E43" s="3" t="n">
-        <v>0.15</v>
+        <v>0.14</v>
       </c>
       <c r="F43" s="3">
-        <f>IF(B43="common", 4, IF(B43="uncommon", 3, IF(B43="rare", 1.22, 1)))</f>
+        <f>IF(B43="common", 4, IF(B43="uncommon", 3, IF(B43="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -1651,10 +1670,10 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="E44" s="3" t="n">
-        <v>0.12</v>
+        <v>0.15</v>
       </c>
       <c r="F44" s="3">
-        <f>IF(B44="common", 4, IF(B44="uncommon", 3, IF(B44="rare", 1.22, 1)))</f>
+        <f>IF(B44="common", 4, IF(B44="uncommon", 3, IF(B44="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -1673,13 +1692,13 @@
         <v>21</v>
       </c>
       <c r="D45" s="3" t="n">
-        <v>0.28</v>
+        <v>0.26</v>
       </c>
       <c r="E45" s="3" t="n">
-        <v>0.84</v>
+        <v>0.64</v>
       </c>
       <c r="F45" s="3">
-        <f>IF(B45="common", 4, IF(B45="uncommon", 3, IF(B45="rare", 1.22, 1)))</f>
+        <f>IF(B45="common", 4, IF(B45="uncommon", 3, IF(B45="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -1698,11 +1717,11 @@
         <v>21</v>
       </c>
       <c r="D46" s="3" t="n">
-        <v>0.33</v>
+        <v>0.34</v>
       </c>
       <c r="E46" s="3" t="inlineStr"/>
       <c r="F46" s="3">
-        <f>IF(B46="common", 4, IF(B46="uncommon", 3, IF(B46="rare", 1.22, 1)))</f>
+        <f>IF(B46="common", 4, IF(B46="uncommon", 3, IF(B46="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -1724,10 +1743,10 @@
         <v>0.14</v>
       </c>
       <c r="E47" s="3" t="n">
-        <v>0.68</v>
+        <v>0.63</v>
       </c>
       <c r="F47" s="3">
-        <f>IF(B47="common", 4, IF(B47="uncommon", 3, IF(B47="rare", 1.22, 1)))</f>
+        <f>IF(B47="common", 4, IF(B47="uncommon", 3, IF(B47="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -1749,10 +1768,10 @@
         <v>0.06</v>
       </c>
       <c r="E48" s="3" t="n">
-        <v>0.16</v>
+        <v>0.19</v>
       </c>
       <c r="F48" s="3">
-        <f>IF(B48="common", 4, IF(B48="uncommon", 3, IF(B48="rare", 1.22, 1)))</f>
+        <f>IF(B48="common", 4, IF(B48="uncommon", 3, IF(B48="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -1774,10 +1793,10 @@
         <v>0.11</v>
       </c>
       <c r="E49" s="3" t="n">
-        <v>1.86</v>
+        <v>2</v>
       </c>
       <c r="F49" s="3">
-        <f>IF(B49="common", 4, IF(B49="uncommon", 3, IF(B49="rare", 1.22, 1)))</f>
+        <f>IF(B49="common", 4, IF(B49="uncommon", 3, IF(B49="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -1796,11 +1815,11 @@
         <v>188</v>
       </c>
       <c r="D50" s="3" t="n">
-        <v>22.83</v>
+        <v>25.78</v>
       </c>
       <c r="E50" s="3" t="inlineStr"/>
       <c r="F50" s="3">
-        <f>IF(B50="common", 4, IF(B50="uncommon", 3, IF(B50="rare", 1.22, 1)))</f>
+        <f>IF(B50="common", 4, IF(B50="uncommon", 3, IF(B50="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -1819,13 +1838,13 @@
         <v>21</v>
       </c>
       <c r="D51" s="3" t="n">
-        <v>0.32</v>
+        <v>0.41</v>
       </c>
       <c r="E51" s="3" t="n">
-        <v>1.54</v>
+        <v>1.32</v>
       </c>
       <c r="F51" s="3">
-        <f>IF(B51="common", 4, IF(B51="uncommon", 3, IF(B51="rare", 1.22, 1)))</f>
+        <f>IF(B51="common", 4, IF(B51="uncommon", 3, IF(B51="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -1844,13 +1863,13 @@
         <v>46</v>
       </c>
       <c r="D52" s="3" t="n">
-        <v>0.09</v>
+        <v>0.11</v>
       </c>
       <c r="E52" s="3" t="n">
-        <v>0.19</v>
+        <v>0.18</v>
       </c>
       <c r="F52" s="3">
-        <f>IF(B52="common", 4, IF(B52="uncommon", 3, IF(B52="rare", 1.22, 1)))</f>
+        <f>IF(B52="common", 4, IF(B52="uncommon", 3, IF(B52="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -1869,13 +1888,13 @@
         <v>46</v>
       </c>
       <c r="D53" s="3" t="n">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="E53" s="3" t="n">
-        <v>0.12</v>
+        <v>0.13</v>
       </c>
       <c r="F53" s="3">
-        <f>IF(B53="common", 4, IF(B53="uncommon", 3, IF(B53="rare", 1.22, 1)))</f>
+        <f>IF(B53="common", 4, IF(B53="uncommon", 3, IF(B53="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -1897,10 +1916,10 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="E54" s="3" t="n">
-        <v>0.31</v>
+        <v>0.13</v>
       </c>
       <c r="F54" s="3">
-        <f>IF(B54="common", 4, IF(B54="uncommon", 3, IF(B54="rare", 1.22, 1)))</f>
+        <f>IF(B54="common", 4, IF(B54="uncommon", 3, IF(B54="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -1919,13 +1938,13 @@
         <v>46</v>
       </c>
       <c r="D55" s="3" t="n">
-        <v>0.12</v>
+        <v>0.09</v>
       </c>
       <c r="E55" s="3" t="n">
-        <v>0.21</v>
+        <v>0.24</v>
       </c>
       <c r="F55" s="3">
-        <f>IF(B55="common", 4, IF(B55="uncommon", 3, IF(B55="rare", 1.22, 1)))</f>
+        <f>IF(B55="common", 4, IF(B55="uncommon", 3, IF(B55="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -1944,13 +1963,13 @@
         <v>46</v>
       </c>
       <c r="D56" s="3" t="n">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="E56" s="3" t="n">
-        <v>0.18</v>
+        <v>0.2</v>
       </c>
       <c r="F56" s="3">
-        <f>IF(B56="common", 4, IF(B56="uncommon", 3, IF(B56="rare", 1.22, 1)))</f>
+        <f>IF(B56="common", 4, IF(B56="uncommon", 3, IF(B56="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -1969,13 +1988,13 @@
         <v>46</v>
       </c>
       <c r="D57" s="3" t="n">
-        <v>0.09</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="E57" s="3" t="n">
-        <v>0.52</v>
+        <v>0.5</v>
       </c>
       <c r="F57" s="3">
-        <f>IF(B57="common", 4, IF(B57="uncommon", 3, IF(B57="rare", 1.22, 1)))</f>
+        <f>IF(B57="common", 4, IF(B57="uncommon", 3, IF(B57="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -1997,10 +2016,10 @@
         <v>0.13</v>
       </c>
       <c r="E58" s="3" t="n">
-        <v>1.68</v>
+        <v>1.27</v>
       </c>
       <c r="F58" s="3">
-        <f>IF(B58="common", 4, IF(B58="uncommon", 3, IF(B58="rare", 1.22, 1)))</f>
+        <f>IF(B58="common", 4, IF(B58="uncommon", 3, IF(B58="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -2019,13 +2038,13 @@
         <v>33</v>
       </c>
       <c r="D59" s="3" t="n">
-        <v>0.15</v>
+        <v>0.16</v>
       </c>
       <c r="E59" s="3" t="n">
-        <v>1.4</v>
+        <v>1.41</v>
       </c>
       <c r="F59" s="3">
-        <f>IF(B59="common", 4, IF(B59="uncommon", 3, IF(B59="rare", 1.22, 1)))</f>
+        <f>IF(B59="common", 4, IF(B59="uncommon", 3, IF(B59="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -2044,13 +2063,13 @@
         <v>33</v>
       </c>
       <c r="D60" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.11</v>
       </c>
       <c r="E60" s="3" t="n">
-        <v>0.92</v>
+        <v>0.8</v>
       </c>
       <c r="F60" s="3">
-        <f>IF(B60="common", 4, IF(B60="uncommon", 3, IF(B60="rare", 1.22, 1)))</f>
+        <f>IF(B60="common", 4, IF(B60="uncommon", 3, IF(B60="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -2069,11 +2088,11 @@
         <v>248</v>
       </c>
       <c r="D61" s="3" t="n">
-        <v>6.39</v>
+        <v>6.99</v>
       </c>
       <c r="E61" s="3" t="inlineStr"/>
       <c r="F61" s="3">
-        <f>IF(B61="common", 4, IF(B61="uncommon", 3, IF(B61="rare", 1.22, 1)))</f>
+        <f>IF(B61="common", 4, IF(B61="uncommon", 3, IF(B61="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -2092,11 +2111,11 @@
         <v>225</v>
       </c>
       <c r="D62" s="3" t="n">
-        <v>14.75</v>
+        <v>14.98</v>
       </c>
       <c r="E62" s="3" t="inlineStr"/>
       <c r="F62" s="3">
-        <f>IF(B62="common", 4, IF(B62="uncommon", 3, IF(B62="rare", 1.22, 1)))</f>
+        <f>IF(B62="common", 4, IF(B62="uncommon", 3, IF(B62="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -2118,10 +2137,10 @@
         <v>0.05</v>
       </c>
       <c r="E63" s="3" t="n">
-        <v>0.16</v>
+        <v>0.12</v>
       </c>
       <c r="F63" s="3">
-        <f>IF(B63="common", 4, IF(B63="uncommon", 3, IF(B63="rare", 1.22, 1)))</f>
+        <f>IF(B63="common", 4, IF(B63="uncommon", 3, IF(B63="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -2140,13 +2159,13 @@
         <v>33</v>
       </c>
       <c r="D64" s="3" t="n">
-        <v>0.08</v>
+        <v>0.1</v>
       </c>
       <c r="E64" s="3" t="n">
-        <v>1.46</v>
+        <v>1.26</v>
       </c>
       <c r="F64" s="3">
-        <f>IF(B64="common", 4, IF(B64="uncommon", 3, IF(B64="rare", 1.22, 1)))</f>
+        <f>IF(B64="common", 4, IF(B64="uncommon", 3, IF(B64="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -2165,13 +2184,13 @@
         <v>46</v>
       </c>
       <c r="D65" s="3" t="n">
-        <v>0.06</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="E65" s="3" t="n">
-        <v>0.14</v>
+        <v>0.13</v>
       </c>
       <c r="F65" s="3">
-        <f>IF(B65="common", 4, IF(B65="uncommon", 3, IF(B65="rare", 1.22, 1)))</f>
+        <f>IF(B65="common", 4, IF(B65="uncommon", 3, IF(B65="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -2190,13 +2209,13 @@
         <v>33</v>
       </c>
       <c r="D66" s="3" t="n">
-        <v>0.06</v>
+        <v>0.08</v>
       </c>
       <c r="E66" s="3" t="n">
-        <v>0.12</v>
+        <v>0.14</v>
       </c>
       <c r="F66" s="3">
-        <f>IF(B66="common", 4, IF(B66="uncommon", 3, IF(B66="rare", 1.22, 1)))</f>
+        <f>IF(B66="common", 4, IF(B66="uncommon", 3, IF(B66="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -2215,13 +2234,13 @@
         <v>21</v>
       </c>
       <c r="D67" s="3" t="n">
-        <v>0.26</v>
+        <v>0.25</v>
       </c>
       <c r="E67" s="3" t="n">
-        <v>1.11</v>
+        <v>1.08</v>
       </c>
       <c r="F67" s="3">
-        <f>IF(B67="common", 4, IF(B67="uncommon", 3, IF(B67="rare", 1.22, 1)))</f>
+        <f>IF(B67="common", 4, IF(B67="uncommon", 3, IF(B67="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -2240,13 +2259,13 @@
         <v>46</v>
       </c>
       <c r="D68" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.08</v>
       </c>
       <c r="E68" s="3" t="n">
-        <v>0.17</v>
+        <v>0.18</v>
       </c>
       <c r="F68" s="3">
-        <f>IF(B68="common", 4, IF(B68="uncommon", 3, IF(B68="rare", 1.22, 1)))</f>
+        <f>IF(B68="common", 4, IF(B68="uncommon", 3, IF(B68="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -2265,13 +2284,13 @@
         <v>21</v>
       </c>
       <c r="D69" s="3" t="n">
-        <v>0.38</v>
+        <v>0.27</v>
       </c>
       <c r="E69" s="3" t="n">
-        <v>1.89</v>
+        <v>1.78</v>
       </c>
       <c r="F69" s="3">
-        <f>IF(B69="common", 4, IF(B69="uncommon", 3, IF(B69="rare", 1.22, 1)))</f>
+        <f>IF(B69="common", 4, IF(B69="uncommon", 3, IF(B69="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -2296,7 +2315,7 @@
         <v>0.15</v>
       </c>
       <c r="F70" s="3">
-        <f>IF(B70="common", 4, IF(B70="uncommon", 3, IF(B70="rare", 1.22, 1)))</f>
+        <f>IF(B70="common", 4, IF(B70="uncommon", 3, IF(B70="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -2315,13 +2334,13 @@
         <v>33</v>
       </c>
       <c r="D71" s="3" t="n">
-        <v>0.13</v>
+        <v>0.1</v>
       </c>
       <c r="E71" s="3" t="n">
-        <v>1.34</v>
+        <v>1.03</v>
       </c>
       <c r="F71" s="3">
-        <f>IF(B71="common", 4, IF(B71="uncommon", 3, IF(B71="rare", 1.22, 1)))</f>
+        <f>IF(B71="common", 4, IF(B71="uncommon", 3, IF(B71="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -2340,11 +2359,11 @@
         <v>248</v>
       </c>
       <c r="D72" s="3" t="n">
-        <v>4.81</v>
+        <v>4.99</v>
       </c>
       <c r="E72" s="3" t="inlineStr"/>
       <c r="F72" s="3">
-        <f>IF(B72="common", 4, IF(B72="uncommon", 3, IF(B72="rare", 1.22, 1)))</f>
+        <f>IF(B72="common", 4, IF(B72="uncommon", 3, IF(B72="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -2363,11 +2382,11 @@
         <v>225</v>
       </c>
       <c r="D73" s="3" t="n">
-        <v>13.81</v>
+        <v>15.6</v>
       </c>
       <c r="E73" s="3" t="inlineStr"/>
       <c r="F73" s="3">
-        <f>IF(B73="common", 4, IF(B73="uncommon", 3, IF(B73="rare", 1.22, 1)))</f>
+        <f>IF(B73="common", 4, IF(B73="uncommon", 3, IF(B73="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -2386,13 +2405,13 @@
         <v>33</v>
       </c>
       <c r="D74" s="3" t="n">
-        <v>0.05</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="E74" s="3" t="n">
-        <v>0.17</v>
+        <v>0.21</v>
       </c>
       <c r="F74" s="3">
-        <f>IF(B74="common", 4, IF(B74="uncommon", 3, IF(B74="rare", 1.22, 1)))</f>
+        <f>IF(B74="common", 4, IF(B74="uncommon", 3, IF(B74="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -2417,7 +2436,7 @@
         <v>0.18</v>
       </c>
       <c r="F75" s="3">
-        <f>IF(B75="common", 4, IF(B75="uncommon", 3, IF(B75="rare", 1.22, 1)))</f>
+        <f>IF(B75="common", 4, IF(B75="uncommon", 3, IF(B75="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -2436,13 +2455,13 @@
         <v>46</v>
       </c>
       <c r="D76" s="3" t="n">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="E76" s="3" t="n">
-        <v>0.15</v>
+        <v>0.16</v>
       </c>
       <c r="F76" s="3">
-        <f>IF(B76="common", 4, IF(B76="uncommon", 3, IF(B76="rare", 1.22, 1)))</f>
+        <f>IF(B76="common", 4, IF(B76="uncommon", 3, IF(B76="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -2461,13 +2480,13 @@
         <v>33</v>
       </c>
       <c r="D77" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06</v>
       </c>
       <c r="E77" s="3" t="n">
-        <v>0.16</v>
+        <v>0.18</v>
       </c>
       <c r="F77" s="3">
-        <f>IF(B77="common", 4, IF(B77="uncommon", 3, IF(B77="rare", 1.22, 1)))</f>
+        <f>IF(B77="common", 4, IF(B77="uncommon", 3, IF(B77="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -2486,11 +2505,11 @@
         <v>90</v>
       </c>
       <c r="D78" s="3" t="n">
-        <v>0.8</v>
+        <v>0.62</v>
       </c>
       <c r="E78" s="3" t="inlineStr"/>
       <c r="F78" s="3">
-        <f>IF(B78="common", 4, IF(B78="uncommon", 3, IF(B78="rare", 1.22, 1)))</f>
+        <f>IF(B78="common", 4, IF(B78="uncommon", 3, IF(B78="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -2509,11 +2528,11 @@
         <v>248</v>
       </c>
       <c r="D79" s="3" t="n">
-        <v>5.64</v>
+        <v>5.18</v>
       </c>
       <c r="E79" s="3" t="inlineStr"/>
       <c r="F79" s="3">
-        <f>IF(B79="common", 4, IF(B79="uncommon", 3, IF(B79="rare", 1.22, 1)))</f>
+        <f>IF(B79="common", 4, IF(B79="uncommon", 3, IF(B79="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -2532,13 +2551,13 @@
         <v>33</v>
       </c>
       <c r="D80" s="3" t="n">
-        <v>0.15</v>
+        <v>0.26</v>
       </c>
       <c r="E80" s="3" t="n">
-        <v>0.84</v>
+        <v>0.73</v>
       </c>
       <c r="F80" s="3">
-        <f>IF(B80="common", 4, IF(B80="uncommon", 3, IF(B80="rare", 1.22, 1)))</f>
+        <f>IF(B80="common", 4, IF(B80="uncommon", 3, IF(B80="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -2557,13 +2576,13 @@
         <v>33</v>
       </c>
       <c r="D81" s="3" t="n">
-        <v>0.08</v>
+        <v>0.06</v>
       </c>
       <c r="E81" s="3" t="n">
-        <v>0.17</v>
+        <v>0.15</v>
       </c>
       <c r="F81" s="3">
-        <f>IF(B81="common", 4, IF(B81="uncommon", 3, IF(B81="rare", 1.22, 1)))</f>
+        <f>IF(B81="common", 4, IF(B81="uncommon", 3, IF(B81="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -2582,13 +2601,13 @@
         <v>46</v>
       </c>
       <c r="D82" s="3" t="n">
-        <v>0.05</v>
+        <v>0.06</v>
       </c>
       <c r="E82" s="3" t="n">
-        <v>0.16</v>
+        <v>0.15</v>
       </c>
       <c r="F82" s="3">
-        <f>IF(B82="common", 4, IF(B82="uncommon", 3, IF(B82="rare", 1.22, 1)))</f>
+        <f>IF(B82="common", 4, IF(B82="uncommon", 3, IF(B82="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -2607,13 +2626,13 @@
         <v>46</v>
       </c>
       <c r="D83" s="3" t="n">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="E83" s="3" t="n">
-        <v>0.22</v>
+        <v>0.14</v>
       </c>
       <c r="F83" s="3">
-        <f>IF(B83="common", 4, IF(B83="uncommon", 3, IF(B83="rare", 1.22, 1)))</f>
+        <f>IF(B83="common", 4, IF(B83="uncommon", 3, IF(B83="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -2632,13 +2651,13 @@
         <v>21</v>
       </c>
       <c r="D84" s="3" t="n">
-        <v>0.16</v>
+        <v>0.19</v>
       </c>
       <c r="E84" s="3" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.76</v>
       </c>
       <c r="F84" s="3">
-        <f>IF(B84="common", 4, IF(B84="uncommon", 3, IF(B84="rare", 1.22, 1)))</f>
+        <f>IF(B84="common", 4, IF(B84="uncommon", 3, IF(B84="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -2660,10 +2679,10 @@
         <v>0.1</v>
       </c>
       <c r="E85" s="3" t="n">
-        <v>0.25</v>
+        <v>0.21</v>
       </c>
       <c r="F85" s="3">
-        <f>IF(B85="common", 4, IF(B85="uncommon", 3, IF(B85="rare", 1.22, 1)))</f>
+        <f>IF(B85="common", 4, IF(B85="uncommon", 3, IF(B85="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -2682,13 +2701,13 @@
         <v>33</v>
       </c>
       <c r="D86" s="3" t="n">
-        <v>0.08</v>
+        <v>0.09</v>
       </c>
       <c r="E86" s="3" t="n">
-        <v>1.73</v>
+        <v>1.5</v>
       </c>
       <c r="F86" s="3">
-        <f>IF(B86="common", 4, IF(B86="uncommon", 3, IF(B86="rare", 1.22, 1)))</f>
+        <f>IF(B86="common", 4, IF(B86="uncommon", 3, IF(B86="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -2710,10 +2729,10 @@
         <v>0.08</v>
       </c>
       <c r="E87" s="3" t="n">
-        <v>1.46</v>
+        <v>1.12</v>
       </c>
       <c r="F87" s="3">
-        <f>IF(B87="common", 4, IF(B87="uncommon", 3, IF(B87="rare", 1.22, 1)))</f>
+        <f>IF(B87="common", 4, IF(B87="uncommon", 3, IF(B87="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -2732,13 +2751,13 @@
         <v>46</v>
       </c>
       <c r="D88" s="3" t="n">
-        <v>0.05</v>
+        <v>0.06</v>
       </c>
       <c r="E88" s="3" t="n">
-        <v>0.15</v>
+        <v>0.14</v>
       </c>
       <c r="F88" s="3">
-        <f>IF(B88="common", 4, IF(B88="uncommon", 3, IF(B88="rare", 1.22, 1)))</f>
+        <f>IF(B88="common", 4, IF(B88="uncommon", 3, IF(B88="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -2757,13 +2776,13 @@
         <v>33</v>
       </c>
       <c r="D89" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.1</v>
       </c>
       <c r="E89" s="3" t="n">
-        <v>1.59</v>
+        <v>1.3</v>
       </c>
       <c r="F89" s="3">
-        <f>IF(B89="common", 4, IF(B89="uncommon", 3, IF(B89="rare", 1.22, 1)))</f>
+        <f>IF(B89="common", 4, IF(B89="uncommon", 3, IF(B89="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -2782,13 +2801,13 @@
         <v>33</v>
       </c>
       <c r="D90" s="3" t="n">
-        <v>0.14</v>
+        <v>0.12</v>
       </c>
       <c r="E90" s="3" t="n">
-        <v>0.27</v>
+        <v>0.28</v>
       </c>
       <c r="F90" s="3">
-        <f>IF(B90="common", 4, IF(B90="uncommon", 3, IF(B90="rare", 1.22, 1)))</f>
+        <f>IF(B90="common", 4, IF(B90="uncommon", 3, IF(B90="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -2807,11 +2826,11 @@
         <v>188</v>
       </c>
       <c r="D91" s="3" t="n">
-        <v>26.54</v>
+        <v>26.26</v>
       </c>
       <c r="E91" s="3" t="inlineStr"/>
       <c r="F91" s="3">
-        <f>IF(B91="common", 4, IF(B91="uncommon", 3, IF(B91="rare", 1.22, 1)))</f>
+        <f>IF(B91="common", 4, IF(B91="uncommon", 3, IF(B91="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -2830,13 +2849,13 @@
         <v>46</v>
       </c>
       <c r="D92" s="3" t="n">
-        <v>0.08</v>
+        <v>0.09</v>
       </c>
       <c r="E92" s="3" t="n">
         <v>0.22</v>
       </c>
       <c r="F92" s="3">
-        <f>IF(B92="common", 4, IF(B92="uncommon", 3, IF(B92="rare", 1.22, 1)))</f>
+        <f>IF(B92="common", 4, IF(B92="uncommon", 3, IF(B92="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -2855,13 +2874,13 @@
         <v>21</v>
       </c>
       <c r="D93" s="3" t="n">
-        <v>0.24</v>
+        <v>0.25</v>
       </c>
       <c r="E93" s="3" t="n">
-        <v>1.66</v>
+        <v>2.24</v>
       </c>
       <c r="F93" s="3">
-        <f>IF(B93="common", 4, IF(B93="uncommon", 3, IF(B93="rare", 1.22, 1)))</f>
+        <f>IF(B93="common", 4, IF(B93="uncommon", 3, IF(B93="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -2880,11 +2899,11 @@
         <v>90</v>
       </c>
       <c r="D94" s="3" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="E94" s="3" t="inlineStr"/>
       <c r="F94" s="3">
-        <f>IF(B94="common", 4, IF(B94="uncommon", 3, IF(B94="rare", 1.22, 1)))</f>
+        <f>IF(B94="common", 4, IF(B94="uncommon", 3, IF(B94="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -2903,11 +2922,11 @@
         <v>248</v>
       </c>
       <c r="D95" s="3" t="n">
-        <v>4.76</v>
+        <v>5.3</v>
       </c>
       <c r="E95" s="3" t="inlineStr"/>
       <c r="F95" s="3">
-        <f>IF(B95="common", 4, IF(B95="uncommon", 3, IF(B95="rare", 1.22, 1)))</f>
+        <f>IF(B95="common", 4, IF(B95="uncommon", 3, IF(B95="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -2926,13 +2945,13 @@
         <v>33</v>
       </c>
       <c r="D96" s="3" t="n">
-        <v>0.06</v>
+        <v>0.09</v>
       </c>
       <c r="E96" s="3" t="n">
-        <v>1.37</v>
+        <v>1.12</v>
       </c>
       <c r="F96" s="3">
-        <f>IF(B96="common", 4, IF(B96="uncommon", 3, IF(B96="rare", 1.22, 1)))</f>
+        <f>IF(B96="common", 4, IF(B96="uncommon", 3, IF(B96="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -2954,10 +2973,10 @@
         <v>0.13</v>
       </c>
       <c r="E97" s="3" t="n">
-        <v>0.87</v>
+        <v>0.89</v>
       </c>
       <c r="F97" s="3">
-        <f>IF(B97="common", 4, IF(B97="uncommon", 3, IF(B97="rare", 1.22, 1)))</f>
+        <f>IF(B97="common", 4, IF(B97="uncommon", 3, IF(B97="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -2976,13 +2995,13 @@
         <v>33</v>
       </c>
       <c r="D98" s="3" t="n">
-        <v>0.09</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="E98" s="3" t="n">
-        <v>0.23</v>
+        <v>0.2</v>
       </c>
       <c r="F98" s="3">
-        <f>IF(B98="common", 4, IF(B98="uncommon", 3, IF(B98="rare", 1.22, 1)))</f>
+        <f>IF(B98="common", 4, IF(B98="uncommon", 3, IF(B98="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -3001,13 +3020,13 @@
         <v>46</v>
       </c>
       <c r="D99" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.1</v>
       </c>
       <c r="E99" s="3" t="n">
-        <v>2.13</v>
+        <v>2.01</v>
       </c>
       <c r="F99" s="3">
-        <f>IF(B99="common", 4, IF(B99="uncommon", 3, IF(B99="rare", 1.22, 1)))</f>
+        <f>IF(B99="common", 4, IF(B99="uncommon", 3, IF(B99="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -3026,11 +3045,11 @@
         <v>90</v>
       </c>
       <c r="D100" s="3" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.59</v>
       </c>
       <c r="E100" s="3" t="inlineStr"/>
       <c r="F100" s="3">
-        <f>IF(B100="common", 4, IF(B100="uncommon", 3, IF(B100="rare", 1.22, 1)))</f>
+        <f>IF(B100="common", 4, IF(B100="uncommon", 3, IF(B100="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -3049,11 +3068,11 @@
         <v>248</v>
       </c>
       <c r="D101" s="3" t="n">
-        <v>5.53</v>
+        <v>5.8</v>
       </c>
       <c r="E101" s="3" t="inlineStr"/>
       <c r="F101" s="3">
-        <f>IF(B101="common", 4, IF(B101="uncommon", 3, IF(B101="rare", 1.22, 1)))</f>
+        <f>IF(B101="common", 4, IF(B101="uncommon", 3, IF(B101="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -3072,13 +3091,13 @@
         <v>33</v>
       </c>
       <c r="D102" s="3" t="n">
-        <v>0.12</v>
+        <v>0.11</v>
       </c>
       <c r="E102" s="3" t="n">
-        <v>1.47</v>
+        <v>1.26</v>
       </c>
       <c r="F102" s="3">
-        <f>IF(B102="common", 4, IF(B102="uncommon", 3, IF(B102="rare", 1.22, 1)))</f>
+        <f>IF(B102="common", 4, IF(B102="uncommon", 3, IF(B102="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -3100,10 +3119,10 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="E103" s="3" t="n">
-        <v>0.18</v>
+        <v>0.14</v>
       </c>
       <c r="F103" s="3">
-        <f>IF(B103="common", 4, IF(B103="uncommon", 3, IF(B103="rare", 1.22, 1)))</f>
+        <f>IF(B103="common", 4, IF(B103="uncommon", 3, IF(B103="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -3122,13 +3141,13 @@
         <v>46</v>
       </c>
       <c r="D104" s="3" t="n">
-        <v>0.04</v>
+        <v>0.06</v>
       </c>
       <c r="E104" s="3" t="n">
-        <v>0.13</v>
+        <v>0.17</v>
       </c>
       <c r="F104" s="3">
-        <f>IF(B104="common", 4, IF(B104="uncommon", 3, IF(B104="rare", 1.22, 1)))</f>
+        <f>IF(B104="common", 4, IF(B104="uncommon", 3, IF(B104="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -3150,10 +3169,10 @@
         <v>0.08</v>
       </c>
       <c r="E105" s="3" t="n">
-        <v>1.51</v>
+        <v>1.65</v>
       </c>
       <c r="F105" s="3">
-        <f>IF(B105="common", 4, IF(B105="uncommon", 3, IF(B105="rare", 1.22, 1)))</f>
+        <f>IF(B105="common", 4, IF(B105="uncommon", 3, IF(B105="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -3172,13 +3191,13 @@
         <v>33</v>
       </c>
       <c r="D106" s="3" t="n">
-        <v>0.09</v>
+        <v>0.11</v>
       </c>
       <c r="E106" s="3" t="n">
-        <v>0.57</v>
+        <v>0.52</v>
       </c>
       <c r="F106" s="3">
-        <f>IF(B106="common", 4, IF(B106="uncommon", 3, IF(B106="rare", 1.22, 1)))</f>
+        <f>IF(B106="common", 4, IF(B106="uncommon", 3, IF(B106="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -3197,13 +3216,13 @@
         <v>46</v>
       </c>
       <c r="D107" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.09</v>
       </c>
       <c r="E107" s="3" t="n">
-        <v>0.14</v>
+        <v>0.15</v>
       </c>
       <c r="F107" s="3">
-        <f>IF(B107="common", 4, IF(B107="uncommon", 3, IF(B107="rare", 1.22, 1)))</f>
+        <f>IF(B107="common", 4, IF(B107="uncommon", 3, IF(B107="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -3222,13 +3241,13 @@
         <v>21</v>
       </c>
       <c r="D108" s="3" t="n">
-        <v>0.14</v>
+        <v>0.17</v>
       </c>
       <c r="E108" s="3" t="n">
-        <v>0.58</v>
+        <v>0.66</v>
       </c>
       <c r="F108" s="3">
-        <f>IF(B108="common", 4, IF(B108="uncommon", 3, IF(B108="rare", 1.22, 1)))</f>
+        <f>IF(B108="common", 4, IF(B108="uncommon", 3, IF(B108="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -3247,13 +3266,13 @@
         <v>33</v>
       </c>
       <c r="D109" s="3" t="n">
-        <v>0.09</v>
+        <v>0.1</v>
       </c>
       <c r="E109" s="3" t="n">
-        <v>0.13</v>
+        <v>0.15</v>
       </c>
       <c r="F109" s="3">
-        <f>IF(B109="common", 4, IF(B109="uncommon", 3, IF(B109="rare", 1.22, 1)))</f>
+        <f>IF(B109="common", 4, IF(B109="uncommon", 3, IF(B109="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -3272,11 +3291,11 @@
         <v>188</v>
       </c>
       <c r="D110" s="3" t="n">
-        <v>10.04</v>
+        <v>11.24</v>
       </c>
       <c r="E110" s="3" t="inlineStr"/>
       <c r="F110" s="3">
-        <f>IF(B110="common", 4, IF(B110="uncommon", 3, IF(B110="rare", 1.22, 1)))</f>
+        <f>IF(B110="common", 4, IF(B110="uncommon", 3, IF(B110="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -3298,10 +3317,10 @@
         <v>0.06</v>
       </c>
       <c r="E111" s="3" t="n">
-        <v>0.18</v>
+        <v>0.15</v>
       </c>
       <c r="F111" s="3">
-        <f>IF(B111="common", 4, IF(B111="uncommon", 3, IF(B111="rare", 1.22, 1)))</f>
+        <f>IF(B111="common", 4, IF(B111="uncommon", 3, IF(B111="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -3320,13 +3339,13 @@
         <v>46</v>
       </c>
       <c r="D112" s="3" t="n">
-        <v>0.06</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="E112" s="3" t="n">
-        <v>0.19</v>
+        <v>0.22</v>
       </c>
       <c r="F112" s="3">
-        <f>IF(B112="common", 4, IF(B112="uncommon", 3, IF(B112="rare", 1.22, 1)))</f>
+        <f>IF(B112="common", 4, IF(B112="uncommon", 3, IF(B112="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -3345,13 +3364,13 @@
         <v>46</v>
       </c>
       <c r="D113" s="3" t="n">
-        <v>0.06</v>
+        <v>0.08</v>
       </c>
       <c r="E113" s="3" t="n">
-        <v>1.26</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="F113" s="3">
-        <f>IF(B113="common", 4, IF(B113="uncommon", 3, IF(B113="rare", 1.22, 1)))</f>
+        <f>IF(B113="common", 4, IF(B113="uncommon", 3, IF(B113="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -3370,13 +3389,13 @@
         <v>46</v>
       </c>
       <c r="D114" s="3" t="n">
-        <v>0.06</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="E114" s="3" t="n">
         <v>0.15</v>
       </c>
       <c r="F114" s="3">
-        <f>IF(B114="common", 4, IF(B114="uncommon", 3, IF(B114="rare", 1.22, 1)))</f>
+        <f>IF(B114="common", 4, IF(B114="uncommon", 3, IF(B114="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -3395,13 +3414,13 @@
         <v>33</v>
       </c>
       <c r="D115" s="3" t="n">
-        <v>0.06</v>
+        <v>0.11</v>
       </c>
       <c r="E115" s="3" t="n">
-        <v>0.17</v>
+        <v>0.13</v>
       </c>
       <c r="F115" s="3">
-        <f>IF(B115="common", 4, IF(B115="uncommon", 3, IF(B115="rare", 1.22, 1)))</f>
+        <f>IF(B115="common", 4, IF(B115="uncommon", 3, IF(B115="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -3420,13 +3439,13 @@
         <v>46</v>
       </c>
       <c r="D116" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.08</v>
       </c>
       <c r="E116" s="3" t="n">
-        <v>0.14</v>
+        <v>0.13</v>
       </c>
       <c r="F116" s="3">
-        <f>IF(B116="common", 4, IF(B116="uncommon", 3, IF(B116="rare", 1.22, 1)))</f>
+        <f>IF(B116="common", 4, IF(B116="uncommon", 3, IF(B116="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -3445,13 +3464,13 @@
         <v>21</v>
       </c>
       <c r="D117" s="3" t="n">
-        <v>0.14</v>
+        <v>0.16</v>
       </c>
       <c r="E117" s="3" t="n">
-        <v>0.71</v>
+        <v>0.54</v>
       </c>
       <c r="F117" s="3">
-        <f>IF(B117="common", 4, IF(B117="uncommon", 3, IF(B117="rare", 1.22, 1)))</f>
+        <f>IF(B117="common", 4, IF(B117="uncommon", 3, IF(B117="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -3470,13 +3489,13 @@
         <v>46</v>
       </c>
       <c r="D118" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06</v>
       </c>
       <c r="E118" s="3" t="n">
-        <v>0.2</v>
+        <v>0.17</v>
       </c>
       <c r="F118" s="3">
-        <f>IF(B118="common", 4, IF(B118="uncommon", 3, IF(B118="rare", 1.22, 1)))</f>
+        <f>IF(B118="common", 4, IF(B118="uncommon", 3, IF(B118="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -3495,13 +3514,13 @@
         <v>46</v>
       </c>
       <c r="D119" s="3" t="n">
-        <v>0.09</v>
+        <v>0.1</v>
       </c>
       <c r="E119" s="3" t="n">
-        <v>2.15</v>
+        <v>2.22</v>
       </c>
       <c r="F119" s="3">
-        <f>IF(B119="common", 4, IF(B119="uncommon", 3, IF(B119="rare", 1.22, 1)))</f>
+        <f>IF(B119="common", 4, IF(B119="uncommon", 3, IF(B119="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -3520,11 +3539,11 @@
         <v>90</v>
       </c>
       <c r="D120" s="3" t="n">
-        <v>6.89</v>
+        <v>7.21</v>
       </c>
       <c r="E120" s="3" t="inlineStr"/>
       <c r="F120" s="3">
-        <f>IF(B120="common", 4, IF(B120="uncommon", 3, IF(B120="rare", 1.22, 1)))</f>
+        <f>IF(B120="common", 4, IF(B120="uncommon", 3, IF(B120="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -3543,11 +3562,11 @@
         <v>248</v>
       </c>
       <c r="D121" s="3" t="n">
-        <v>18.01</v>
+        <v>19.11</v>
       </c>
       <c r="E121" s="3" t="inlineStr"/>
       <c r="F121" s="3">
-        <f>IF(B121="common", 4, IF(B121="uncommon", 3, IF(B121="rare", 1.22, 1)))</f>
+        <f>IF(B121="common", 4, IF(B121="uncommon", 3, IF(B121="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -3566,11 +3585,11 @@
         <v>154</v>
       </c>
       <c r="D122" s="3" t="n">
-        <v>13.15</v>
+        <v>13.27</v>
       </c>
       <c r="E122" s="3" t="inlineStr"/>
       <c r="F122" s="3">
-        <f>IF(B122="common", 4, IF(B122="uncommon", 3, IF(B122="rare", 1.22, 1)))</f>
+        <f>IF(B122="common", 4, IF(B122="uncommon", 3, IF(B122="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -3589,11 +3608,11 @@
         <v>90</v>
       </c>
       <c r="D123" s="3" t="n">
-        <v>9.84</v>
+        <v>9.75</v>
       </c>
       <c r="E123" s="3" t="inlineStr"/>
       <c r="F123" s="3">
-        <f>IF(B123="common", 4, IF(B123="uncommon", 3, IF(B123="rare", 1.22, 1)))</f>
+        <f>IF(B123="common", 4, IF(B123="uncommon", 3, IF(B123="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -3612,13 +3631,13 @@
         <v>21</v>
       </c>
       <c r="D124" s="3" t="n">
-        <v>0.54</v>
+        <v>0.51</v>
       </c>
       <c r="E124" s="3" t="n">
-        <v>1.62</v>
+        <v>1.58</v>
       </c>
       <c r="F124" s="3">
-        <f>IF(B124="common", 4, IF(B124="uncommon", 3, IF(B124="rare", 1.22, 1)))</f>
+        <f>IF(B124="common", 4, IF(B124="uncommon", 3, IF(B124="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -3637,13 +3656,13 @@
         <v>21</v>
       </c>
       <c r="D125" s="3" t="n">
-        <v>0.17</v>
+        <v>0.21</v>
       </c>
       <c r="E125" s="3" t="n">
-        <v>1.01</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="F125" s="3">
-        <f>IF(B125="common", 4, IF(B125="uncommon", 3, IF(B125="rare", 1.22, 1)))</f>
+        <f>IF(B125="common", 4, IF(B125="uncommon", 3, IF(B125="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -3662,13 +3681,13 @@
         <v>21</v>
       </c>
       <c r="D126" s="3" t="n">
-        <v>0.14</v>
+        <v>0.15</v>
       </c>
       <c r="E126" s="3" t="n">
-        <v>0.54</v>
+        <v>0.51</v>
       </c>
       <c r="F126" s="3">
-        <f>IF(B126="common", 4, IF(B126="uncommon", 3, IF(B126="rare", 1.22, 1)))</f>
+        <f>IF(B126="common", 4, IF(B126="uncommon", 3, IF(B126="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -3687,11 +3706,11 @@
         <v>188</v>
       </c>
       <c r="D127" s="3" t="n">
-        <v>6.68</v>
+        <v>5.79</v>
       </c>
       <c r="E127" s="3" t="inlineStr"/>
       <c r="F127" s="3">
-        <f>IF(B127="common", 4, IF(B127="uncommon", 3, IF(B127="rare", 1.22, 1)))</f>
+        <f>IF(B127="common", 4, IF(B127="uncommon", 3, IF(B127="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -3710,13 +3729,13 @@
         <v>33</v>
       </c>
       <c r="D128" s="3" t="n">
-        <v>0.06</v>
+        <v>0.09</v>
       </c>
       <c r="E128" s="3" t="n">
-        <v>0.17</v>
+        <v>0.22</v>
       </c>
       <c r="F128" s="3">
-        <f>IF(B128="common", 4, IF(B128="uncommon", 3, IF(B128="rare", 1.22, 1)))</f>
+        <f>IF(B128="common", 4, IF(B128="uncommon", 3, IF(B128="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -3735,13 +3754,13 @@
         <v>21</v>
       </c>
       <c r="D129" s="3" t="n">
-        <v>0.2</v>
+        <v>0.19</v>
       </c>
       <c r="E129" s="3" t="n">
-        <v>0.92</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="F129" s="3">
-        <f>IF(B129="common", 4, IF(B129="uncommon", 3, IF(B129="rare", 1.22, 1)))</f>
+        <f>IF(B129="common", 4, IF(B129="uncommon", 3, IF(B129="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -3760,11 +3779,11 @@
         <v>188</v>
       </c>
       <c r="D130" s="3" t="n">
-        <v>10.45</v>
+        <v>9.58</v>
       </c>
       <c r="E130" s="3" t="inlineStr"/>
       <c r="F130" s="3">
-        <f>IF(B130="common", 4, IF(B130="uncommon", 3, IF(B130="rare", 1.22, 1)))</f>
+        <f>IF(B130="common", 4, IF(B130="uncommon", 3, IF(B130="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -3783,13 +3802,13 @@
         <v>33</v>
       </c>
       <c r="D131" s="3" t="n">
-        <v>0.08</v>
+        <v>0.06</v>
       </c>
       <c r="E131" s="3" t="n">
-        <v>0.19</v>
+        <v>0.21</v>
       </c>
       <c r="F131" s="3">
-        <f>IF(B131="common", 4, IF(B131="uncommon", 3, IF(B131="rare", 1.22, 1)))</f>
+        <f>IF(B131="common", 4, IF(B131="uncommon", 3, IF(B131="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -3808,13 +3827,13 @@
         <v>46</v>
       </c>
       <c r="D132" s="3" t="n">
-        <v>0.13</v>
+        <v>0.15</v>
       </c>
       <c r="E132" s="3" t="n">
-        <v>1.95</v>
+        <v>1.98</v>
       </c>
       <c r="F132" s="3">
-        <f>IF(B132="common", 4, IF(B132="uncommon", 3, IF(B132="rare", 1.22, 1)))</f>
+        <f>IF(B132="common", 4, IF(B132="uncommon", 3, IF(B132="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -3833,13 +3852,13 @@
         <v>46</v>
       </c>
       <c r="D133" s="3" t="n">
-        <v>0.14</v>
+        <v>0.13</v>
       </c>
       <c r="E133" s="3" t="n">
-        <v>2.12</v>
+        <v>1.56</v>
       </c>
       <c r="F133" s="3">
-        <f>IF(B133="common", 4, IF(B133="uncommon", 3, IF(B133="rare", 1.22, 1)))</f>
+        <f>IF(B133="common", 4, IF(B133="uncommon", 3, IF(B133="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -3861,10 +3880,10 @@
         <v>0.08</v>
       </c>
       <c r="E134" s="3" t="n">
-        <v>0.16</v>
+        <v>0.19</v>
       </c>
       <c r="F134" s="3">
-        <f>IF(B134="common", 4, IF(B134="uncommon", 3, IF(B134="rare", 1.22, 1)))</f>
+        <f>IF(B134="common", 4, IF(B134="uncommon", 3, IF(B134="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -3883,13 +3902,13 @@
         <v>33</v>
       </c>
       <c r="D135" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06</v>
       </c>
       <c r="E135" s="3" t="n">
-        <v>0.16</v>
+        <v>0.21</v>
       </c>
       <c r="F135" s="3">
-        <f>IF(B135="common", 4, IF(B135="uncommon", 3, IF(B135="rare", 1.22, 1)))</f>
+        <f>IF(B135="common", 4, IF(B135="uncommon", 3, IF(B135="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -3908,11 +3927,11 @@
         <v>90</v>
       </c>
       <c r="D136" s="3" t="n">
-        <v>0.59</v>
+        <v>0.83</v>
       </c>
       <c r="E136" s="3" t="inlineStr"/>
       <c r="F136" s="3">
-        <f>IF(B136="common", 4, IF(B136="uncommon", 3, IF(B136="rare", 1.22, 1)))</f>
+        <f>IF(B136="common", 4, IF(B136="uncommon", 3, IF(B136="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -3931,11 +3950,11 @@
         <v>248</v>
       </c>
       <c r="D137" s="3" t="n">
-        <v>9.24</v>
+        <v>7.87</v>
       </c>
       <c r="E137" s="3" t="inlineStr"/>
       <c r="F137" s="3">
-        <f>IF(B137="common", 4, IF(B137="uncommon", 3, IF(B137="rare", 1.22, 1)))</f>
+        <f>IF(B137="common", 4, IF(B137="uncommon", 3, IF(B137="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -3954,13 +3973,13 @@
         <v>46</v>
       </c>
       <c r="D138" s="3" t="n">
-        <v>0.06</v>
+        <v>0.08</v>
       </c>
       <c r="E138" s="3" t="n">
-        <v>0.16</v>
+        <v>0.19</v>
       </c>
       <c r="F138" s="3">
-        <f>IF(B138="common", 4, IF(B138="uncommon", 3, IF(B138="rare", 1.22, 1)))</f>
+        <f>IF(B138="common", 4, IF(B138="uncommon", 3, IF(B138="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -3979,13 +3998,13 @@
         <v>33</v>
       </c>
       <c r="D139" s="3" t="n">
-        <v>0.1</v>
+        <v>0.06</v>
       </c>
       <c r="E139" s="3" t="n">
-        <v>2.34</v>
+        <v>2.36</v>
       </c>
       <c r="F139" s="3">
-        <f>IF(B139="common", 4, IF(B139="uncommon", 3, IF(B139="rare", 1.22, 1)))</f>
+        <f>IF(B139="common", 4, IF(B139="uncommon", 3, IF(B139="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -4004,11 +4023,11 @@
         <v>188</v>
       </c>
       <c r="D140" s="3" t="n">
-        <v>7.26</v>
+        <v>8</v>
       </c>
       <c r="E140" s="3" t="inlineStr"/>
       <c r="F140" s="3">
-        <f>IF(B140="common", 4, IF(B140="uncommon", 3, IF(B140="rare", 1.22, 1)))</f>
+        <f>IF(B140="common", 4, IF(B140="uncommon", 3, IF(B140="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -4027,13 +4046,13 @@
         <v>21</v>
       </c>
       <c r="D141" s="3" t="n">
-        <v>0.13</v>
+        <v>0.14</v>
       </c>
       <c r="E141" s="3" t="n">
-        <v>0.62</v>
+        <v>0.59</v>
       </c>
       <c r="F141" s="3">
-        <f>IF(B141="common", 4, IF(B141="uncommon", 3, IF(B141="rare", 1.22, 1)))</f>
+        <f>IF(B141="common", 4, IF(B141="uncommon", 3, IF(B141="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -4052,13 +4071,13 @@
         <v>33</v>
       </c>
       <c r="D142" s="3" t="n">
-        <v>0.05</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="E142" s="3" t="n">
-        <v>1.28</v>
+        <v>1.36</v>
       </c>
       <c r="F142" s="3">
-        <f>IF(B142="common", 4, IF(B142="uncommon", 3, IF(B142="rare", 1.22, 1)))</f>
+        <f>IF(B142="common", 4, IF(B142="uncommon", 3, IF(B142="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -4077,13 +4096,13 @@
         <v>46</v>
       </c>
       <c r="D143" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.08</v>
       </c>
       <c r="E143" s="3" t="n">
         <v>0.16</v>
       </c>
       <c r="F143" s="3">
-        <f>IF(B143="common", 4, IF(B143="uncommon", 3, IF(B143="rare", 1.22, 1)))</f>
+        <f>IF(B143="common", 4, IF(B143="uncommon", 3, IF(B143="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -4102,13 +4121,13 @@
         <v>33</v>
       </c>
       <c r="D144" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.1</v>
       </c>
       <c r="E144" s="3" t="n">
-        <v>0.13</v>
+        <v>0.19</v>
       </c>
       <c r="F144" s="3">
-        <f>IF(B144="common", 4, IF(B144="uncommon", 3, IF(B144="rare", 1.22, 1)))</f>
+        <f>IF(B144="common", 4, IF(B144="uncommon", 3, IF(B144="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -4127,13 +4146,13 @@
         <v>33</v>
       </c>
       <c r="D145" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06</v>
       </c>
       <c r="E145" s="3" t="n">
-        <v>0.13</v>
+        <v>0.21</v>
       </c>
       <c r="F145" s="3">
-        <f>IF(B145="common", 4, IF(B145="uncommon", 3, IF(B145="rare", 1.22, 1)))</f>
+        <f>IF(B145="common", 4, IF(B145="uncommon", 3, IF(B145="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -4152,13 +4171,13 @@
         <v>33</v>
       </c>
       <c r="D146" s="3" t="n">
-        <v>0.1</v>
+        <v>0.06</v>
       </c>
       <c r="E146" s="3" t="n">
-        <v>0.18</v>
+        <v>0.2</v>
       </c>
       <c r="F146" s="3">
-        <f>IF(B146="common", 4, IF(B146="uncommon", 3, IF(B146="rare", 1.22, 1)))</f>
+        <f>IF(B146="common", 4, IF(B146="uncommon", 3, IF(B146="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -4177,13 +4196,13 @@
         <v>46</v>
       </c>
       <c r="D147" s="3" t="n">
-        <v>0.16</v>
+        <v>0.17</v>
       </c>
       <c r="E147" s="3" t="n">
-        <v>3.16</v>
+        <v>2.19</v>
       </c>
       <c r="F147" s="3">
-        <f>IF(B147="common", 4, IF(B147="uncommon", 3, IF(B147="rare", 1.22, 1)))</f>
+        <f>IF(B147="common", 4, IF(B147="uncommon", 3, IF(B147="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -4202,13 +4221,13 @@
         <v>46</v>
       </c>
       <c r="D148" s="3" t="n">
-        <v>0.12</v>
+        <v>0.09</v>
       </c>
       <c r="E148" s="3" t="n">
-        <v>0.2</v>
+        <v>0.24</v>
       </c>
       <c r="F148" s="3">
-        <f>IF(B148="common", 4, IF(B148="uncommon", 3, IF(B148="rare", 1.22, 1)))</f>
+        <f>IF(B148="common", 4, IF(B148="uncommon", 3, IF(B148="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -4230,10 +4249,10 @@
         <v>0.1</v>
       </c>
       <c r="E149" s="3" t="n">
-        <v>0.24</v>
+        <v>0.25</v>
       </c>
       <c r="F149" s="3">
-        <f>IF(B149="common", 4, IF(B149="uncommon", 3, IF(B149="rare", 1.22, 1)))</f>
+        <f>IF(B149="common", 4, IF(B149="uncommon", 3, IF(B149="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -4252,11 +4271,11 @@
         <v>188</v>
       </c>
       <c r="D150" s="3" t="n">
-        <v>28.19</v>
+        <v>28.89</v>
       </c>
       <c r="E150" s="3" t="inlineStr"/>
       <c r="F150" s="3">
-        <f>IF(B150="common", 4, IF(B150="uncommon", 3, IF(B150="rare", 1.22, 1)))</f>
+        <f>IF(B150="common", 4, IF(B150="uncommon", 3, IF(B150="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -4275,13 +4294,13 @@
         <v>33</v>
       </c>
       <c r="D151" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.08</v>
       </c>
       <c r="E151" s="3" t="n">
-        <v>1.36</v>
+        <v>1.65</v>
       </c>
       <c r="F151" s="3">
-        <f>IF(B151="common", 4, IF(B151="uncommon", 3, IF(B151="rare", 1.22, 1)))</f>
+        <f>IF(B151="common", 4, IF(B151="uncommon", 3, IF(B151="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -4303,10 +4322,10 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="E152" s="3" t="n">
-        <v>0.18</v>
+        <v>0.15</v>
       </c>
       <c r="F152" s="3">
-        <f>IF(B152="common", 4, IF(B152="uncommon", 3, IF(B152="rare", 1.22, 1)))</f>
+        <f>IF(B152="common", 4, IF(B152="uncommon", 3, IF(B152="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -4328,10 +4347,10 @@
         <v>0.1</v>
       </c>
       <c r="E153" s="3" t="n">
-        <v>1.44</v>
+        <v>1.14</v>
       </c>
       <c r="F153" s="3">
-        <f>IF(B153="common", 4, IF(B153="uncommon", 3, IF(B153="rare", 1.22, 1)))</f>
+        <f>IF(B153="common", 4, IF(B153="uncommon", 3, IF(B153="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -4350,11 +4369,11 @@
         <v>188</v>
       </c>
       <c r="D154" s="3" t="n">
-        <v>15.76</v>
+        <v>18.96</v>
       </c>
       <c r="E154" s="3" t="inlineStr"/>
       <c r="F154" s="3">
-        <f>IF(B154="common", 4, IF(B154="uncommon", 3, IF(B154="rare", 1.22, 1)))</f>
+        <f>IF(B154="common", 4, IF(B154="uncommon", 3, IF(B154="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -4373,13 +4392,13 @@
         <v>33</v>
       </c>
       <c r="D155" s="3" t="n">
-        <v>0.08</v>
+        <v>0.06</v>
       </c>
       <c r="E155" s="3" t="n">
-        <v>0.17</v>
+        <v>0.16</v>
       </c>
       <c r="F155" s="3">
-        <f>IF(B155="common", 4, IF(B155="uncommon", 3, IF(B155="rare", 1.22, 1)))</f>
+        <f>IF(B155="common", 4, IF(B155="uncommon", 3, IF(B155="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -4398,13 +4417,13 @@
         <v>46</v>
       </c>
       <c r="D156" s="3" t="n">
-        <v>0.06</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="E156" s="3" t="n">
-        <v>0.13</v>
+        <v>0.16</v>
       </c>
       <c r="F156" s="3">
-        <f>IF(B156="common", 4, IF(B156="uncommon", 3, IF(B156="rare", 1.22, 1)))</f>
+        <f>IF(B156="common", 4, IF(B156="uncommon", 3, IF(B156="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -4423,13 +4442,13 @@
         <v>46</v>
       </c>
       <c r="D157" s="3" t="n">
-        <v>0.08</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="E157" s="3" t="n">
-        <v>0.14</v>
+        <v>0.17</v>
       </c>
       <c r="F157" s="3">
-        <f>IF(B157="common", 4, IF(B157="uncommon", 3, IF(B157="rare", 1.22, 1)))</f>
+        <f>IF(B157="common", 4, IF(B157="uncommon", 3, IF(B157="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -4448,13 +4467,13 @@
         <v>33</v>
       </c>
       <c r="D158" s="3" t="n">
-        <v>0.05</v>
+        <v>0.09</v>
       </c>
       <c r="E158" s="3" t="n">
-        <v>0.19</v>
+        <v>0.16</v>
       </c>
       <c r="F158" s="3">
-        <f>IF(B158="common", 4, IF(B158="uncommon", 3, IF(B158="rare", 1.22, 1)))</f>
+        <f>IF(B158="common", 4, IF(B158="uncommon", 3, IF(B158="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -4473,13 +4492,13 @@
         <v>33</v>
       </c>
       <c r="D159" s="3" t="n">
-        <v>0.11</v>
+        <v>0.13</v>
       </c>
       <c r="E159" s="3" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.61</v>
       </c>
       <c r="F159" s="3">
-        <f>IF(B159="common", 4, IF(B159="uncommon", 3, IF(B159="rare", 1.22, 1)))</f>
+        <f>IF(B159="common", 4, IF(B159="uncommon", 3, IF(B159="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -4498,13 +4517,13 @@
         <v>46</v>
       </c>
       <c r="D160" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.09</v>
       </c>
       <c r="E160" s="3" t="n">
-        <v>0.34</v>
+        <v>0.22</v>
       </c>
       <c r="F160" s="3">
-        <f>IF(B160="common", 4, IF(B160="uncommon", 3, IF(B160="rare", 1.22, 1)))</f>
+        <f>IF(B160="common", 4, IF(B160="uncommon", 3, IF(B160="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -4523,11 +4542,11 @@
         <v>188</v>
       </c>
       <c r="D161" s="3" t="n">
-        <v>20.61</v>
+        <v>21.1</v>
       </c>
       <c r="E161" s="3" t="inlineStr"/>
       <c r="F161" s="3">
-        <f>IF(B161="common", 4, IF(B161="uncommon", 3, IF(B161="rare", 1.22, 1)))</f>
+        <f>IF(B161="common", 4, IF(B161="uncommon", 3, IF(B161="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -4549,10 +4568,10 @@
         <v>0.14</v>
       </c>
       <c r="E162" s="3" t="n">
-        <v>0.95</v>
+        <v>0.86</v>
       </c>
       <c r="F162" s="3">
-        <f>IF(B162="common", 4, IF(B162="uncommon", 3, IF(B162="rare", 1.22, 1)))</f>
+        <f>IF(B162="common", 4, IF(B162="uncommon", 3, IF(B162="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -4574,10 +4593,10 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="E163" s="3" t="n">
-        <v>0.17</v>
+        <v>0.18</v>
       </c>
       <c r="F163" s="3">
-        <f>IF(B163="common", 4, IF(B163="uncommon", 3, IF(B163="rare", 1.22, 1)))</f>
+        <f>IF(B163="common", 4, IF(B163="uncommon", 3, IF(B163="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -4596,13 +4615,13 @@
         <v>33</v>
       </c>
       <c r="D164" s="3" t="n">
-        <v>0.06</v>
+        <v>0.08</v>
       </c>
       <c r="E164" s="3" t="n">
         <v>0.17</v>
       </c>
       <c r="F164" s="3">
-        <f>IF(B164="common", 4, IF(B164="uncommon", 3, IF(B164="rare", 1.22, 1)))</f>
+        <f>IF(B164="common", 4, IF(B164="uncommon", 3, IF(B164="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -4624,10 +4643,10 @@
         <v>0.06</v>
       </c>
       <c r="E165" s="3" t="n">
-        <v>0.12</v>
+        <v>0.19</v>
       </c>
       <c r="F165" s="3">
-        <f>IF(B165="common", 4, IF(B165="uncommon", 3, IF(B165="rare", 1.22, 1)))</f>
+        <f>IF(B165="common", 4, IF(B165="uncommon", 3, IF(B165="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -4646,13 +4665,13 @@
         <v>33</v>
       </c>
       <c r="D166" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.09</v>
       </c>
       <c r="E166" s="3" t="n">
-        <v>0.15</v>
+        <v>0.14</v>
       </c>
       <c r="F166" s="3">
-        <f>IF(B166="common", 4, IF(B166="uncommon", 3, IF(B166="rare", 1.22, 1)))</f>
+        <f>IF(B166="common", 4, IF(B166="uncommon", 3, IF(B166="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -4671,13 +4690,13 @@
         <v>46</v>
       </c>
       <c r="D167" s="3" t="n">
-        <v>0.05</v>
+        <v>0.06</v>
       </c>
       <c r="E167" s="3" t="n">
-        <v>0.14</v>
+        <v>0.15</v>
       </c>
       <c r="F167" s="3">
-        <f>IF(B167="common", 4, IF(B167="uncommon", 3, IF(B167="rare", 1.22, 1)))</f>
+        <f>IF(B167="common", 4, IF(B167="uncommon", 3, IF(B167="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -4696,13 +4715,13 @@
         <v>33</v>
       </c>
       <c r="D168" s="3" t="n">
-        <v>0.12</v>
+        <v>0.1</v>
       </c>
       <c r="E168" s="3" t="n">
-        <v>1.43</v>
+        <v>1.08</v>
       </c>
       <c r="F168" s="3">
-        <f>IF(B168="common", 4, IF(B168="uncommon", 3, IF(B168="rare", 1.22, 1)))</f>
+        <f>IF(B168="common", 4, IF(B168="uncommon", 3, IF(B168="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -4721,13 +4740,13 @@
         <v>46</v>
       </c>
       <c r="D169" s="3" t="n">
-        <v>0.05</v>
+        <v>0.08</v>
       </c>
       <c r="E169" s="3" t="n">
-        <v>0.16</v>
+        <v>0.17</v>
       </c>
       <c r="F169" s="3">
-        <f>IF(B169="common", 4, IF(B169="uncommon", 3, IF(B169="rare", 1.22, 1)))</f>
+        <f>IF(B169="common", 4, IF(B169="uncommon", 3, IF(B169="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -4746,13 +4765,13 @@
         <v>33</v>
       </c>
       <c r="D170" s="3" t="n">
-        <v>0.09</v>
+        <v>0.08</v>
       </c>
       <c r="E170" s="3" t="n">
-        <v>0.18</v>
+        <v>0.17</v>
       </c>
       <c r="F170" s="3">
-        <f>IF(B170="common", 4, IF(B170="uncommon", 3, IF(B170="rare", 1.22, 1)))</f>
+        <f>IF(B170="common", 4, IF(B170="uncommon", 3, IF(B170="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -4771,13 +4790,13 @@
         <v>33</v>
       </c>
       <c r="D171" s="3" t="n">
-        <v>0.12</v>
+        <v>0.11</v>
       </c>
       <c r="E171" s="3" t="n">
-        <v>2.57</v>
+        <v>2.4</v>
       </c>
       <c r="F171" s="3">
-        <f>IF(B171="common", 4, IF(B171="uncommon", 3, IF(B171="rare", 1.22, 1)))</f>
+        <f>IF(B171="common", 4, IF(B171="uncommon", 3, IF(B171="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -4796,13 +4815,13 @@
         <v>33</v>
       </c>
       <c r="D172" s="3" t="n">
-        <v>0.05</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="E172" s="3" t="n">
         <v>0.14</v>
       </c>
       <c r="F172" s="3">
-        <f>IF(B172="common", 4, IF(B172="uncommon", 3, IF(B172="rare", 1.22, 1)))</f>
+        <f>IF(B172="common", 4, IF(B172="uncommon", 3, IF(B172="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -4821,13 +4840,13 @@
         <v>33</v>
       </c>
       <c r="D173" s="3" t="n">
-        <v>0.06</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="E173" s="3" t="n">
-        <v>1.02</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="F173" s="3">
-        <f>IF(B173="common", 4, IF(B173="uncommon", 3, IF(B173="rare", 1.22, 1)))</f>
+        <f>IF(B173="common", 4, IF(B173="uncommon", 3, IF(B173="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -4849,10 +4868,10 @@
         <v>0.08</v>
       </c>
       <c r="E174" s="3" t="n">
-        <v>0.15</v>
+        <v>0.11</v>
       </c>
       <c r="F174" s="3">
-        <f>IF(B174="common", 4, IF(B174="uncommon", 3, IF(B174="rare", 1.22, 1)))</f>
+        <f>IF(B174="common", 4, IF(B174="uncommon", 3, IF(B174="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -4874,10 +4893,10 @@
         <v>0.06</v>
       </c>
       <c r="E175" s="3" t="n">
-        <v>0.16</v>
+        <v>0.15</v>
       </c>
       <c r="F175" s="3">
-        <f>IF(B175="common", 4, IF(B175="uncommon", 3, IF(B175="rare", 1.22, 1)))</f>
+        <f>IF(B175="common", 4, IF(B175="uncommon", 3, IF(B175="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -4896,13 +4915,13 @@
         <v>33</v>
       </c>
       <c r="D176" s="3" t="n">
-        <v>0.06</v>
+        <v>0.08</v>
       </c>
       <c r="E176" s="3" t="n">
-        <v>0.19</v>
+        <v>0.17</v>
       </c>
       <c r="F176" s="3">
-        <f>IF(B176="common", 4, IF(B176="uncommon", 3, IF(B176="rare", 1.22, 1)))</f>
+        <f>IF(B176="common", 4, IF(B176="uncommon", 3, IF(B176="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -4921,13 +4940,13 @@
         <v>46</v>
       </c>
       <c r="D177" s="3" t="n">
-        <v>0.08</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="E177" s="3" t="n">
-        <v>0.2</v>
+        <v>0.22</v>
       </c>
       <c r="F177" s="3">
-        <f>IF(B177="common", 4, IF(B177="uncommon", 3, IF(B177="rare", 1.22, 1)))</f>
+        <f>IF(B177="common", 4, IF(B177="uncommon", 3, IF(B177="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -4946,13 +4965,13 @@
         <v>33</v>
       </c>
       <c r="D178" s="3" t="n">
-        <v>0.12</v>
+        <v>0.16</v>
       </c>
       <c r="E178" s="3" t="n">
-        <v>1.96</v>
+        <v>1.27</v>
       </c>
       <c r="F178" s="3">
-        <f>IF(B178="common", 4, IF(B178="uncommon", 3, IF(B178="rare", 1.22, 1)))</f>
+        <f>IF(B178="common", 4, IF(B178="uncommon", 3, IF(B178="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -4971,13 +4990,13 @@
         <v>46</v>
       </c>
       <c r="D179" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06</v>
       </c>
       <c r="E179" s="3" t="n">
-        <v>1.3</v>
+        <v>0.9</v>
       </c>
       <c r="F179" s="3">
-        <f>IF(B179="common", 4, IF(B179="uncommon", 3, IF(B179="rare", 1.22, 1)))</f>
+        <f>IF(B179="common", 4, IF(B179="uncommon", 3, IF(B179="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -4996,13 +5015,13 @@
         <v>46</v>
       </c>
       <c r="D180" s="3" t="n">
-        <v>0.12</v>
+        <v>0.11</v>
       </c>
       <c r="E180" s="3" t="n">
-        <v>0.16</v>
+        <v>0.23</v>
       </c>
       <c r="F180" s="3">
-        <f>IF(B180="common", 4, IF(B180="uncommon", 3, IF(B180="rare", 1.22, 1)))</f>
+        <f>IF(B180="common", 4, IF(B180="uncommon", 3, IF(B180="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -5021,11 +5040,11 @@
         <v>188</v>
       </c>
       <c r="D181" s="3" t="n">
-        <v>45.51</v>
+        <v>46.05</v>
       </c>
       <c r="E181" s="3" t="inlineStr"/>
       <c r="F181" s="3">
-        <f>IF(B181="common", 4, IF(B181="uncommon", 3, IF(B181="rare", 1.22, 1)))</f>
+        <f>IF(B181="common", 4, IF(B181="uncommon", 3, IF(B181="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -5044,13 +5063,13 @@
         <v>21</v>
       </c>
       <c r="D182" s="3" t="n">
-        <v>0.13</v>
+        <v>0.16</v>
       </c>
       <c r="E182" s="3" t="n">
-        <v>0.75</v>
+        <v>0.64</v>
       </c>
       <c r="F182" s="3">
-        <f>IF(B182="common", 4, IF(B182="uncommon", 3, IF(B182="rare", 1.22, 1)))</f>
+        <f>IF(B182="common", 4, IF(B182="uncommon", 3, IF(B182="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -5069,13 +5088,13 @@
         <v>46</v>
       </c>
       <c r="D183" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06</v>
       </c>
       <c r="E183" s="3" t="n">
-        <v>0.15</v>
+        <v>0.17</v>
       </c>
       <c r="F183" s="3">
-        <f>IF(B183="common", 4, IF(B183="uncommon", 3, IF(B183="rare", 1.22, 1)))</f>
+        <f>IF(B183="common", 4, IF(B183="uncommon", 3, IF(B183="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -5094,11 +5113,11 @@
         <v>154</v>
       </c>
       <c r="D184" s="3" t="n">
-        <v>2.38</v>
+        <v>2.56</v>
       </c>
       <c r="E184" s="3" t="inlineStr"/>
       <c r="F184" s="3">
-        <f>IF(B184="common", 4, IF(B184="uncommon", 3, IF(B184="rare", 1.22, 1)))</f>
+        <f>IF(B184="common", 4, IF(B184="uncommon", 3, IF(B184="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -5117,13 +5136,13 @@
         <v>46</v>
       </c>
       <c r="D185" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06</v>
       </c>
       <c r="E185" s="3" t="n">
-        <v>0.14</v>
+        <v>0.15</v>
       </c>
       <c r="F185" s="3">
-        <f>IF(B185="common", 4, IF(B185="uncommon", 3, IF(B185="rare", 1.22, 1)))</f>
+        <f>IF(B185="common", 4, IF(B185="uncommon", 3, IF(B185="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -5142,11 +5161,11 @@
         <v>188</v>
       </c>
       <c r="D186" s="3" t="n">
-        <v>7.57</v>
+        <v>7.68</v>
       </c>
       <c r="E186" s="3" t="inlineStr"/>
       <c r="F186" s="3">
-        <f>IF(B186="common", 4, IF(B186="uncommon", 3, IF(B186="rare", 1.22, 1)))</f>
+        <f>IF(B186="common", 4, IF(B186="uncommon", 3, IF(B186="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -5165,13 +5184,13 @@
         <v>33</v>
       </c>
       <c r="D187" s="3" t="n">
-        <v>0.06</v>
+        <v>0.08</v>
       </c>
       <c r="E187" s="3" t="n">
-        <v>0.7</v>
+        <v>0.77</v>
       </c>
       <c r="F187" s="3">
-        <f>IF(B187="common", 4, IF(B187="uncommon", 3, IF(B187="rare", 1.22, 1)))</f>
+        <f>IF(B187="common", 4, IF(B187="uncommon", 3, IF(B187="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -5190,13 +5209,13 @@
         <v>46</v>
       </c>
       <c r="D188" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06</v>
       </c>
       <c r="E188" s="3" t="n">
-        <v>0.13</v>
+        <v>0.16</v>
       </c>
       <c r="F188" s="3">
-        <f>IF(B188="common", 4, IF(B188="uncommon", 3, IF(B188="rare", 1.22, 1)))</f>
+        <f>IF(B188="common", 4, IF(B188="uncommon", 3, IF(B188="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -5215,13 +5234,13 @@
         <v>33</v>
       </c>
       <c r="D189" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06</v>
       </c>
       <c r="E189" s="3" t="n">
-        <v>0.14</v>
+        <v>0.15</v>
       </c>
       <c r="F189" s="3">
-        <f>IF(B189="common", 4, IF(B189="uncommon", 3, IF(B189="rare", 1.22, 1)))</f>
+        <f>IF(B189="common", 4, IF(B189="uncommon", 3, IF(B189="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -5243,10 +5262,10 @@
         <v>0.28</v>
       </c>
       <c r="E190" s="3" t="n">
-        <v>1.44</v>
+        <v>1.28</v>
       </c>
       <c r="F190" s="3">
-        <f>IF(B190="common", 4, IF(B190="uncommon", 3, IF(B190="rare", 1.22, 1)))</f>
+        <f>IF(B190="common", 4, IF(B190="uncommon", 3, IF(B190="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -5268,10 +5287,10 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="E191" s="3" t="n">
-        <v>0.17</v>
+        <v>0.18</v>
       </c>
       <c r="F191" s="3">
-        <f>IF(B191="common", 4, IF(B191="uncommon", 3, IF(B191="rare", 1.22, 1)))</f>
+        <f>IF(B191="common", 4, IF(B191="uncommon", 3, IF(B191="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -5290,13 +5309,13 @@
         <v>46</v>
       </c>
       <c r="D192" s="3" t="n">
-        <v>0.04</v>
+        <v>0.05</v>
       </c>
       <c r="E192" s="3" t="n">
         <v>0.14</v>
       </c>
       <c r="F192" s="3">
-        <f>IF(B192="common", 4, IF(B192="uncommon", 3, IF(B192="rare", 1.22, 1)))</f>
+        <f>IF(B192="common", 4, IF(B192="uncommon", 3, IF(B192="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -5315,11 +5334,11 @@
         <v>90</v>
       </c>
       <c r="D193" s="3" t="n">
-        <v>0.58</v>
+        <v>0.77</v>
       </c>
       <c r="E193" s="3" t="inlineStr"/>
       <c r="F193" s="3">
-        <f>IF(B193="common", 4, IF(B193="uncommon", 3, IF(B193="rare", 1.22, 1)))</f>
+        <f>IF(B193="common", 4, IF(B193="uncommon", 3, IF(B193="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -5338,11 +5357,11 @@
         <v>248</v>
       </c>
       <c r="D194" s="3" t="n">
-        <v>11.85</v>
+        <v>11.82</v>
       </c>
       <c r="E194" s="3" t="inlineStr"/>
       <c r="F194" s="3">
-        <f>IF(B194="common", 4, IF(B194="uncommon", 3, IF(B194="rare", 1.22, 1)))</f>
+        <f>IF(B194="common", 4, IF(B194="uncommon", 3, IF(B194="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -5361,11 +5380,11 @@
         <v>225</v>
       </c>
       <c r="D195" s="3" t="n">
-        <v>66.20999999999999</v>
+        <v>68.69</v>
       </c>
       <c r="E195" s="3" t="inlineStr"/>
       <c r="F195" s="3">
-        <f>IF(B195="common", 4, IF(B195="uncommon", 3, IF(B195="rare", 1.22, 1)))</f>
+        <f>IF(B195="common", 4, IF(B195="uncommon", 3, IF(B195="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -5387,10 +5406,10 @@
         <v>0.05</v>
       </c>
       <c r="E196" s="3" t="n">
-        <v>0.31</v>
+        <v>0.17</v>
       </c>
       <c r="F196" s="3">
-        <f>IF(B196="common", 4, IF(B196="uncommon", 3, IF(B196="rare", 1.22, 1)))</f>
+        <f>IF(B196="common", 4, IF(B196="uncommon", 3, IF(B196="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -5409,13 +5428,13 @@
         <v>21</v>
       </c>
       <c r="D197" s="3" t="n">
-        <v>0.15</v>
+        <v>0.2</v>
       </c>
       <c r="E197" s="3" t="n">
-        <v>0.88</v>
+        <v>0.93</v>
       </c>
       <c r="F197" s="3">
-        <f>IF(B197="common", 4, IF(B197="uncommon", 3, IF(B197="rare", 1.22, 1)))</f>
+        <f>IF(B197="common", 4, IF(B197="uncommon", 3, IF(B197="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -5434,13 +5453,13 @@
         <v>46</v>
       </c>
       <c r="D198" s="3" t="n">
-        <v>0.05</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="E198" s="3" t="n">
-        <v>0.16</v>
+        <v>0.17</v>
       </c>
       <c r="F198" s="3">
-        <f>IF(B198="common", 4, IF(B198="uncommon", 3, IF(B198="rare", 1.22, 1)))</f>
+        <f>IF(B198="common", 4, IF(B198="uncommon", 3, IF(B198="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -5459,13 +5478,13 @@
         <v>46</v>
       </c>
       <c r="D199" s="3" t="n">
-        <v>0.06</v>
+        <v>0.09</v>
       </c>
       <c r="E199" s="3" t="n">
-        <v>0.15</v>
+        <v>0.21</v>
       </c>
       <c r="F199" s="3">
-        <f>IF(B199="common", 4, IF(B199="uncommon", 3, IF(B199="rare", 1.22, 1)))</f>
+        <f>IF(B199="common", 4, IF(B199="uncommon", 3, IF(B199="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -5487,10 +5506,10 @@
         <v>0.12</v>
       </c>
       <c r="E200" s="3" t="n">
-        <v>0.25</v>
+        <v>0.22</v>
       </c>
       <c r="F200" s="3">
-        <f>IF(B200="common", 4, IF(B200="uncommon", 3, IF(B200="rare", 1.22, 1)))</f>
+        <f>IF(B200="common", 4, IF(B200="uncommon", 3, IF(B200="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -5509,11 +5528,11 @@
         <v>188</v>
       </c>
       <c r="D201" s="3" t="n">
-        <v>29.75</v>
+        <v>30.34</v>
       </c>
       <c r="E201" s="3" t="inlineStr"/>
       <c r="F201" s="3">
-        <f>IF(B201="common", 4, IF(B201="uncommon", 3, IF(B201="rare", 1.22, 1)))</f>
+        <f>IF(B201="common", 4, IF(B201="uncommon", 3, IF(B201="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -5532,13 +5551,13 @@
         <v>46</v>
       </c>
       <c r="D202" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06</v>
       </c>
       <c r="E202" s="3" t="n">
-        <v>0.16</v>
+        <v>0.11</v>
       </c>
       <c r="F202" s="3">
-        <f>IF(B202="common", 4, IF(B202="uncommon", 3, IF(B202="rare", 1.22, 1)))</f>
+        <f>IF(B202="common", 4, IF(B202="uncommon", 3, IF(B202="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -5557,13 +5576,13 @@
         <v>46</v>
       </c>
       <c r="D203" s="3" t="n">
-        <v>0.11</v>
+        <v>0.1</v>
       </c>
       <c r="E203" s="3" t="n">
-        <v>1.85</v>
+        <v>1.51</v>
       </c>
       <c r="F203" s="3">
-        <f>IF(B203="common", 4, IF(B203="uncommon", 3, IF(B203="rare", 1.22, 1)))</f>
+        <f>IF(B203="common", 4, IF(B203="uncommon", 3, IF(B203="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -5582,13 +5601,13 @@
         <v>21</v>
       </c>
       <c r="D204" s="3" t="n">
-        <v>0.12</v>
+        <v>0.15</v>
       </c>
       <c r="E204" s="3" t="n">
-        <v>0.55</v>
+        <v>0.58</v>
       </c>
       <c r="F204" s="3">
-        <f>IF(B204="common", 4, IF(B204="uncommon", 3, IF(B204="rare", 1.22, 1)))</f>
+        <f>IF(B204="common", 4, IF(B204="uncommon", 3, IF(B204="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -5607,11 +5626,11 @@
         <v>90</v>
       </c>
       <c r="D205" s="3" t="n">
-        <v>0.73</v>
+        <v>0.77</v>
       </c>
       <c r="E205" s="3" t="inlineStr"/>
       <c r="F205" s="3">
-        <f>IF(B205="common", 4, IF(B205="uncommon", 3, IF(B205="rare", 1.22, 1)))</f>
+        <f>IF(B205="common", 4, IF(B205="uncommon", 3, IF(B205="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -5630,11 +5649,11 @@
         <v>248</v>
       </c>
       <c r="D206" s="3" t="n">
-        <v>6.95</v>
+        <v>7.9</v>
       </c>
       <c r="E206" s="3" t="inlineStr"/>
       <c r="F206" s="3">
-        <f>IF(B206="common", 4, IF(B206="uncommon", 3, IF(B206="rare", 1.22, 1)))</f>
+        <f>IF(B206="common", 4, IF(B206="uncommon", 3, IF(B206="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -5653,11 +5672,11 @@
         <v>90</v>
       </c>
       <c r="D207" s="3" t="n">
-        <v>0.7</v>
+        <v>0.71</v>
       </c>
       <c r="E207" s="3" t="inlineStr"/>
       <c r="F207" s="3">
-        <f>IF(B207="common", 4, IF(B207="uncommon", 3, IF(B207="rare", 1.22, 1)))</f>
+        <f>IF(B207="common", 4, IF(B207="uncommon", 3, IF(B207="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -5676,11 +5695,11 @@
         <v>248</v>
       </c>
       <c r="D208" s="3" t="n">
-        <v>7.9</v>
+        <v>8.06</v>
       </c>
       <c r="E208" s="3" t="inlineStr"/>
       <c r="F208" s="3">
-        <f>IF(B208="common", 4, IF(B208="uncommon", 3, IF(B208="rare", 1.22, 1)))</f>
+        <f>IF(B208="common", 4, IF(B208="uncommon", 3, IF(B208="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -5699,11 +5718,11 @@
         <v>225</v>
       </c>
       <c r="D209" s="3" t="n">
-        <v>52.05</v>
+        <v>55.36</v>
       </c>
       <c r="E209" s="3" t="inlineStr"/>
       <c r="F209" s="3">
-        <f>IF(B209="common", 4, IF(B209="uncommon", 3, IF(B209="rare", 1.22, 1)))</f>
+        <f>IF(B209="common", 4, IF(B209="uncommon", 3, IF(B209="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -5725,10 +5744,10 @@
         <v>0.06</v>
       </c>
       <c r="E210" s="3" t="n">
-        <v>0.15</v>
+        <v>0.21</v>
       </c>
       <c r="F210" s="3">
-        <f>IF(B210="common", 4, IF(B210="uncommon", 3, IF(B210="rare", 1.22, 1)))</f>
+        <f>IF(B210="common", 4, IF(B210="uncommon", 3, IF(B210="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -5753,7 +5772,7 @@
         <v>0.59</v>
       </c>
       <c r="F211" s="3">
-        <f>IF(B211="common", 4, IF(B211="uncommon", 3, IF(B211="rare", 1.22, 1)))</f>
+        <f>IF(B211="common", 4, IF(B211="uncommon", 3, IF(B211="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -5776,7 +5795,7 @@
       </c>
       <c r="E212" s="3" t="n"/>
       <c r="F212" s="3">
-        <f>IF(B212="common", 4, IF(B212="uncommon", 3, IF(B212="rare", 1.22, 1)))</f>
+        <f>IF(B212="common", 4, IF(B212="uncommon", 3, IF(B212="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -5799,7 +5818,7 @@
       </c>
       <c r="E213" s="3" t="n"/>
       <c r="F213" s="3">
-        <f>IF(B213="common", 4, IF(B213="uncommon", 3, IF(B213="rare", 1.22, 1)))</f>
+        <f>IF(B213="common", 4, IF(B213="uncommon", 3, IF(B213="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -5822,7 +5841,7 @@
       </c>
       <c r="E214" s="3" t="n"/>
       <c r="F214" s="3">
-        <f>IF(B214="common", 4, IF(B214="uncommon", 3, IF(B214="rare", 1.22, 1)))</f>
+        <f>IF(B214="common", 4, IF(B214="uncommon", 3, IF(B214="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -5845,7 +5864,7 @@
       </c>
       <c r="E215" s="3" t="n"/>
       <c r="F215" s="3">
-        <f>IF(B215="common", 4, IF(B215="uncommon", 3, IF(B215="rare", 1.22, 1)))</f>
+        <f>IF(B215="common", 4, IF(B215="uncommon", 3, IF(B215="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -5868,7 +5887,7 @@
       </c>
       <c r="E216" s="3" t="n"/>
       <c r="F216" s="3">
-        <f>IF(B216="common", 4, IF(B216="uncommon", 3, IF(B216="rare", 1.22, 1)))</f>
+        <f>IF(B216="common", 4, IF(B216="uncommon", 3, IF(B216="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -5893,7 +5912,7 @@
         <v>0.14</v>
       </c>
       <c r="F217" s="3">
-        <f>IF(B217="common", 4, IF(B217="uncommon", 3, IF(B217="rare", 1.22, 1)))</f>
+        <f>IF(B217="common", 4, IF(B217="uncommon", 3, IF(B217="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
     </row>
@@ -12441,7 +12460,7 @@
       <c r="E1263" s="3" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N210"/>
+  <autoFilter ref="A1:K210"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -12452,7 +12471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -12460,194 +12479,224 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="B1" s="5" t="inlineStr">
+      <c r="B1" s="9" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
+      <c r="A2" s="10" t="inlineStr">
         <is>
           <t>ev_common_total</t>
         </is>
       </c>
-      <c r="B2" s="7" t="n">
-        <v>0.1093478260869565</v>
+      <c r="B2" s="11" t="n">
+        <v>0.1123913043478261</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="10" t="inlineStr">
         <is>
           <t>ev_uncommon_total</t>
         </is>
       </c>
-      <c r="B3" s="7" t="n">
-        <v>0.1560606060606061</v>
+      <c r="B3" s="11" t="n">
+        <v>0.1696969696969697</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>ev_rare_total</t>
         </is>
       </c>
-      <c r="B4" s="7" t="n">
-        <v>0.2604761904761905</v>
+      <c r="B4" s="11" t="n">
+        <v>0.2695238095238095</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>ev_double_rare_total</t>
         </is>
       </c>
-      <c r="B5" s="7" t="n">
-        <v>0.3288888888888888</v>
+      <c r="B5" s="11" t="n">
+        <v>0.3478888888888889</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>ev_pokeball_total</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>ev_master_ball_total</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>ev_hyper_rare_total</t>
         </is>
       </c>
-      <c r="B6" s="7" t="n">
-        <v>0.1356493506493506</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="B8" s="11" t="n">
+        <v>0.1349350649350649</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>ev_ultra_rare_total</t>
         </is>
       </c>
-      <c r="B7" s="7" t="n">
-        <v>0.6429435483870968</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="B9" s="11" t="n">
+        <v>0.6597580645161291</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="inlineStr">
         <is>
           <t>ev_SIR_total</t>
         </is>
       </c>
-      <c r="B8" s="7" t="n">
-        <v>2.301644444444444</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="B10" s="11" t="n">
+        <v>2.366622222222222</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
         <is>
           <t>ev_IR_total</t>
         </is>
       </c>
-      <c r="B9" s="7" t="n">
-        <v>1.902606382978723</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="B11" s="11" t="n">
+        <v>1.987606382978723</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="10" t="inlineStr">
         <is>
           <t>ev_reverse_total</t>
         </is>
       </c>
-      <c r="B10" s="7" t="n">
-        <v>3.066667607754564</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="B12" s="11" t="n">
+        <v>2.824572746094485</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="inlineStr">
         <is>
           <t>reverse_multiplier</t>
         </is>
       </c>
-      <c r="B11" s="7" t="n">
+      <c r="B13" s="11" t="n">
         <v>1.879338061465721</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="10" t="inlineStr">
         <is>
           <t>rare_multiplier</t>
         </is>
       </c>
-      <c r="B12" s="6" t="n">
+      <c r="B14" s="10" t="n">
         <v>1.741272168691524</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="10" t="inlineStr">
         <is>
           <t>ev_total_for_hits</t>
         </is>
       </c>
-      <c r="B13" s="7" t="n">
-        <v>4.982843726459615</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
+      <c r="B15" s="11" t="n">
+        <v>5.14892173465214</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="10" t="inlineStr">
         <is>
           <t>ev_hits_total</t>
         </is>
       </c>
-      <c r="B14" s="7" t="n">
-        <v>5.311732615348505</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
+      <c r="B16" s="11" t="n">
+        <v>5.496810623541029</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="10" t="inlineStr">
         <is>
           <t>total_ev</t>
         </is>
       </c>
-      <c r="B15" s="7" t="n">
-        <v>12.43417083607831</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr">
+      <c r="B17" s="11" t="n">
+        <v>11.07690299510566</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="10" t="inlineStr">
         <is>
           <t>net_value</t>
         </is>
       </c>
-      <c r="B16" s="7" t="n">
-        <v>1.544170836078312</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="6" t="inlineStr">
+      <c r="B18" s="11" t="n">
+        <v>0.1869029951056582</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
         <is>
           <t>roi</t>
         </is>
       </c>
-      <c r="B17" s="8" t="n">
-        <v>0.1417971382992023</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="6" t="inlineStr">
+      <c r="B19" s="12" t="n">
+        <v>0.01716280946792081</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="inlineStr">
         <is>
           <t>roi_percent</t>
         </is>
       </c>
-      <c r="B18" s="8" t="n">
-        <v>13.17971382992023</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t>hit_prob_pct</t>
-        </is>
-      </c>
-      <c r="B19" s="8" t="n">
+      <c r="B20" s="12" t="n">
+        <v>0.7162809467920814</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="10" t="inlineStr">
+        <is>
+          <t>no_hit_probability_percentage</t>
+        </is>
+      </c>
+      <c r="B21" s="12" t="n">
+        <v>68.32877110235633</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>hit_probability_percentage</t>
+        </is>
+      </c>
+      <c r="B22" s="12" t="n">
         <v>31.67122889764367</v>
       </c>
     </row>

</xml_diff>

<commit_message>
now works for 2 sets. Need to automate price pulling
</commit_message>
<xml_diff>
--- a/Expected Value and Cost Ratio Calculator Pokemon/excelDocs/scarletAndViolet151/pokemon_data.xlsx
+++ b/Expected Value and Cost Ratio Calculator Pokemon/excelDocs/scarletAndViolet151/pokemon_data.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-27375" yWindow="90" windowWidth="25260" windowHeight="11385" tabRatio="797" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="3450" yWindow="825" windowWidth="25260" windowHeight="11385" tabRatio="797" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" state="visible" r:id="rId1"/>
@@ -115,7 +115,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -138,6 +138,9 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
@@ -148,6 +151,9 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -597,7 +603,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C2" s="3" t="n">
@@ -607,7 +613,7 @@
         <v>0.06</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>0.15</v>
+        <v>0.14</v>
       </c>
       <c r="F2" s="3">
         <f>IF(B2="common", 4, IF(B2="uncommon", 3, IF(B2="rare", 1.74127216869152, 1)))</f>
@@ -639,17 +645,17 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Rare</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="C3" s="3" t="n">
         <v>21</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>0.2</v>
+        <v>0.16</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>0.55</v>
+        <v>0.53</v>
       </c>
       <c r="F3" s="3">
         <f>IF(B3="common", 4, IF(B3="uncommon", 3, IF(B3="rare", 1.74127216869152, 1)))</f>
@@ -668,14 +674,14 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Double Rare</t>
+          <t>double rare</t>
         </is>
       </c>
       <c r="C4" s="3" t="n">
         <v>90</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>1.12</v>
+        <v>1.13</v>
       </c>
       <c r="E4" s="3" t="inlineStr"/>
       <c r="F4" s="3">
@@ -683,7 +689,7 @@
         <v/>
       </c>
       <c r="H4">
-        <f>SUMPRODUCT((B2:B210="Rare") * D2:D210 * F2:F210 / C2:C210)</f>
+        <f>0.792892156862745*SUMPRODUCT((B2:B217="Rare") * D2:D217 / C2:C217)</f>
         <v/>
       </c>
     </row>
@@ -695,14 +701,14 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Ultra Rare</t>
+          <t>ultra rare</t>
         </is>
       </c>
       <c r="C5" s="3" t="n">
         <v>248</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>7.46</v>
+        <v>7.37</v>
       </c>
       <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="3">
@@ -710,7 +716,7 @@
         <v/>
       </c>
       <c r="H5">
-        <f>SUMPRODUCT((B2:B217="Double Rare") * D2:D217 * F2:F217 / C2:C217)</f>
+        <f>1.88541666666666* SUMPRODUCT((C2:C217&lt;&gt;"") * (E2:E217&lt;&gt;"") * (E2:E217 / C2:C217))</f>
         <v/>
       </c>
     </row>
@@ -722,14 +728,14 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Special Illustration Rare</t>
+          <t>special illustration rare</t>
         </is>
       </c>
       <c r="C6" s="3" t="n">
         <v>225</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>43.34</v>
+        <v>43.91</v>
       </c>
       <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="3">
@@ -737,7 +743,7 @@
         <v/>
       </c>
       <c r="H6">
-        <f>SUMPRODUCT((B2:B210="Hyper Rare") * D2:D210 * F2:F210 / C2:C210)</f>
+        <f>SUMPRODUCT((B2:B217="Illustration Rare") * D2:D217 * F2:F217 / C2:C217)</f>
         <v/>
       </c>
     </row>
@@ -749,7 +755,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C7" s="3" t="n">
@@ -759,14 +765,14 @@
         <v>0.08</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>0.64</v>
+        <v>0.61</v>
       </c>
       <c r="F7" s="3">
         <f>IF(B7="common", 4, IF(B7="uncommon", 3, IF(B7="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
       <c r="H7">
-        <f>SUMPRODUCT((B2:B217="Illustration Rare") * D2:D217 * F2:F217 / C2:C217)</f>
+        <f>SUMPRODUCT((B2:B217="Special Illustration Rare") * D2:D217 * F2:F217 / C2:C217)</f>
         <v/>
       </c>
     </row>
@@ -778,24 +784,24 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C8" s="3" t="n">
         <v>46</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>0.12</v>
+        <v>0.11</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>1.06</v>
+        <v>0.95</v>
       </c>
       <c r="F8" s="3">
         <f>IF(B8="common", 4, IF(B8="uncommon", 3, IF(B8="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
       <c r="H8">
-        <f>SUMPRODUCT((B2:B217="Special Illustration Rare") * D2:D217 * F2:F217 / C2:C217)</f>
+        <f>SUMPRODUCT((B2:B217="Double Rare") * D2:D217 * F2:F217 / C2:C217)</f>
         <v/>
       </c>
     </row>
@@ -807,24 +813,24 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C9" s="3" t="n">
         <v>46</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>0.11</v>
+        <v>0.12</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>0.65</v>
+        <v>0.67</v>
       </c>
       <c r="F9" s="3">
         <f>IF(B9="common", 4, IF(B9="uncommon", 3, IF(B9="rare", 1.74127216869152, 1)))</f>
         <v/>
       </c>
       <c r="H9">
-        <f>SUMPRODUCT((B2:B217="Ultra Rare") * D2:D217 * F2:F217 / C2:C217)</f>
+        <f>SUMPRODUCT((B2:B217="Hyper Rare") * D2:D217 * F2:F217 / C2:C217)</f>
         <v/>
       </c>
     </row>
@@ -836,14 +842,14 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Double Rare</t>
+          <t>double rare</t>
         </is>
       </c>
       <c r="C10" s="3" t="n">
         <v>90</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>0.76</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="E10" s="3" t="inlineStr"/>
       <c r="F10" s="3">
@@ -851,7 +857,7 @@
         <v/>
       </c>
       <c r="H10">
-        <f>1.88 * SUMPRODUCT((C2:C217&lt;&gt;"") * (E2:E217&lt;&gt;"") * (E2:E217 / C2:C217))</f>
+        <f>SUMPRODUCT((B2:B217="Ultra Rare") * D2:D217 * F2:F217 / C2:C217)</f>
         <v/>
       </c>
     </row>
@@ -863,14 +869,14 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Ultra Rare</t>
+          <t>ultra rare</t>
         </is>
       </c>
       <c r="C11" s="3" t="n">
         <v>248</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>4.89</v>
+        <v>4.98</v>
       </c>
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="3">
@@ -886,17 +892,17 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C12" s="3" t="n">
         <v>33</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>0.11</v>
+        <v>0.1</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>0.18</v>
+        <v>0.17</v>
       </c>
       <c r="F12" s="3">
         <f>IF(B12="common", 4, IF(B12="uncommon", 3, IF(B12="rare", 1.74127216869152, 1)))</f>
@@ -911,17 +917,17 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Rare</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="C13" s="3" t="n">
         <v>21</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>0.2</v>
+        <v>0.19</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>0.74</v>
+        <v>0.71</v>
       </c>
       <c r="F13" s="3">
         <f>IF(B13="common", 4, IF(B13="uncommon", 3, IF(B13="rare", 1.74127216869152, 1)))</f>
@@ -936,14 +942,14 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Hyper Rare</t>
+          <t>hyper rare</t>
         </is>
       </c>
       <c r="C14" s="3" t="n">
         <v>154</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>4.95</v>
+        <v>4.7</v>
       </c>
       <c r="E14" s="3" t="inlineStr"/>
       <c r="F14" s="3">
@@ -959,7 +965,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Rare</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="C15" s="3" t="n">
@@ -984,7 +990,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C16" s="3" t="n">
@@ -994,7 +1000,7 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>0.14</v>
+        <v>0.13</v>
       </c>
       <c r="F16" s="3">
         <f>IF(B16="common", 4, IF(B16="uncommon", 3, IF(B16="rare", 1.74127216869152, 1)))</f>
@@ -1009,17 +1015,17 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C17" s="3" t="n">
         <v>33</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.08</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>1.12</v>
+        <v>1.22</v>
       </c>
       <c r="F17" s="3">
         <f>IF(B17="common", 4, IF(B17="uncommon", 3, IF(B17="rare", 1.74127216869152, 1)))</f>
@@ -1034,7 +1040,7 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C18" s="3" t="n">
@@ -1044,7 +1050,7 @@
         <v>0.12</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>0.44</v>
+        <v>0.43</v>
       </c>
       <c r="F18" s="3">
         <f>IF(B18="common", 4, IF(B18="uncommon", 3, IF(B18="rare", 1.74127216869152, 1)))</f>
@@ -1059,14 +1065,14 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Ultra Rare</t>
+          <t>ultra rare</t>
         </is>
       </c>
       <c r="C19" s="3" t="n">
         <v>248</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>3.05</v>
+        <v>3.07</v>
       </c>
       <c r="E19" s="3" t="inlineStr"/>
       <c r="F19" s="3">
@@ -1082,14 +1088,14 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Double Rare</t>
+          <t>double rare</t>
         </is>
       </c>
       <c r="C20" s="3" t="n">
         <v>90</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>1.18</v>
+        <v>0.96</v>
       </c>
       <c r="E20" s="3" t="inlineStr"/>
       <c r="F20" s="3">
@@ -1105,14 +1111,14 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Ultra Rare</t>
+          <t>ultra rare</t>
         </is>
       </c>
       <c r="C21" s="3" t="n">
         <v>248</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>14.89</v>
+        <v>14.5</v>
       </c>
       <c r="E21" s="3" t="inlineStr"/>
       <c r="F21" s="3">
@@ -1128,14 +1134,14 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Special Illustration Rare</t>
+          <t>special illustration rare</t>
         </is>
       </c>
       <c r="C22" s="3" t="n">
         <v>225</v>
       </c>
       <c r="D22" s="3" t="n">
-        <v>73.55</v>
+        <v>73.09999999999999</v>
       </c>
       <c r="E22" s="3" t="inlineStr"/>
       <c r="F22" s="3">
@@ -1151,17 +1157,17 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C23" s="3" t="n">
         <v>46</v>
       </c>
       <c r="D23" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.08</v>
       </c>
       <c r="E23" s="3" t="n">
-        <v>0.24</v>
+        <v>0.23</v>
       </c>
       <c r="F23" s="3">
         <f>IF(B23="common", 4, IF(B23="uncommon", 3, IF(B23="rare", 1.74127216869152, 1)))</f>
@@ -1176,14 +1182,14 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Illustration Rare</t>
+          <t>illustration rare</t>
         </is>
       </c>
       <c r="C24" s="3" t="n">
         <v>188</v>
       </c>
       <c r="D24" s="3" t="n">
-        <v>37.52</v>
+        <v>37.01</v>
       </c>
       <c r="E24" s="3" t="inlineStr"/>
       <c r="F24" s="3">
@@ -1199,7 +1205,7 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C25" s="3" t="n">
@@ -1209,7 +1215,7 @@
         <v>0.1</v>
       </c>
       <c r="E25" s="3" t="n">
-        <v>0.16</v>
+        <v>0.15</v>
       </c>
       <c r="F25" s="3">
         <f>IF(B25="common", 4, IF(B25="uncommon", 3, IF(B25="rare", 1.74127216869152, 1)))</f>
@@ -1224,14 +1230,14 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C26" s="3" t="n">
         <v>46</v>
       </c>
       <c r="D26" s="3" t="n">
-        <v>0.04</v>
+        <v>0.05</v>
       </c>
       <c r="E26" s="3" t="n">
         <v>0.21</v>
@@ -1249,14 +1255,14 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Illustration Rare</t>
+          <t>illustration rare</t>
         </is>
       </c>
       <c r="C27" s="3" t="n">
         <v>188</v>
       </c>
       <c r="D27" s="3" t="n">
-        <v>9.56</v>
+        <v>9.460000000000001</v>
       </c>
       <c r="E27" s="3" t="inlineStr"/>
       <c r="F27" s="3">
@@ -1272,17 +1278,17 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Rare</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="C28" s="3" t="n">
         <v>21</v>
       </c>
       <c r="D28" s="3" t="n">
-        <v>0.15</v>
+        <v>0.13</v>
       </c>
       <c r="E28" s="3" t="n">
-        <v>0.65</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="F28" s="3">
         <f>IF(B28="common", 4, IF(B28="uncommon", 3, IF(B28="rare", 1.74127216869152, 1)))</f>
@@ -1297,14 +1303,14 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>Double Rare</t>
+          <t>double rare</t>
         </is>
       </c>
       <c r="C29" s="3" t="n">
         <v>90</v>
       </c>
       <c r="D29" s="3" t="n">
-        <v>4.71</v>
+        <v>5.05</v>
       </c>
       <c r="E29" s="3" t="inlineStr"/>
       <c r="F29" s="3">
@@ -1320,14 +1326,14 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Ultra Rare</t>
+          <t>ultra rare</t>
         </is>
       </c>
       <c r="C30" s="3" t="n">
         <v>248</v>
       </c>
       <c r="D30" s="3" t="n">
-        <v>31.27</v>
+        <v>31.25</v>
       </c>
       <c r="E30" s="3" t="inlineStr"/>
       <c r="F30" s="3">
@@ -1343,14 +1349,14 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>Special Illustration Rare</t>
+          <t>special illustration rare</t>
         </is>
       </c>
       <c r="C31" s="3" t="n">
         <v>225</v>
       </c>
       <c r="D31" s="3" t="n">
-        <v>210.14</v>
+        <v>214.14</v>
       </c>
       <c r="E31" s="3" t="inlineStr"/>
       <c r="F31" s="3">
@@ -1366,14 +1372,14 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C32" s="3" t="n">
         <v>46</v>
       </c>
       <c r="D32" s="3" t="n">
-        <v>0.08</v>
+        <v>0.09</v>
       </c>
       <c r="E32" s="3" t="n">
         <v>0.19</v>
@@ -1391,14 +1397,14 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Illustration Rare</t>
+          <t>illustration rare</t>
         </is>
       </c>
       <c r="C33" s="3" t="n">
         <v>188</v>
       </c>
       <c r="D33" s="3" t="n">
-        <v>52.06</v>
+        <v>51.42</v>
       </c>
       <c r="E33" s="3" t="inlineStr"/>
       <c r="F33" s="3">
@@ -1414,7 +1420,7 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C34" s="3" t="n">
@@ -1424,7 +1430,7 @@
         <v>0.1</v>
       </c>
       <c r="E34" s="3" t="n">
-        <v>0.23</v>
+        <v>0.24</v>
       </c>
       <c r="F34" s="3">
         <f>IF(B34="common", 4, IF(B34="uncommon", 3, IF(B34="rare", 1.74127216869152, 1)))</f>
@@ -1439,14 +1445,14 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>Illustration Rare</t>
+          <t>illustration rare</t>
         </is>
       </c>
       <c r="C35" s="3" t="n">
         <v>188</v>
       </c>
       <c r="D35" s="3" t="n">
-        <v>34.86</v>
+        <v>34.16</v>
       </c>
       <c r="E35" s="3" t="inlineStr"/>
       <c r="F35" s="3">
@@ -1462,7 +1468,7 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C36" s="3" t="n">
@@ -1487,7 +1493,7 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C37" s="3" t="n">
@@ -1512,17 +1518,17 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C38" s="3" t="n">
         <v>33</v>
       </c>
       <c r="D38" s="3" t="n">
-        <v>0.08</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="E38" s="3" t="n">
-        <v>0.15</v>
+        <v>0.14</v>
       </c>
       <c r="F38" s="3">
         <f>IF(B38="common", 4, IF(B38="uncommon", 3, IF(B38="rare", 1.74127216869152, 1)))</f>
@@ -1537,17 +1543,17 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C39" s="3" t="n">
         <v>46</v>
       </c>
       <c r="D39" s="3" t="n">
-        <v>0.11</v>
+        <v>0.08</v>
       </c>
       <c r="E39" s="3" t="n">
-        <v>0.14</v>
+        <v>0.13</v>
       </c>
       <c r="F39" s="3">
         <f>IF(B39="common", 4, IF(B39="uncommon", 3, IF(B39="rare", 1.74127216869152, 1)))</f>
@@ -1562,17 +1568,17 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C40" s="3" t="n">
         <v>33</v>
       </c>
       <c r="D40" s="3" t="n">
-        <v>0.1</v>
+        <v>0.11</v>
       </c>
       <c r="E40" s="3" t="n">
-        <v>0.59</v>
+        <v>0.62</v>
       </c>
       <c r="F40" s="3">
         <f>IF(B40="common", 4, IF(B40="uncommon", 3, IF(B40="rare", 1.74127216869152, 1)))</f>
@@ -1587,17 +1593,17 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C41" s="3" t="n">
         <v>33</v>
       </c>
       <c r="D41" s="3" t="n">
-        <v>0.09</v>
+        <v>0.1</v>
       </c>
       <c r="E41" s="3" t="n">
-        <v>0.43</v>
+        <v>0.42</v>
       </c>
       <c r="F41" s="3">
         <f>IF(B41="common", 4, IF(B41="uncommon", 3, IF(B41="rare", 1.74127216869152, 1)))</f>
@@ -1612,14 +1618,14 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>Ultra Rare</t>
+          <t>ultra rare</t>
         </is>
       </c>
       <c r="C42" s="3" t="n">
         <v>248</v>
       </c>
       <c r="D42" s="3" t="n">
-        <v>4.04</v>
+        <v>3.92</v>
       </c>
       <c r="E42" s="3" t="inlineStr"/>
       <c r="F42" s="3">
@@ -1635,17 +1641,17 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C43" s="3" t="n">
         <v>33</v>
       </c>
       <c r="D43" s="3" t="n">
-        <v>0.06</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="E43" s="3" t="n">
-        <v>0.14</v>
+        <v>0.13</v>
       </c>
       <c r="F43" s="3">
         <f>IF(B43="common", 4, IF(B43="uncommon", 3, IF(B43="rare", 1.74127216869152, 1)))</f>
@@ -1660,14 +1666,14 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C44" s="3" t="n">
         <v>46</v>
       </c>
       <c r="D44" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06</v>
       </c>
       <c r="E44" s="3" t="n">
         <v>0.15</v>
@@ -1685,17 +1691,17 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>Rare</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="C45" s="3" t="n">
         <v>21</v>
       </c>
       <c r="D45" s="3" t="n">
-        <v>0.26</v>
+        <v>0.27</v>
       </c>
       <c r="E45" s="3" t="n">
-        <v>0.64</v>
+        <v>0.63</v>
       </c>
       <c r="F45" s="3">
         <f>IF(B45="common", 4, IF(B45="uncommon", 3, IF(B45="rare", 1.74127216869152, 1)))</f>
@@ -1710,14 +1716,14 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>Rare</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="C46" s="3" t="n">
         <v>21</v>
       </c>
       <c r="D46" s="3" t="n">
-        <v>0.34</v>
+        <v>0.47</v>
       </c>
       <c r="E46" s="3" t="inlineStr"/>
       <c r="F46" s="3">
@@ -1733,17 +1739,17 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>Rare</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="C47" s="3" t="n">
         <v>21</v>
       </c>
       <c r="D47" s="3" t="n">
-        <v>0.14</v>
+        <v>0.13</v>
       </c>
       <c r="E47" s="3" t="n">
-        <v>0.63</v>
+        <v>0.62</v>
       </c>
       <c r="F47" s="3">
         <f>IF(B47="common", 4, IF(B47="uncommon", 3, IF(B47="rare", 1.74127216869152, 1)))</f>
@@ -1758,7 +1764,7 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C48" s="3" t="n">
@@ -1783,17 +1789,17 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C49" s="3" t="n">
         <v>33</v>
       </c>
       <c r="D49" s="3" t="n">
-        <v>0.11</v>
+        <v>0.13</v>
       </c>
       <c r="E49" s="3" t="n">
-        <v>2</v>
+        <v>2.18</v>
       </c>
       <c r="F49" s="3">
         <f>IF(B49="common", 4, IF(B49="uncommon", 3, IF(B49="rare", 1.74127216869152, 1)))</f>
@@ -1808,14 +1814,14 @@
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>Illustration Rare</t>
+          <t>illustration rare</t>
         </is>
       </c>
       <c r="C50" s="3" t="n">
         <v>188</v>
       </c>
       <c r="D50" s="3" t="n">
-        <v>25.78</v>
+        <v>25.53</v>
       </c>
       <c r="E50" s="3" t="inlineStr"/>
       <c r="F50" s="3">
@@ -1831,17 +1837,17 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>Rare</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="C51" s="3" t="n">
         <v>21</v>
       </c>
       <c r="D51" s="3" t="n">
-        <v>0.41</v>
+        <v>0.37</v>
       </c>
       <c r="E51" s="3" t="n">
-        <v>1.32</v>
+        <v>1.3</v>
       </c>
       <c r="F51" s="3">
         <f>IF(B51="common", 4, IF(B51="uncommon", 3, IF(B51="rare", 1.74127216869152, 1)))</f>
@@ -1856,17 +1862,17 @@
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C52" s="3" t="n">
         <v>46</v>
       </c>
       <c r="D52" s="3" t="n">
-        <v>0.11</v>
+        <v>0.12</v>
       </c>
       <c r="E52" s="3" t="n">
-        <v>0.18</v>
+        <v>0.17</v>
       </c>
       <c r="F52" s="3">
         <f>IF(B52="common", 4, IF(B52="uncommon", 3, IF(B52="rare", 1.74127216869152, 1)))</f>
@@ -1881,7 +1887,7 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C53" s="3" t="n">
@@ -1891,7 +1897,7 @@
         <v>0.05</v>
       </c>
       <c r="E53" s="3" t="n">
-        <v>0.13</v>
+        <v>0.12</v>
       </c>
       <c r="F53" s="3">
         <f>IF(B53="common", 4, IF(B53="uncommon", 3, IF(B53="rare", 1.74127216869152, 1)))</f>
@@ -1906,7 +1912,7 @@
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C54" s="3" t="n">
@@ -1931,17 +1937,17 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C55" s="3" t="n">
         <v>46</v>
       </c>
       <c r="D55" s="3" t="n">
-        <v>0.09</v>
+        <v>0.1</v>
       </c>
       <c r="E55" s="3" t="n">
-        <v>0.24</v>
+        <v>0.23</v>
       </c>
       <c r="F55" s="3">
         <f>IF(B55="common", 4, IF(B55="uncommon", 3, IF(B55="rare", 1.74127216869152, 1)))</f>
@@ -1956,7 +1962,7 @@
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C56" s="3" t="n">
@@ -1966,7 +1972,7 @@
         <v>0.05</v>
       </c>
       <c r="E56" s="3" t="n">
-        <v>0.2</v>
+        <v>0.19</v>
       </c>
       <c r="F56" s="3">
         <f>IF(B56="common", 4, IF(B56="uncommon", 3, IF(B56="rare", 1.74127216869152, 1)))</f>
@@ -1981,7 +1987,7 @@
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C57" s="3" t="n">
@@ -1991,7 +1997,7 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="E57" s="3" t="n">
-        <v>0.5</v>
+        <v>0.51</v>
       </c>
       <c r="F57" s="3">
         <f>IF(B57="common", 4, IF(B57="uncommon", 3, IF(B57="rare", 1.74127216869152, 1)))</f>
@@ -2006,7 +2012,7 @@
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>Rare</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="C58" s="3" t="n">
@@ -2016,7 +2022,7 @@
         <v>0.13</v>
       </c>
       <c r="E58" s="3" t="n">
-        <v>1.27</v>
+        <v>1.23</v>
       </c>
       <c r="F58" s="3">
         <f>IF(B58="common", 4, IF(B58="uncommon", 3, IF(B58="rare", 1.74127216869152, 1)))</f>
@@ -2031,7 +2037,7 @@
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C59" s="3" t="n">
@@ -2041,7 +2047,7 @@
         <v>0.16</v>
       </c>
       <c r="E59" s="3" t="n">
-        <v>1.41</v>
+        <v>1.43</v>
       </c>
       <c r="F59" s="3">
         <f>IF(B59="common", 4, IF(B59="uncommon", 3, IF(B59="rare", 1.74127216869152, 1)))</f>
@@ -2056,17 +2062,17 @@
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C60" s="3" t="n">
         <v>33</v>
       </c>
       <c r="D60" s="3" t="n">
-        <v>0.11</v>
+        <v>0.15</v>
       </c>
       <c r="E60" s="3" t="n">
-        <v>0.8</v>
+        <v>0.84</v>
       </c>
       <c r="F60" s="3">
         <f>IF(B60="common", 4, IF(B60="uncommon", 3, IF(B60="rare", 1.74127216869152, 1)))</f>
@@ -2081,14 +2087,14 @@
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>Ultra Rare</t>
+          <t>ultra rare</t>
         </is>
       </c>
       <c r="C61" s="3" t="n">
         <v>248</v>
       </c>
       <c r="D61" s="3" t="n">
-        <v>6.99</v>
+        <v>6.92</v>
       </c>
       <c r="E61" s="3" t="inlineStr"/>
       <c r="F61" s="3">
@@ -2104,14 +2110,14 @@
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>Special Illustration Rare</t>
+          <t>special illustration rare</t>
         </is>
       </c>
       <c r="C62" s="3" t="n">
         <v>225</v>
       </c>
       <c r="D62" s="3" t="n">
-        <v>14.98</v>
+        <v>14.48</v>
       </c>
       <c r="E62" s="3" t="inlineStr"/>
       <c r="F62" s="3">
@@ -2127,7 +2133,7 @@
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C63" s="3" t="n">
@@ -2152,7 +2158,7 @@
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C64" s="3" t="n">
@@ -2162,7 +2168,7 @@
         <v>0.1</v>
       </c>
       <c r="E64" s="3" t="n">
-        <v>1.26</v>
+        <v>1.31</v>
       </c>
       <c r="F64" s="3">
         <f>IF(B64="common", 4, IF(B64="uncommon", 3, IF(B64="rare", 1.74127216869152, 1)))</f>
@@ -2177,7 +2183,7 @@
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C65" s="3" t="n">
@@ -2187,7 +2193,7 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="E65" s="3" t="n">
-        <v>0.13</v>
+        <v>0.14</v>
       </c>
       <c r="F65" s="3">
         <f>IF(B65="common", 4, IF(B65="uncommon", 3, IF(B65="rare", 1.74127216869152, 1)))</f>
@@ -2202,17 +2208,17 @@
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C66" s="3" t="n">
         <v>33</v>
       </c>
       <c r="D66" s="3" t="n">
-        <v>0.08</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="E66" s="3" t="n">
-        <v>0.14</v>
+        <v>0.15</v>
       </c>
       <c r="F66" s="3">
         <f>IF(B66="common", 4, IF(B66="uncommon", 3, IF(B66="rare", 1.74127216869152, 1)))</f>
@@ -2227,14 +2233,14 @@
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>Rare</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="C67" s="3" t="n">
         <v>21</v>
       </c>
       <c r="D67" s="3" t="n">
-        <v>0.25</v>
+        <v>0.29</v>
       </c>
       <c r="E67" s="3" t="n">
         <v>1.08</v>
@@ -2252,14 +2258,14 @@
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C68" s="3" t="n">
         <v>46</v>
       </c>
       <c r="D68" s="3" t="n">
-        <v>0.08</v>
+        <v>0.09</v>
       </c>
       <c r="E68" s="3" t="n">
         <v>0.18</v>
@@ -2277,17 +2283,17 @@
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>Rare</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="C69" s="3" t="n">
         <v>21</v>
       </c>
       <c r="D69" s="3" t="n">
-        <v>0.27</v>
+        <v>0.3</v>
       </c>
       <c r="E69" s="3" t="n">
-        <v>1.78</v>
+        <v>1.82</v>
       </c>
       <c r="F69" s="3">
         <f>IF(B69="common", 4, IF(B69="uncommon", 3, IF(B69="rare", 1.74127216869152, 1)))</f>
@@ -2302,7 +2308,7 @@
       </c>
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C70" s="3" t="n">
@@ -2327,17 +2333,17 @@
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C71" s="3" t="n">
         <v>33</v>
       </c>
       <c r="D71" s="3" t="n">
-        <v>0.1</v>
+        <v>0.12</v>
       </c>
       <c r="E71" s="3" t="n">
-        <v>1.03</v>
+        <v>0.98</v>
       </c>
       <c r="F71" s="3">
         <f>IF(B71="common", 4, IF(B71="uncommon", 3, IF(B71="rare", 1.74127216869152, 1)))</f>
@@ -2352,14 +2358,14 @@
       </c>
       <c r="B72" s="3" t="inlineStr">
         <is>
-          <t>Ultra Rare</t>
+          <t>ultra rare</t>
         </is>
       </c>
       <c r="C72" s="3" t="n">
         <v>248</v>
       </c>
       <c r="D72" s="3" t="n">
-        <v>4.99</v>
+        <v>5.05</v>
       </c>
       <c r="E72" s="3" t="inlineStr"/>
       <c r="F72" s="3">
@@ -2375,14 +2381,14 @@
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>Special Illustration Rare</t>
+          <t>special illustration rare</t>
         </is>
       </c>
       <c r="C73" s="3" t="n">
         <v>225</v>
       </c>
       <c r="D73" s="3" t="n">
-        <v>15.6</v>
+        <v>13.93</v>
       </c>
       <c r="E73" s="3" t="inlineStr"/>
       <c r="F73" s="3">
@@ -2398,14 +2404,14 @@
       </c>
       <c r="B74" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C74" s="3" t="n">
         <v>33</v>
       </c>
       <c r="D74" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.08</v>
       </c>
       <c r="E74" s="3" t="n">
         <v>0.21</v>
@@ -2423,7 +2429,7 @@
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C75" s="3" t="n">
@@ -2448,17 +2454,17 @@
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C76" s="3" t="n">
         <v>46</v>
       </c>
       <c r="D76" s="3" t="n">
-        <v>0.04</v>
+        <v>0.05</v>
       </c>
       <c r="E76" s="3" t="n">
-        <v>0.16</v>
+        <v>0.15</v>
       </c>
       <c r="F76" s="3">
         <f>IF(B76="common", 4, IF(B76="uncommon", 3, IF(B76="rare", 1.74127216869152, 1)))</f>
@@ -2473,7 +2479,7 @@
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C77" s="3" t="n">
@@ -2498,14 +2504,14 @@
       </c>
       <c r="B78" s="3" t="inlineStr">
         <is>
-          <t>Double Rare</t>
+          <t>double rare</t>
         </is>
       </c>
       <c r="C78" s="3" t="n">
         <v>90</v>
       </c>
       <c r="D78" s="3" t="n">
-        <v>0.62</v>
+        <v>0.63</v>
       </c>
       <c r="E78" s="3" t="inlineStr"/>
       <c r="F78" s="3">
@@ -2521,14 +2527,14 @@
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>Ultra Rare</t>
+          <t>ultra rare</t>
         </is>
       </c>
       <c r="C79" s="3" t="n">
         <v>248</v>
       </c>
       <c r="D79" s="3" t="n">
-        <v>5.18</v>
+        <v>4.83</v>
       </c>
       <c r="E79" s="3" t="inlineStr"/>
       <c r="F79" s="3">
@@ -2544,17 +2550,17 @@
       </c>
       <c r="B80" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C80" s="3" t="n">
         <v>33</v>
       </c>
       <c r="D80" s="3" t="n">
-        <v>0.26</v>
+        <v>0.14</v>
       </c>
       <c r="E80" s="3" t="n">
-        <v>0.73</v>
+        <v>0.71</v>
       </c>
       <c r="F80" s="3">
         <f>IF(B80="common", 4, IF(B80="uncommon", 3, IF(B80="rare", 1.74127216869152, 1)))</f>
@@ -2569,7 +2575,7 @@
       </c>
       <c r="B81" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C81" s="3" t="n">
@@ -2594,14 +2600,14 @@
       </c>
       <c r="B82" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C82" s="3" t="n">
         <v>46</v>
       </c>
       <c r="D82" s="3" t="n">
-        <v>0.06</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="E82" s="3" t="n">
         <v>0.15</v>
@@ -2619,7 +2625,7 @@
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C83" s="3" t="n">
@@ -2644,17 +2650,17 @@
       </c>
       <c r="B84" s="3" t="inlineStr">
         <is>
-          <t>Rare</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="C84" s="3" t="n">
         <v>21</v>
       </c>
       <c r="D84" s="3" t="n">
-        <v>0.19</v>
+        <v>0.17</v>
       </c>
       <c r="E84" s="3" t="n">
-        <v>0.76</v>
+        <v>0.85</v>
       </c>
       <c r="F84" s="3">
         <f>IF(B84="common", 4, IF(B84="uncommon", 3, IF(B84="rare", 1.74127216869152, 1)))</f>
@@ -2669,17 +2675,17 @@
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C85" s="3" t="n">
         <v>33</v>
       </c>
       <c r="D85" s="3" t="n">
-        <v>0.1</v>
+        <v>0.09</v>
       </c>
       <c r="E85" s="3" t="n">
-        <v>0.21</v>
+        <v>0.2</v>
       </c>
       <c r="F85" s="3">
         <f>IF(B85="common", 4, IF(B85="uncommon", 3, IF(B85="rare", 1.74127216869152, 1)))</f>
@@ -2694,17 +2700,17 @@
       </c>
       <c r="B86" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C86" s="3" t="n">
         <v>33</v>
       </c>
       <c r="D86" s="3" t="n">
-        <v>0.09</v>
+        <v>0.1</v>
       </c>
       <c r="E86" s="3" t="n">
-        <v>1.5</v>
+        <v>1.51</v>
       </c>
       <c r="F86" s="3">
         <f>IF(B86="common", 4, IF(B86="uncommon", 3, IF(B86="rare", 1.74127216869152, 1)))</f>
@@ -2719,17 +2725,17 @@
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C87" s="3" t="n">
         <v>33</v>
       </c>
       <c r="D87" s="3" t="n">
-        <v>0.08</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="E87" s="3" t="n">
-        <v>1.12</v>
+        <v>1.26</v>
       </c>
       <c r="F87" s="3">
         <f>IF(B87="common", 4, IF(B87="uncommon", 3, IF(B87="rare", 1.74127216869152, 1)))</f>
@@ -2744,7 +2750,7 @@
       </c>
       <c r="B88" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C88" s="3" t="n">
@@ -2754,7 +2760,7 @@
         <v>0.06</v>
       </c>
       <c r="E88" s="3" t="n">
-        <v>0.14</v>
+        <v>0.13</v>
       </c>
       <c r="F88" s="3">
         <f>IF(B88="common", 4, IF(B88="uncommon", 3, IF(B88="rare", 1.74127216869152, 1)))</f>
@@ -2769,7 +2775,7 @@
       </c>
       <c r="B89" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C89" s="3" t="n">
@@ -2779,7 +2785,7 @@
         <v>0.1</v>
       </c>
       <c r="E89" s="3" t="n">
-        <v>1.3</v>
+        <v>1.32</v>
       </c>
       <c r="F89" s="3">
         <f>IF(B89="common", 4, IF(B89="uncommon", 3, IF(B89="rare", 1.74127216869152, 1)))</f>
@@ -2794,7 +2800,7 @@
       </c>
       <c r="B90" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C90" s="3" t="n">
@@ -2819,14 +2825,14 @@
       </c>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>Illustration Rare</t>
+          <t>illustration rare</t>
         </is>
       </c>
       <c r="C91" s="3" t="n">
         <v>188</v>
       </c>
       <c r="D91" s="3" t="n">
-        <v>26.26</v>
+        <v>26.78</v>
       </c>
       <c r="E91" s="3" t="inlineStr"/>
       <c r="F91" s="3">
@@ -2842,17 +2848,17 @@
       </c>
       <c r="B92" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C92" s="3" t="n">
         <v>46</v>
       </c>
       <c r="D92" s="3" t="n">
-        <v>0.09</v>
+        <v>0.1</v>
       </c>
       <c r="E92" s="3" t="n">
-        <v>0.22</v>
+        <v>0.21</v>
       </c>
       <c r="F92" s="3">
         <f>IF(B92="common", 4, IF(B92="uncommon", 3, IF(B92="rare", 1.74127216869152, 1)))</f>
@@ -2867,17 +2873,17 @@
       </c>
       <c r="B93" s="3" t="inlineStr">
         <is>
-          <t>Rare</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="C93" s="3" t="n">
         <v>21</v>
       </c>
       <c r="D93" s="3" t="n">
-        <v>0.25</v>
+        <v>0.24</v>
       </c>
       <c r="E93" s="3" t="n">
-        <v>2.24</v>
+        <v>2.36</v>
       </c>
       <c r="F93" s="3">
         <f>IF(B93="common", 4, IF(B93="uncommon", 3, IF(B93="rare", 1.74127216869152, 1)))</f>
@@ -2892,14 +2898,14 @@
       </c>
       <c r="B94" s="3" t="inlineStr">
         <is>
-          <t>Double Rare</t>
+          <t>double rare</t>
         </is>
       </c>
       <c r="C94" s="3" t="n">
         <v>90</v>
       </c>
       <c r="D94" s="3" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.98</v>
       </c>
       <c r="E94" s="3" t="inlineStr"/>
       <c r="F94" s="3">
@@ -2915,14 +2921,14 @@
       </c>
       <c r="B95" s="3" t="inlineStr">
         <is>
-          <t>Ultra Rare</t>
+          <t>ultra rare</t>
         </is>
       </c>
       <c r="C95" s="3" t="n">
         <v>248</v>
       </c>
       <c r="D95" s="3" t="n">
-        <v>5.3</v>
+        <v>5.09</v>
       </c>
       <c r="E95" s="3" t="inlineStr"/>
       <c r="F95" s="3">
@@ -2938,7 +2944,7 @@
       </c>
       <c r="B96" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C96" s="3" t="n">
@@ -2948,7 +2954,7 @@
         <v>0.09</v>
       </c>
       <c r="E96" s="3" t="n">
-        <v>1.12</v>
+        <v>1.06</v>
       </c>
       <c r="F96" s="3">
         <f>IF(B96="common", 4, IF(B96="uncommon", 3, IF(B96="rare", 1.74127216869152, 1)))</f>
@@ -2963,17 +2969,17 @@
       </c>
       <c r="B97" s="3" t="inlineStr">
         <is>
-          <t>Rare</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="C97" s="3" t="n">
         <v>21</v>
       </c>
       <c r="D97" s="3" t="n">
-        <v>0.13</v>
+        <v>0.12</v>
       </c>
       <c r="E97" s="3" t="n">
-        <v>0.89</v>
+        <v>0.87</v>
       </c>
       <c r="F97" s="3">
         <f>IF(B97="common", 4, IF(B97="uncommon", 3, IF(B97="rare", 1.74127216869152, 1)))</f>
@@ -2988,17 +2994,17 @@
       </c>
       <c r="B98" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C98" s="3" t="n">
         <v>33</v>
       </c>
       <c r="D98" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.1</v>
       </c>
       <c r="E98" s="3" t="n">
-        <v>0.2</v>
+        <v>0.19</v>
       </c>
       <c r="F98" s="3">
         <f>IF(B98="common", 4, IF(B98="uncommon", 3, IF(B98="rare", 1.74127216869152, 1)))</f>
@@ -3013,7 +3019,7 @@
       </c>
       <c r="B99" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C99" s="3" t="n">
@@ -3023,7 +3029,7 @@
         <v>0.1</v>
       </c>
       <c r="E99" s="3" t="n">
-        <v>2.01</v>
+        <v>2.1</v>
       </c>
       <c r="F99" s="3">
         <f>IF(B99="common", 4, IF(B99="uncommon", 3, IF(B99="rare", 1.74127216869152, 1)))</f>
@@ -3038,14 +3044,14 @@
       </c>
       <c r="B100" s="3" t="inlineStr">
         <is>
-          <t>Double Rare</t>
+          <t>double rare</t>
         </is>
       </c>
       <c r="C100" s="3" t="n">
         <v>90</v>
       </c>
       <c r="D100" s="3" t="n">
-        <v>0.59</v>
+        <v>0.7</v>
       </c>
       <c r="E100" s="3" t="inlineStr"/>
       <c r="F100" s="3">
@@ -3061,14 +3067,14 @@
       </c>
       <c r="B101" s="3" t="inlineStr">
         <is>
-          <t>Ultra Rare</t>
+          <t>ultra rare</t>
         </is>
       </c>
       <c r="C101" s="3" t="n">
         <v>248</v>
       </c>
       <c r="D101" s="3" t="n">
-        <v>5.8</v>
+        <v>5.55</v>
       </c>
       <c r="E101" s="3" t="inlineStr"/>
       <c r="F101" s="3">
@@ -3084,17 +3090,17 @@
       </c>
       <c r="B102" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C102" s="3" t="n">
         <v>33</v>
       </c>
       <c r="D102" s="3" t="n">
-        <v>0.11</v>
+        <v>0.12</v>
       </c>
       <c r="E102" s="3" t="n">
-        <v>1.26</v>
+        <v>1.3</v>
       </c>
       <c r="F102" s="3">
         <f>IF(B102="common", 4, IF(B102="uncommon", 3, IF(B102="rare", 1.74127216869152, 1)))</f>
@@ -3109,7 +3115,7 @@
       </c>
       <c r="B103" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C103" s="3" t="n">
@@ -3134,7 +3140,7 @@
       </c>
       <c r="B104" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C104" s="3" t="n">
@@ -3159,7 +3165,7 @@
       </c>
       <c r="B105" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C105" s="3" t="n">
@@ -3169,7 +3175,7 @@
         <v>0.08</v>
       </c>
       <c r="E105" s="3" t="n">
-        <v>1.65</v>
+        <v>1.63</v>
       </c>
       <c r="F105" s="3">
         <f>IF(B105="common", 4, IF(B105="uncommon", 3, IF(B105="rare", 1.74127216869152, 1)))</f>
@@ -3184,17 +3190,17 @@
       </c>
       <c r="B106" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C106" s="3" t="n">
         <v>33</v>
       </c>
       <c r="D106" s="3" t="n">
-        <v>0.11</v>
+        <v>0.12</v>
       </c>
       <c r="E106" s="3" t="n">
-        <v>0.52</v>
+        <v>0.54</v>
       </c>
       <c r="F106" s="3">
         <f>IF(B106="common", 4, IF(B106="uncommon", 3, IF(B106="rare", 1.74127216869152, 1)))</f>
@@ -3209,17 +3215,17 @@
       </c>
       <c r="B107" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C107" s="3" t="n">
         <v>46</v>
       </c>
       <c r="D107" s="3" t="n">
-        <v>0.09</v>
+        <v>0.08</v>
       </c>
       <c r="E107" s="3" t="n">
-        <v>0.15</v>
+        <v>0.14</v>
       </c>
       <c r="F107" s="3">
         <f>IF(B107="common", 4, IF(B107="uncommon", 3, IF(B107="rare", 1.74127216869152, 1)))</f>
@@ -3234,17 +3240,17 @@
       </c>
       <c r="B108" s="3" t="inlineStr">
         <is>
-          <t>Rare</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="C108" s="3" t="n">
         <v>21</v>
       </c>
       <c r="D108" s="3" t="n">
-        <v>0.17</v>
+        <v>0.16</v>
       </c>
       <c r="E108" s="3" t="n">
-        <v>0.66</v>
+        <v>0.63</v>
       </c>
       <c r="F108" s="3">
         <f>IF(B108="common", 4, IF(B108="uncommon", 3, IF(B108="rare", 1.74127216869152, 1)))</f>
@@ -3259,17 +3265,17 @@
       </c>
       <c r="B109" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C109" s="3" t="n">
         <v>33</v>
       </c>
       <c r="D109" s="3" t="n">
-        <v>0.1</v>
+        <v>0.09</v>
       </c>
       <c r="E109" s="3" t="n">
-        <v>0.15</v>
+        <v>0.14</v>
       </c>
       <c r="F109" s="3">
         <f>IF(B109="common", 4, IF(B109="uncommon", 3, IF(B109="rare", 1.74127216869152, 1)))</f>
@@ -3284,14 +3290,14 @@
       </c>
       <c r="B110" s="3" t="inlineStr">
         <is>
-          <t>Illustration Rare</t>
+          <t>illustration rare</t>
         </is>
       </c>
       <c r="C110" s="3" t="n">
         <v>188</v>
       </c>
       <c r="D110" s="3" t="n">
-        <v>11.24</v>
+        <v>11.22</v>
       </c>
       <c r="E110" s="3" t="inlineStr"/>
       <c r="F110" s="3">
@@ -3307,17 +3313,17 @@
       </c>
       <c r="B111" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C111" s="3" t="n">
         <v>46</v>
       </c>
       <c r="D111" s="3" t="n">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="E111" s="3" t="n">
-        <v>0.15</v>
+        <v>0.13</v>
       </c>
       <c r="F111" s="3">
         <f>IF(B111="common", 4, IF(B111="uncommon", 3, IF(B111="rare", 1.74127216869152, 1)))</f>
@@ -3332,7 +3338,7 @@
       </c>
       <c r="B112" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C112" s="3" t="n">
@@ -3342,7 +3348,7 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="E112" s="3" t="n">
-        <v>0.22</v>
+        <v>0.24</v>
       </c>
       <c r="F112" s="3">
         <f>IF(B112="common", 4, IF(B112="uncommon", 3, IF(B112="rare", 1.74127216869152, 1)))</f>
@@ -3357,14 +3363,14 @@
       </c>
       <c r="B113" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C113" s="3" t="n">
         <v>46</v>
       </c>
       <c r="D113" s="3" t="n">
-        <v>0.08</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="E113" s="3" t="n">
         <v>0.9399999999999999</v>
@@ -3382,7 +3388,7 @@
       </c>
       <c r="B114" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C114" s="3" t="n">
@@ -3392,7 +3398,7 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="E114" s="3" t="n">
-        <v>0.15</v>
+        <v>0.14</v>
       </c>
       <c r="F114" s="3">
         <f>IF(B114="common", 4, IF(B114="uncommon", 3, IF(B114="rare", 1.74127216869152, 1)))</f>
@@ -3407,14 +3413,14 @@
       </c>
       <c r="B115" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C115" s="3" t="n">
         <v>33</v>
       </c>
       <c r="D115" s="3" t="n">
-        <v>0.11</v>
+        <v>0.1</v>
       </c>
       <c r="E115" s="3" t="n">
         <v>0.13</v>
@@ -3432,14 +3438,14 @@
       </c>
       <c r="B116" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C116" s="3" t="n">
         <v>46</v>
       </c>
       <c r="D116" s="3" t="n">
-        <v>0.08</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="E116" s="3" t="n">
         <v>0.13</v>
@@ -3457,7 +3463,7 @@
       </c>
       <c r="B117" s="3" t="inlineStr">
         <is>
-          <t>Rare</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="C117" s="3" t="n">
@@ -3467,7 +3473,7 @@
         <v>0.16</v>
       </c>
       <c r="E117" s="3" t="n">
-        <v>0.54</v>
+        <v>0.58</v>
       </c>
       <c r="F117" s="3">
         <f>IF(B117="common", 4, IF(B117="uncommon", 3, IF(B117="rare", 1.74127216869152, 1)))</f>
@@ -3482,7 +3488,7 @@
       </c>
       <c r="B118" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C118" s="3" t="n">
@@ -3492,7 +3498,7 @@
         <v>0.06</v>
       </c>
       <c r="E118" s="3" t="n">
-        <v>0.17</v>
+        <v>0.15</v>
       </c>
       <c r="F118" s="3">
         <f>IF(B118="common", 4, IF(B118="uncommon", 3, IF(B118="rare", 1.74127216869152, 1)))</f>
@@ -3507,17 +3513,17 @@
       </c>
       <c r="B119" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C119" s="3" t="n">
         <v>46</v>
       </c>
       <c r="D119" s="3" t="n">
-        <v>0.1</v>
+        <v>0.11</v>
       </c>
       <c r="E119" s="3" t="n">
-        <v>2.22</v>
+        <v>2.31</v>
       </c>
       <c r="F119" s="3">
         <f>IF(B119="common", 4, IF(B119="uncommon", 3, IF(B119="rare", 1.74127216869152, 1)))</f>
@@ -3532,14 +3538,14 @@
       </c>
       <c r="B120" s="3" t="inlineStr">
         <is>
-          <t>Double Rare</t>
+          <t>double rare</t>
         </is>
       </c>
       <c r="C120" s="3" t="n">
         <v>90</v>
       </c>
       <c r="D120" s="3" t="n">
-        <v>7.21</v>
+        <v>6.62</v>
       </c>
       <c r="E120" s="3" t="inlineStr"/>
       <c r="F120" s="3">
@@ -3555,14 +3561,14 @@
       </c>
       <c r="B121" s="3" t="inlineStr">
         <is>
-          <t>Ultra Rare</t>
+          <t>ultra rare</t>
         </is>
       </c>
       <c r="C121" s="3" t="n">
         <v>248</v>
       </c>
       <c r="D121" s="3" t="n">
-        <v>19.11</v>
+        <v>18.71</v>
       </c>
       <c r="E121" s="3" t="inlineStr"/>
       <c r="F121" s="3">
@@ -3578,14 +3584,14 @@
       </c>
       <c r="B122" s="3" t="inlineStr">
         <is>
-          <t>Hyper Rare</t>
+          <t>hyper rare</t>
         </is>
       </c>
       <c r="C122" s="3" t="n">
         <v>154</v>
       </c>
       <c r="D122" s="3" t="n">
-        <v>13.27</v>
+        <v>13.41</v>
       </c>
       <c r="E122" s="3" t="inlineStr"/>
       <c r="F122" s="3">
@@ -3601,14 +3607,14 @@
       </c>
       <c r="B123" s="3" t="inlineStr">
         <is>
-          <t>Double Rare</t>
+          <t>double rare</t>
         </is>
       </c>
       <c r="C123" s="3" t="n">
         <v>90</v>
       </c>
       <c r="D123" s="3" t="n">
-        <v>9.75</v>
+        <v>9.140000000000001</v>
       </c>
       <c r="E123" s="3" t="inlineStr"/>
       <c r="F123" s="3">
@@ -3624,17 +3630,17 @@
       </c>
       <c r="B124" s="3" t="inlineStr">
         <is>
-          <t>Rare</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="C124" s="3" t="n">
         <v>21</v>
       </c>
       <c r="D124" s="3" t="n">
-        <v>0.51</v>
+        <v>0.55</v>
       </c>
       <c r="E124" s="3" t="n">
-        <v>1.58</v>
+        <v>1.57</v>
       </c>
       <c r="F124" s="3">
         <f>IF(B124="common", 4, IF(B124="uncommon", 3, IF(B124="rare", 1.74127216869152, 1)))</f>
@@ -3649,7 +3655,7 @@
       </c>
       <c r="B125" s="3" t="inlineStr">
         <is>
-          <t>Rare</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="C125" s="3" t="n">
@@ -3659,7 +3665,7 @@
         <v>0.21</v>
       </c>
       <c r="E125" s="3" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.67</v>
       </c>
       <c r="F125" s="3">
         <f>IF(B125="common", 4, IF(B125="uncommon", 3, IF(B125="rare", 1.74127216869152, 1)))</f>
@@ -3674,7 +3680,7 @@
       </c>
       <c r="B126" s="3" t="inlineStr">
         <is>
-          <t>Rare</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="C126" s="3" t="n">
@@ -3699,14 +3705,14 @@
       </c>
       <c r="B127" s="3" t="inlineStr">
         <is>
-          <t>Illustration Rare</t>
+          <t>illustration rare</t>
         </is>
       </c>
       <c r="C127" s="3" t="n">
         <v>188</v>
       </c>
       <c r="D127" s="3" t="n">
-        <v>5.79</v>
+        <v>5.49</v>
       </c>
       <c r="E127" s="3" t="inlineStr"/>
       <c r="F127" s="3">
@@ -3722,14 +3728,14 @@
       </c>
       <c r="B128" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C128" s="3" t="n">
         <v>33</v>
       </c>
       <c r="D128" s="3" t="n">
-        <v>0.09</v>
+        <v>0.08</v>
       </c>
       <c r="E128" s="3" t="n">
         <v>0.22</v>
@@ -3747,7 +3753,7 @@
       </c>
       <c r="B129" s="3" t="inlineStr">
         <is>
-          <t>Rare</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="C129" s="3" t="n">
@@ -3757,7 +3763,7 @@
         <v>0.19</v>
       </c>
       <c r="E129" s="3" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.77</v>
       </c>
       <c r="F129" s="3">
         <f>IF(B129="common", 4, IF(B129="uncommon", 3, IF(B129="rare", 1.74127216869152, 1)))</f>
@@ -3772,14 +3778,14 @@
       </c>
       <c r="B130" s="3" t="inlineStr">
         <is>
-          <t>Illustration Rare</t>
+          <t>illustration rare</t>
         </is>
       </c>
       <c r="C130" s="3" t="n">
         <v>188</v>
       </c>
       <c r="D130" s="3" t="n">
-        <v>9.58</v>
+        <v>9.9</v>
       </c>
       <c r="E130" s="3" t="inlineStr"/>
       <c r="F130" s="3">
@@ -3795,7 +3801,7 @@
       </c>
       <c r="B131" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C131" s="3" t="n">
@@ -3805,7 +3811,7 @@
         <v>0.06</v>
       </c>
       <c r="E131" s="3" t="n">
-        <v>0.21</v>
+        <v>0.22</v>
       </c>
       <c r="F131" s="3">
         <f>IF(B131="common", 4, IF(B131="uncommon", 3, IF(B131="rare", 1.74127216869152, 1)))</f>
@@ -3820,17 +3826,17 @@
       </c>
       <c r="B132" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C132" s="3" t="n">
         <v>46</v>
       </c>
       <c r="D132" s="3" t="n">
-        <v>0.15</v>
+        <v>0.16</v>
       </c>
       <c r="E132" s="3" t="n">
-        <v>1.98</v>
+        <v>1.95</v>
       </c>
       <c r="F132" s="3">
         <f>IF(B132="common", 4, IF(B132="uncommon", 3, IF(B132="rare", 1.74127216869152, 1)))</f>
@@ -3845,17 +3851,17 @@
       </c>
       <c r="B133" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C133" s="3" t="n">
         <v>46</v>
       </c>
       <c r="D133" s="3" t="n">
-        <v>0.13</v>
+        <v>0.12</v>
       </c>
       <c r="E133" s="3" t="n">
-        <v>1.56</v>
+        <v>1.53</v>
       </c>
       <c r="F133" s="3">
         <f>IF(B133="common", 4, IF(B133="uncommon", 3, IF(B133="rare", 1.74127216869152, 1)))</f>
@@ -3870,14 +3876,14 @@
       </c>
       <c r="B134" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C134" s="3" t="n">
         <v>33</v>
       </c>
       <c r="D134" s="3" t="n">
-        <v>0.08</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="E134" s="3" t="n">
         <v>0.19</v>
@@ -3895,17 +3901,17 @@
       </c>
       <c r="B135" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C135" s="3" t="n">
         <v>33</v>
       </c>
       <c r="D135" s="3" t="n">
-        <v>0.06</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="E135" s="3" t="n">
-        <v>0.21</v>
+        <v>0.19</v>
       </c>
       <c r="F135" s="3">
         <f>IF(B135="common", 4, IF(B135="uncommon", 3, IF(B135="rare", 1.74127216869152, 1)))</f>
@@ -3920,14 +3926,14 @@
       </c>
       <c r="B136" s="3" t="inlineStr">
         <is>
-          <t>Double Rare</t>
+          <t>double rare</t>
         </is>
       </c>
       <c r="C136" s="3" t="n">
         <v>90</v>
       </c>
       <c r="D136" s="3" t="n">
-        <v>0.83</v>
+        <v>0.9</v>
       </c>
       <c r="E136" s="3" t="inlineStr"/>
       <c r="F136" s="3">
@@ -3943,14 +3949,14 @@
       </c>
       <c r="B137" s="3" t="inlineStr">
         <is>
-          <t>Ultra Rare</t>
+          <t>ultra rare</t>
         </is>
       </c>
       <c r="C137" s="3" t="n">
         <v>248</v>
       </c>
       <c r="D137" s="3" t="n">
-        <v>7.87</v>
+        <v>6.83</v>
       </c>
       <c r="E137" s="3" t="inlineStr"/>
       <c r="F137" s="3">
@@ -3966,7 +3972,7 @@
       </c>
       <c r="B138" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C138" s="3" t="n">
@@ -3976,7 +3982,7 @@
         <v>0.08</v>
       </c>
       <c r="E138" s="3" t="n">
-        <v>0.19</v>
+        <v>0.16</v>
       </c>
       <c r="F138" s="3">
         <f>IF(B138="common", 4, IF(B138="uncommon", 3, IF(B138="rare", 1.74127216869152, 1)))</f>
@@ -3991,7 +3997,7 @@
       </c>
       <c r="B139" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C139" s="3" t="n">
@@ -4001,7 +4007,7 @@
         <v>0.06</v>
       </c>
       <c r="E139" s="3" t="n">
-        <v>2.36</v>
+        <v>2.33</v>
       </c>
       <c r="F139" s="3">
         <f>IF(B139="common", 4, IF(B139="uncommon", 3, IF(B139="rare", 1.74127216869152, 1)))</f>
@@ -4016,14 +4022,14 @@
       </c>
       <c r="B140" s="3" t="inlineStr">
         <is>
-          <t>Illustration Rare</t>
+          <t>illustration rare</t>
         </is>
       </c>
       <c r="C140" s="3" t="n">
         <v>188</v>
       </c>
       <c r="D140" s="3" t="n">
-        <v>8</v>
+        <v>7.85</v>
       </c>
       <c r="E140" s="3" t="inlineStr"/>
       <c r="F140" s="3">
@@ -4039,14 +4045,14 @@
       </c>
       <c r="B141" s="3" t="inlineStr">
         <is>
-          <t>Rare</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="C141" s="3" t="n">
         <v>21</v>
       </c>
       <c r="D141" s="3" t="n">
-        <v>0.14</v>
+        <v>0.13</v>
       </c>
       <c r="E141" s="3" t="n">
         <v>0.59</v>
@@ -4064,7 +4070,7 @@
       </c>
       <c r="B142" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C142" s="3" t="n">
@@ -4074,7 +4080,7 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="E142" s="3" t="n">
-        <v>1.36</v>
+        <v>1.29</v>
       </c>
       <c r="F142" s="3">
         <f>IF(B142="common", 4, IF(B142="uncommon", 3, IF(B142="rare", 1.74127216869152, 1)))</f>
@@ -4089,7 +4095,7 @@
       </c>
       <c r="B143" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C143" s="3" t="n">
@@ -4114,7 +4120,7 @@
       </c>
       <c r="B144" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C144" s="3" t="n">
@@ -4124,7 +4130,7 @@
         <v>0.1</v>
       </c>
       <c r="E144" s="3" t="n">
-        <v>0.19</v>
+        <v>0.18</v>
       </c>
       <c r="F144" s="3">
         <f>IF(B144="common", 4, IF(B144="uncommon", 3, IF(B144="rare", 1.74127216869152, 1)))</f>
@@ -4139,17 +4145,17 @@
       </c>
       <c r="B145" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C145" s="3" t="n">
         <v>33</v>
       </c>
       <c r="D145" s="3" t="n">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="E145" s="3" t="n">
-        <v>0.21</v>
+        <v>0.18</v>
       </c>
       <c r="F145" s="3">
         <f>IF(B145="common", 4, IF(B145="uncommon", 3, IF(B145="rare", 1.74127216869152, 1)))</f>
@@ -4164,7 +4170,7 @@
       </c>
       <c r="B146" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C146" s="3" t="n">
@@ -4174,7 +4180,7 @@
         <v>0.06</v>
       </c>
       <c r="E146" s="3" t="n">
-        <v>0.2</v>
+        <v>0.19</v>
       </c>
       <c r="F146" s="3">
         <f>IF(B146="common", 4, IF(B146="uncommon", 3, IF(B146="rare", 1.74127216869152, 1)))</f>
@@ -4189,17 +4195,17 @@
       </c>
       <c r="B147" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C147" s="3" t="n">
         <v>46</v>
       </c>
       <c r="D147" s="3" t="n">
-        <v>0.17</v>
+        <v>0.18</v>
       </c>
       <c r="E147" s="3" t="n">
-        <v>2.19</v>
+        <v>2.01</v>
       </c>
       <c r="F147" s="3">
         <f>IF(B147="common", 4, IF(B147="uncommon", 3, IF(B147="rare", 1.74127216869152, 1)))</f>
@@ -4214,7 +4220,7 @@
       </c>
       <c r="B148" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C148" s="3" t="n">
@@ -4224,7 +4230,7 @@
         <v>0.09</v>
       </c>
       <c r="E148" s="3" t="n">
-        <v>0.24</v>
+        <v>0.23</v>
       </c>
       <c r="F148" s="3">
         <f>IF(B148="common", 4, IF(B148="uncommon", 3, IF(B148="rare", 1.74127216869152, 1)))</f>
@@ -4239,7 +4245,7 @@
       </c>
       <c r="B149" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C149" s="3" t="n">
@@ -4249,7 +4255,7 @@
         <v>0.1</v>
       </c>
       <c r="E149" s="3" t="n">
-        <v>0.25</v>
+        <v>0.26</v>
       </c>
       <c r="F149" s="3">
         <f>IF(B149="common", 4, IF(B149="uncommon", 3, IF(B149="rare", 1.74127216869152, 1)))</f>
@@ -4264,14 +4270,14 @@
       </c>
       <c r="B150" s="3" t="inlineStr">
         <is>
-          <t>Illustration Rare</t>
+          <t>illustration rare</t>
         </is>
       </c>
       <c r="C150" s="3" t="n">
         <v>188</v>
       </c>
       <c r="D150" s="3" t="n">
-        <v>28.89</v>
+        <v>28.78</v>
       </c>
       <c r="E150" s="3" t="inlineStr"/>
       <c r="F150" s="3">
@@ -4287,17 +4293,17 @@
       </c>
       <c r="B151" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C151" s="3" t="n">
         <v>33</v>
       </c>
       <c r="D151" s="3" t="n">
-        <v>0.08</v>
+        <v>0.09</v>
       </c>
       <c r="E151" s="3" t="n">
-        <v>1.65</v>
+        <v>1.61</v>
       </c>
       <c r="F151" s="3">
         <f>IF(B151="common", 4, IF(B151="uncommon", 3, IF(B151="rare", 1.74127216869152, 1)))</f>
@@ -4312,7 +4318,7 @@
       </c>
       <c r="B152" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C152" s="3" t="n">
@@ -4322,7 +4328,7 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="E152" s="3" t="n">
-        <v>0.15</v>
+        <v>0.16</v>
       </c>
       <c r="F152" s="3">
         <f>IF(B152="common", 4, IF(B152="uncommon", 3, IF(B152="rare", 1.74127216869152, 1)))</f>
@@ -4337,17 +4343,17 @@
       </c>
       <c r="B153" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C153" s="3" t="n">
         <v>46</v>
       </c>
       <c r="D153" s="3" t="n">
-        <v>0.1</v>
+        <v>0.11</v>
       </c>
       <c r="E153" s="3" t="n">
-        <v>1.14</v>
+        <v>1.24</v>
       </c>
       <c r="F153" s="3">
         <f>IF(B153="common", 4, IF(B153="uncommon", 3, IF(B153="rare", 1.74127216869152, 1)))</f>
@@ -4362,14 +4368,14 @@
       </c>
       <c r="B154" s="3" t="inlineStr">
         <is>
-          <t>Illustration Rare</t>
+          <t>illustration rare</t>
         </is>
       </c>
       <c r="C154" s="3" t="n">
         <v>188</v>
       </c>
       <c r="D154" s="3" t="n">
-        <v>18.96</v>
+        <v>19.64</v>
       </c>
       <c r="E154" s="3" t="inlineStr"/>
       <c r="F154" s="3">
@@ -4385,7 +4391,7 @@
       </c>
       <c r="B155" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C155" s="3" t="n">
@@ -4410,7 +4416,7 @@
       </c>
       <c r="B156" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C156" s="3" t="n">
@@ -4420,7 +4426,7 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="E156" s="3" t="n">
-        <v>0.16</v>
+        <v>0.12</v>
       </c>
       <c r="F156" s="3">
         <f>IF(B156="common", 4, IF(B156="uncommon", 3, IF(B156="rare", 1.74127216869152, 1)))</f>
@@ -4435,14 +4441,14 @@
       </c>
       <c r="B157" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C157" s="3" t="n">
         <v>46</v>
       </c>
       <c r="D157" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06</v>
       </c>
       <c r="E157" s="3" t="n">
         <v>0.17</v>
@@ -4460,7 +4466,7 @@
       </c>
       <c r="B158" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C158" s="3" t="n">
@@ -4470,7 +4476,7 @@
         <v>0.09</v>
       </c>
       <c r="E158" s="3" t="n">
-        <v>0.16</v>
+        <v>0.15</v>
       </c>
       <c r="F158" s="3">
         <f>IF(B158="common", 4, IF(B158="uncommon", 3, IF(B158="rare", 1.74127216869152, 1)))</f>
@@ -4485,17 +4491,17 @@
       </c>
       <c r="B159" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C159" s="3" t="n">
         <v>33</v>
       </c>
       <c r="D159" s="3" t="n">
-        <v>0.13</v>
+        <v>0.14</v>
       </c>
       <c r="E159" s="3" t="n">
-        <v>0.61</v>
+        <v>0.6</v>
       </c>
       <c r="F159" s="3">
         <f>IF(B159="common", 4, IF(B159="uncommon", 3, IF(B159="rare", 1.74127216869152, 1)))</f>
@@ -4510,7 +4516,7 @@
       </c>
       <c r="B160" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C160" s="3" t="n">
@@ -4535,14 +4541,14 @@
       </c>
       <c r="B161" s="3" t="inlineStr">
         <is>
-          <t>Illustration Rare</t>
+          <t>illustration rare</t>
         </is>
       </c>
       <c r="C161" s="3" t="n">
         <v>188</v>
       </c>
       <c r="D161" s="3" t="n">
-        <v>21.1</v>
+        <v>20.45</v>
       </c>
       <c r="E161" s="3" t="inlineStr"/>
       <c r="F161" s="3">
@@ -4558,17 +4564,17 @@
       </c>
       <c r="B162" s="3" t="inlineStr">
         <is>
-          <t>Rare</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="C162" s="3" t="n">
         <v>21</v>
       </c>
       <c r="D162" s="3" t="n">
-        <v>0.14</v>
+        <v>0.11</v>
       </c>
       <c r="E162" s="3" t="n">
-        <v>0.86</v>
+        <v>0.83</v>
       </c>
       <c r="F162" s="3">
         <f>IF(B162="common", 4, IF(B162="uncommon", 3, IF(B162="rare", 1.74127216869152, 1)))</f>
@@ -4583,7 +4589,7 @@
       </c>
       <c r="B163" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C163" s="3" t="n">
@@ -4593,7 +4599,7 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="E163" s="3" t="n">
-        <v>0.18</v>
+        <v>0.16</v>
       </c>
       <c r="F163" s="3">
         <f>IF(B163="common", 4, IF(B163="uncommon", 3, IF(B163="rare", 1.74127216869152, 1)))</f>
@@ -4608,7 +4614,7 @@
       </c>
       <c r="B164" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C164" s="3" t="n">
@@ -4633,7 +4639,7 @@
       </c>
       <c r="B165" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C165" s="3" t="n">
@@ -4643,7 +4649,7 @@
         <v>0.06</v>
       </c>
       <c r="E165" s="3" t="n">
-        <v>0.19</v>
+        <v>0.17</v>
       </c>
       <c r="F165" s="3">
         <f>IF(B165="common", 4, IF(B165="uncommon", 3, IF(B165="rare", 1.74127216869152, 1)))</f>
@@ -4658,17 +4664,17 @@
       </c>
       <c r="B166" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C166" s="3" t="n">
         <v>33</v>
       </c>
       <c r="D166" s="3" t="n">
-        <v>0.09</v>
+        <v>0.08</v>
       </c>
       <c r="E166" s="3" t="n">
-        <v>0.14</v>
+        <v>0.16</v>
       </c>
       <c r="F166" s="3">
         <f>IF(B166="common", 4, IF(B166="uncommon", 3, IF(B166="rare", 1.74127216869152, 1)))</f>
@@ -4683,7 +4689,7 @@
       </c>
       <c r="B167" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C167" s="3" t="n">
@@ -4693,7 +4699,7 @@
         <v>0.06</v>
       </c>
       <c r="E167" s="3" t="n">
-        <v>0.15</v>
+        <v>0.14</v>
       </c>
       <c r="F167" s="3">
         <f>IF(B167="common", 4, IF(B167="uncommon", 3, IF(B167="rare", 1.74127216869152, 1)))</f>
@@ -4708,17 +4714,17 @@
       </c>
       <c r="B168" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C168" s="3" t="n">
         <v>33</v>
       </c>
       <c r="D168" s="3" t="n">
-        <v>0.1</v>
+        <v>0.12</v>
       </c>
       <c r="E168" s="3" t="n">
-        <v>1.08</v>
+        <v>1.05</v>
       </c>
       <c r="F168" s="3">
         <f>IF(B168="common", 4, IF(B168="uncommon", 3, IF(B168="rare", 1.74127216869152, 1)))</f>
@@ -4733,17 +4739,17 @@
       </c>
       <c r="B169" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C169" s="3" t="n">
         <v>46</v>
       </c>
       <c r="D169" s="3" t="n">
-        <v>0.08</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="E169" s="3" t="n">
-        <v>0.17</v>
+        <v>0.18</v>
       </c>
       <c r="F169" s="3">
         <f>IF(B169="common", 4, IF(B169="uncommon", 3, IF(B169="rare", 1.74127216869152, 1)))</f>
@@ -4758,7 +4764,7 @@
       </c>
       <c r="B170" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C170" s="3" t="n">
@@ -4768,7 +4774,7 @@
         <v>0.08</v>
       </c>
       <c r="E170" s="3" t="n">
-        <v>0.17</v>
+        <v>0.18</v>
       </c>
       <c r="F170" s="3">
         <f>IF(B170="common", 4, IF(B170="uncommon", 3, IF(B170="rare", 1.74127216869152, 1)))</f>
@@ -4783,7 +4789,7 @@
       </c>
       <c r="B171" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C171" s="3" t="n">
@@ -4793,7 +4799,7 @@
         <v>0.11</v>
       </c>
       <c r="E171" s="3" t="n">
-        <v>2.4</v>
+        <v>2.25</v>
       </c>
       <c r="F171" s="3">
         <f>IF(B171="common", 4, IF(B171="uncommon", 3, IF(B171="rare", 1.74127216869152, 1)))</f>
@@ -4808,7 +4814,7 @@
       </c>
       <c r="B172" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C172" s="3" t="n">
@@ -4818,7 +4824,7 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="E172" s="3" t="n">
-        <v>0.14</v>
+        <v>0.15</v>
       </c>
       <c r="F172" s="3">
         <f>IF(B172="common", 4, IF(B172="uncommon", 3, IF(B172="rare", 1.74127216869152, 1)))</f>
@@ -4833,7 +4839,7 @@
       </c>
       <c r="B173" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C173" s="3" t="n">
@@ -4858,7 +4864,7 @@
       </c>
       <c r="B174" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C174" s="3" t="n">
@@ -4883,7 +4889,7 @@
       </c>
       <c r="B175" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C175" s="3" t="n">
@@ -4893,7 +4899,7 @@
         <v>0.06</v>
       </c>
       <c r="E175" s="3" t="n">
-        <v>0.15</v>
+        <v>0.14</v>
       </c>
       <c r="F175" s="3">
         <f>IF(B175="common", 4, IF(B175="uncommon", 3, IF(B175="rare", 1.74127216869152, 1)))</f>
@@ -4908,7 +4914,7 @@
       </c>
       <c r="B176" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C176" s="3" t="n">
@@ -4933,7 +4939,7 @@
       </c>
       <c r="B177" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C177" s="3" t="n">
@@ -4943,7 +4949,7 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="E177" s="3" t="n">
-        <v>0.22</v>
+        <v>0.19</v>
       </c>
       <c r="F177" s="3">
         <f>IF(B177="common", 4, IF(B177="uncommon", 3, IF(B177="rare", 1.74127216869152, 1)))</f>
@@ -4958,7 +4964,7 @@
       </c>
       <c r="B178" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C178" s="3" t="n">
@@ -4968,7 +4974,7 @@
         <v>0.16</v>
       </c>
       <c r="E178" s="3" t="n">
-        <v>1.27</v>
+        <v>1.31</v>
       </c>
       <c r="F178" s="3">
         <f>IF(B178="common", 4, IF(B178="uncommon", 3, IF(B178="rare", 1.74127216869152, 1)))</f>
@@ -4983,7 +4989,7 @@
       </c>
       <c r="B179" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C179" s="3" t="n">
@@ -4993,7 +4999,7 @@
         <v>0.06</v>
       </c>
       <c r="E179" s="3" t="n">
-        <v>0.9</v>
+        <v>0.85</v>
       </c>
       <c r="F179" s="3">
         <f>IF(B179="common", 4, IF(B179="uncommon", 3, IF(B179="rare", 1.74127216869152, 1)))</f>
@@ -5008,7 +5014,7 @@
       </c>
       <c r="B180" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C180" s="3" t="n">
@@ -5018,7 +5024,7 @@
         <v>0.11</v>
       </c>
       <c r="E180" s="3" t="n">
-        <v>0.23</v>
+        <v>0.2</v>
       </c>
       <c r="F180" s="3">
         <f>IF(B180="common", 4, IF(B180="uncommon", 3, IF(B180="rare", 1.74127216869152, 1)))</f>
@@ -5033,14 +5039,14 @@
       </c>
       <c r="B181" s="3" t="inlineStr">
         <is>
-          <t>Illustration Rare</t>
+          <t>illustration rare</t>
         </is>
       </c>
       <c r="C181" s="3" t="n">
         <v>188</v>
       </c>
       <c r="D181" s="3" t="n">
-        <v>46.05</v>
+        <v>45.09</v>
       </c>
       <c r="E181" s="3" t="inlineStr"/>
       <c r="F181" s="3">
@@ -5056,17 +5062,17 @@
       </c>
       <c r="B182" s="3" t="inlineStr">
         <is>
-          <t>Rare</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="C182" s="3" t="n">
         <v>21</v>
       </c>
       <c r="D182" s="3" t="n">
-        <v>0.16</v>
+        <v>0.15</v>
       </c>
       <c r="E182" s="3" t="n">
-        <v>0.64</v>
+        <v>0.63</v>
       </c>
       <c r="F182" s="3">
         <f>IF(B182="common", 4, IF(B182="uncommon", 3, IF(B182="rare", 1.74127216869152, 1)))</f>
@@ -5081,7 +5087,7 @@
       </c>
       <c r="B183" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C183" s="3" t="n">
@@ -5106,14 +5112,14 @@
       </c>
       <c r="B184" s="3" t="inlineStr">
         <is>
-          <t>Hyper Rare</t>
+          <t>hyper rare</t>
         </is>
       </c>
       <c r="C184" s="3" t="n">
         <v>154</v>
       </c>
       <c r="D184" s="3" t="n">
-        <v>2.56</v>
+        <v>2.93</v>
       </c>
       <c r="E184" s="3" t="inlineStr"/>
       <c r="F184" s="3">
@@ -5129,17 +5135,17 @@
       </c>
       <c r="B185" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C185" s="3" t="n">
         <v>46</v>
       </c>
       <c r="D185" s="3" t="n">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="E185" s="3" t="n">
-        <v>0.15</v>
+        <v>0.17</v>
       </c>
       <c r="F185" s="3">
         <f>IF(B185="common", 4, IF(B185="uncommon", 3, IF(B185="rare", 1.74127216869152, 1)))</f>
@@ -5154,14 +5160,14 @@
       </c>
       <c r="B186" s="3" t="inlineStr">
         <is>
-          <t>Illustration Rare</t>
+          <t>illustration rare</t>
         </is>
       </c>
       <c r="C186" s="3" t="n">
         <v>188</v>
       </c>
       <c r="D186" s="3" t="n">
-        <v>7.68</v>
+        <v>7.56</v>
       </c>
       <c r="E186" s="3" t="inlineStr"/>
       <c r="F186" s="3">
@@ -5177,17 +5183,17 @@
       </c>
       <c r="B187" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C187" s="3" t="n">
         <v>33</v>
       </c>
       <c r="D187" s="3" t="n">
-        <v>0.08</v>
+        <v>0.1</v>
       </c>
       <c r="E187" s="3" t="n">
-        <v>0.77</v>
+        <v>0.75</v>
       </c>
       <c r="F187" s="3">
         <f>IF(B187="common", 4, IF(B187="uncommon", 3, IF(B187="rare", 1.74127216869152, 1)))</f>
@@ -5202,7 +5208,7 @@
       </c>
       <c r="B188" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C188" s="3" t="n">
@@ -5212,7 +5218,7 @@
         <v>0.06</v>
       </c>
       <c r="E188" s="3" t="n">
-        <v>0.16</v>
+        <v>0.17</v>
       </c>
       <c r="F188" s="3">
         <f>IF(B188="common", 4, IF(B188="uncommon", 3, IF(B188="rare", 1.74127216869152, 1)))</f>
@@ -5227,7 +5233,7 @@
       </c>
       <c r="B189" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C189" s="3" t="n">
@@ -5252,17 +5258,17 @@
       </c>
       <c r="B190" s="3" t="inlineStr">
         <is>
-          <t>Rare</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="C190" s="3" t="n">
         <v>21</v>
       </c>
       <c r="D190" s="3" t="n">
-        <v>0.28</v>
+        <v>0.25</v>
       </c>
       <c r="E190" s="3" t="n">
-        <v>1.28</v>
+        <v>1.25</v>
       </c>
       <c r="F190" s="3">
         <f>IF(B190="common", 4, IF(B190="uncommon", 3, IF(B190="rare", 1.74127216869152, 1)))</f>
@@ -5277,7 +5283,7 @@
       </c>
       <c r="B191" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C191" s="3" t="n">
@@ -5287,7 +5293,7 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="E191" s="3" t="n">
-        <v>0.18</v>
+        <v>0.19</v>
       </c>
       <c r="F191" s="3">
         <f>IF(B191="common", 4, IF(B191="uncommon", 3, IF(B191="rare", 1.74127216869152, 1)))</f>
@@ -5302,7 +5308,7 @@
       </c>
       <c r="B192" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C192" s="3" t="n">
@@ -5327,14 +5333,14 @@
       </c>
       <c r="B193" s="3" t="inlineStr">
         <is>
-          <t>Double Rare</t>
+          <t>double rare</t>
         </is>
       </c>
       <c r="C193" s="3" t="n">
         <v>90</v>
       </c>
       <c r="D193" s="3" t="n">
-        <v>0.77</v>
+        <v>0.95</v>
       </c>
       <c r="E193" s="3" t="inlineStr"/>
       <c r="F193" s="3">
@@ -5350,14 +5356,14 @@
       </c>
       <c r="B194" s="3" t="inlineStr">
         <is>
-          <t>Ultra Rare</t>
+          <t>ultra rare</t>
         </is>
       </c>
       <c r="C194" s="3" t="n">
         <v>248</v>
       </c>
       <c r="D194" s="3" t="n">
-        <v>11.82</v>
+        <v>11.58</v>
       </c>
       <c r="E194" s="3" t="inlineStr"/>
       <c r="F194" s="3">
@@ -5373,14 +5379,14 @@
       </c>
       <c r="B195" s="3" t="inlineStr">
         <is>
-          <t>Special Illustration Rare</t>
+          <t>special illustration rare</t>
         </is>
       </c>
       <c r="C195" s="3" t="n">
         <v>225</v>
       </c>
       <c r="D195" s="3" t="n">
-        <v>68.69</v>
+        <v>67.88</v>
       </c>
       <c r="E195" s="3" t="inlineStr"/>
       <c r="F195" s="3">
@@ -5396,7 +5402,7 @@
       </c>
       <c r="B196" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C196" s="3" t="n">
@@ -5406,7 +5412,7 @@
         <v>0.05</v>
       </c>
       <c r="E196" s="3" t="n">
-        <v>0.17</v>
+        <v>0.16</v>
       </c>
       <c r="F196" s="3">
         <f>IF(B196="common", 4, IF(B196="uncommon", 3, IF(B196="rare", 1.74127216869152, 1)))</f>
@@ -5421,17 +5427,17 @@
       </c>
       <c r="B197" s="3" t="inlineStr">
         <is>
-          <t>Rare</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="C197" s="3" t="n">
         <v>21</v>
       </c>
       <c r="D197" s="3" t="n">
-        <v>0.2</v>
+        <v>0.18</v>
       </c>
       <c r="E197" s="3" t="n">
-        <v>0.93</v>
+        <v>0.91</v>
       </c>
       <c r="F197" s="3">
         <f>IF(B197="common", 4, IF(B197="uncommon", 3, IF(B197="rare", 1.74127216869152, 1)))</f>
@@ -5446,7 +5452,7 @@
       </c>
       <c r="B198" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C198" s="3" t="n">
@@ -5456,7 +5462,7 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="E198" s="3" t="n">
-        <v>0.17</v>
+        <v>0.16</v>
       </c>
       <c r="F198" s="3">
         <f>IF(B198="common", 4, IF(B198="uncommon", 3, IF(B198="rare", 1.74127216869152, 1)))</f>
@@ -5471,7 +5477,7 @@
       </c>
       <c r="B199" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C199" s="3" t="n">
@@ -5481,7 +5487,7 @@
         <v>0.09</v>
       </c>
       <c r="E199" s="3" t="n">
-        <v>0.21</v>
+        <v>0.18</v>
       </c>
       <c r="F199" s="3">
         <f>IF(B199="common", 4, IF(B199="uncommon", 3, IF(B199="rare", 1.74127216869152, 1)))</f>
@@ -5496,17 +5502,17 @@
       </c>
       <c r="B200" s="3" t="inlineStr">
         <is>
-          <t>Uncommon</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="C200" s="3" t="n">
         <v>33</v>
       </c>
       <c r="D200" s="3" t="n">
-        <v>0.12</v>
+        <v>0.09</v>
       </c>
       <c r="E200" s="3" t="n">
-        <v>0.22</v>
+        <v>0.23</v>
       </c>
       <c r="F200" s="3">
         <f>IF(B200="common", 4, IF(B200="uncommon", 3, IF(B200="rare", 1.74127216869152, 1)))</f>
@@ -5521,14 +5527,14 @@
       </c>
       <c r="B201" s="3" t="inlineStr">
         <is>
-          <t>Illustration Rare</t>
+          <t>illustration rare</t>
         </is>
       </c>
       <c r="C201" s="3" t="n">
         <v>188</v>
       </c>
       <c r="D201" s="3" t="n">
-        <v>30.34</v>
+        <v>29.96</v>
       </c>
       <c r="E201" s="3" t="inlineStr"/>
       <c r="F201" s="3">
@@ -5544,7 +5550,7 @@
       </c>
       <c r="B202" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C202" s="3" t="n">
@@ -5554,7 +5560,7 @@
         <v>0.06</v>
       </c>
       <c r="E202" s="3" t="n">
-        <v>0.11</v>
+        <v>0.13</v>
       </c>
       <c r="F202" s="3">
         <f>IF(B202="common", 4, IF(B202="uncommon", 3, IF(B202="rare", 1.74127216869152, 1)))</f>
@@ -5569,17 +5575,17 @@
       </c>
       <c r="B203" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C203" s="3" t="n">
         <v>46</v>
       </c>
       <c r="D203" s="3" t="n">
-        <v>0.1</v>
+        <v>0.11</v>
       </c>
       <c r="E203" s="3" t="n">
-        <v>1.51</v>
+        <v>1.54</v>
       </c>
       <c r="F203" s="3">
         <f>IF(B203="common", 4, IF(B203="uncommon", 3, IF(B203="rare", 1.74127216869152, 1)))</f>
@@ -5594,17 +5600,17 @@
       </c>
       <c r="B204" s="3" t="inlineStr">
         <is>
-          <t>Rare</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="C204" s="3" t="n">
         <v>21</v>
       </c>
       <c r="D204" s="3" t="n">
-        <v>0.15</v>
+        <v>0.17</v>
       </c>
       <c r="E204" s="3" t="n">
-        <v>0.58</v>
+        <v>0.57</v>
       </c>
       <c r="F204" s="3">
         <f>IF(B204="common", 4, IF(B204="uncommon", 3, IF(B204="rare", 1.74127216869152, 1)))</f>
@@ -5619,14 +5625,14 @@
       </c>
       <c r="B205" s="3" t="inlineStr">
         <is>
-          <t>Double Rare</t>
+          <t>double rare</t>
         </is>
       </c>
       <c r="C205" s="3" t="n">
         <v>90</v>
       </c>
       <c r="D205" s="3" t="n">
-        <v>0.77</v>
+        <v>0.84</v>
       </c>
       <c r="E205" s="3" t="inlineStr"/>
       <c r="F205" s="3">
@@ -5642,14 +5648,14 @@
       </c>
       <c r="B206" s="3" t="inlineStr">
         <is>
-          <t>Ultra Rare</t>
+          <t>ultra rare</t>
         </is>
       </c>
       <c r="C206" s="3" t="n">
         <v>248</v>
       </c>
       <c r="D206" s="3" t="n">
-        <v>7.9</v>
+        <v>7.25</v>
       </c>
       <c r="E206" s="3" t="inlineStr"/>
       <c r="F206" s="3">
@@ -5665,14 +5671,14 @@
       </c>
       <c r="B207" s="3" t="inlineStr">
         <is>
-          <t>Double Rare</t>
+          <t>double rare</t>
         </is>
       </c>
       <c r="C207" s="3" t="n">
         <v>90</v>
       </c>
       <c r="D207" s="3" t="n">
-        <v>0.71</v>
+        <v>0.77</v>
       </c>
       <c r="E207" s="3" t="inlineStr"/>
       <c r="F207" s="3">
@@ -5688,14 +5694,14 @@
       </c>
       <c r="B208" s="3" t="inlineStr">
         <is>
-          <t>Ultra Rare</t>
+          <t>ultra rare</t>
         </is>
       </c>
       <c r="C208" s="3" t="n">
         <v>248</v>
       </c>
       <c r="D208" s="3" t="n">
-        <v>8.06</v>
+        <v>8.050000000000001</v>
       </c>
       <c r="E208" s="3" t="inlineStr"/>
       <c r="F208" s="3">
@@ -5711,14 +5717,14 @@
       </c>
       <c r="B209" s="3" t="inlineStr">
         <is>
-          <t>Special Illustration Rare</t>
+          <t>special illustration rare</t>
         </is>
       </c>
       <c r="C209" s="3" t="n">
         <v>225</v>
       </c>
       <c r="D209" s="3" t="n">
-        <v>55.36</v>
+        <v>55.64</v>
       </c>
       <c r="E209" s="3" t="inlineStr"/>
       <c r="F209" s="3">
@@ -5734,7 +5740,7 @@
       </c>
       <c r="B210" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C210" s="3" t="n">
@@ -5759,7 +5765,7 @@
       </c>
       <c r="B211" s="3" t="inlineStr">
         <is>
-          <t>Rare</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="C211" s="3" t="n">
@@ -5784,7 +5790,7 @@
       </c>
       <c r="B212" s="3" t="inlineStr">
         <is>
-          <t>Double Rare</t>
+          <t>double rare</t>
         </is>
       </c>
       <c r="C212" s="3" t="n">
@@ -5807,7 +5813,7 @@
       </c>
       <c r="B213" s="3" t="inlineStr">
         <is>
-          <t>Ultra Rare</t>
+          <t>ultra rare</t>
         </is>
       </c>
       <c r="C213" s="3" t="n">
@@ -5830,7 +5836,7 @@
       </c>
       <c r="B214" s="3" t="inlineStr">
         <is>
-          <t>Double Rare</t>
+          <t>double rare</t>
         </is>
       </c>
       <c r="C214" s="3" t="n">
@@ -5853,7 +5859,7 @@
       </c>
       <c r="B215" s="3" t="inlineStr">
         <is>
-          <t>Ultra Rare</t>
+          <t>ultra rare</t>
         </is>
       </c>
       <c r="C215" s="3" t="n">
@@ -5876,7 +5882,7 @@
       </c>
       <c r="B216" s="3" t="inlineStr">
         <is>
-          <t>Special Illustration Rare</t>
+          <t>special illustration rare</t>
         </is>
       </c>
       <c r="C216" s="3" t="n">
@@ -5899,7 +5905,7 @@
       </c>
       <c r="B217" s="3" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>common</t>
         </is>
       </c>
       <c r="C217" s="3" t="n">
@@ -12479,225 +12485,225 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="B1" s="9" t="inlineStr">
+      <c r="B1" s="10" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>ev_common_total</t>
         </is>
       </c>
-      <c r="B2" s="11" t="n">
-        <v>0.1123913043478261</v>
+      <c r="B2" s="12" t="n">
+        <v>0.451304347826087</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="inlineStr">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>ev_uncommon_total</t>
         </is>
       </c>
-      <c r="B3" s="11" t="n">
-        <v>0.1696969696969697</v>
+      <c r="B3" s="12" t="n">
+        <v>0.5090909090909091</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="A4" s="11" t="inlineStr">
         <is>
           <t>ev_rare_total</t>
         </is>
       </c>
-      <c r="B4" s="11" t="n">
-        <v>0.2695238095238095</v>
+      <c r="B4" s="12" t="n">
+        <v>0.213703314659197</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>ev_reverse_total</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="n">
+        <v>5.313106295878034</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>ev_ace_spec_total</t>
+        </is>
+      </c>
+      <c r="B6" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>ev_pokeball_total</t>
+        </is>
+      </c>
+      <c r="B7" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>ev_master_ball_total</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>ev_IR_total</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="n">
+        <v>1.96968085106383</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>ev_SIR_total</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="n">
+        <v>2.372933333333333</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="11" t="inlineStr">
         <is>
           <t>ev_double_rare_total</t>
         </is>
       </c>
-      <c r="B5" s="11" t="n">
-        <v>0.3478888888888889</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="10" t="inlineStr">
-        <is>
-          <t>ev_pokeball_total</t>
-        </is>
-      </c>
-      <c r="B6" s="11" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="10" t="inlineStr">
-        <is>
-          <t>ev_master_ball_total</t>
-        </is>
-      </c>
-      <c r="B7" s="11" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="10" t="inlineStr">
+      <c r="B11" s="12" t="n">
+        <v>0.3439999999999999</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="inlineStr">
         <is>
           <t>ev_hyper_rare_total</t>
         </is>
       </c>
-      <c r="B8" s="11" t="n">
-        <v>0.1349350649350649</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="B12" s="12" t="n">
+        <v>0.1366233766233766</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="inlineStr">
         <is>
           <t>ev_ultra_rare_total</t>
         </is>
       </c>
-      <c r="B9" s="11" t="n">
-        <v>0.6597580645161291</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="10" t="inlineStr">
-        <is>
-          <t>ev_SIR_total</t>
-        </is>
-      </c>
-      <c r="B10" s="11" t="n">
-        <v>2.366622222222222</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="10" t="inlineStr">
-        <is>
-          <t>ev_IR_total</t>
-        </is>
-      </c>
-      <c r="B11" s="11" t="n">
-        <v>1.987606382978723</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="10" t="inlineStr">
-        <is>
-          <t>ev_reverse_total</t>
-        </is>
-      </c>
-      <c r="B12" s="11" t="n">
-        <v>2.824572746094485</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="10" t="inlineStr">
+      <c r="B13" s="12" t="n">
+        <v>0.6449596774193548</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="11" t="inlineStr">
         <is>
           <t>reverse_multiplier</t>
         </is>
       </c>
-      <c r="B13" s="11" t="n">
-        <v>1.879338061465721</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="10" t="inlineStr">
+      <c r="B14" s="11" t="n">
+        <v>1.885416666666667</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="11" t="inlineStr">
         <is>
           <t>rare_multiplier</t>
         </is>
       </c>
-      <c r="B14" s="10" t="n">
-        <v>1.741272168691524</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="10" t="inlineStr">
-        <is>
-          <t>ev_total_for_hits</t>
-        </is>
-      </c>
       <c r="B15" s="11" t="n">
-        <v>5.14892173465214</v>
+        <v>0.7928921568627451</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="10" t="inlineStr">
+      <c r="A16" s="11" t="inlineStr">
         <is>
           <t>ev_hits_total</t>
         </is>
       </c>
-      <c r="B16" s="11" t="n">
-        <v>5.496810623541029</v>
+      <c r="B16" s="12" t="n">
+        <v>5.468197238439894</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="10" t="inlineStr">
+      <c r="A17" s="11" t="inlineStr">
         <is>
           <t>total_ev</t>
         </is>
       </c>
-      <c r="B17" s="11" t="n">
-        <v>11.07690299510566</v>
+      <c r="B17" s="12" t="n">
+        <v>11.95540210589412</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="10" t="inlineStr">
+      <c r="A18" s="11" t="inlineStr">
         <is>
           <t>net_value</t>
         </is>
       </c>
-      <c r="B18" s="11" t="n">
-        <v>0.1869029951056582</v>
+      <c r="B18" s="12" t="n">
+        <v>1.065402105894121</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="10" t="inlineStr">
+      <c r="A19" s="11" t="inlineStr">
         <is>
           <t>roi</t>
         </is>
       </c>
-      <c r="B19" s="12" t="n">
-        <v>0.01716280946792081</v>
+      <c r="B19" s="13" t="n">
+        <v>1.097833067575218</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="10" t="inlineStr">
+      <c r="A20" s="11" t="inlineStr">
         <is>
           <t>roi_percent</t>
         </is>
       </c>
-      <c r="B20" s="12" t="n">
-        <v>0.7162809467920814</v>
+      <c r="B20" s="14" t="n">
+        <v>0.09783306757521772</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="10" t="inlineStr">
+      <c r="A21" s="11" t="inlineStr">
         <is>
           <t>no_hit_probability_percentage</t>
         </is>
       </c>
-      <c r="B21" s="12" t="n">
-        <v>68.32877110235633</v>
+      <c r="B21" s="14" t="n">
+        <v>0.6832877110235632</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="10" t="inlineStr">
+      <c r="A22" s="11" t="inlineStr">
         <is>
           <t>hit_probability_percentage</t>
         </is>
       </c>
-      <c r="B22" s="12" t="n">
-        <v>31.67122889764367</v>
+      <c r="B22" s="14" t="n">
+        <v>0.3167122889764367</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
major refractoring for scaling
</commit_message>
<xml_diff>
--- a/Expected Value and Cost Ratio Calculator Pokemon/excelDocs/scarletAndViolet151/pokemon_data.xlsx
+++ b/Expected Value and Cost Ratio Calculator Pokemon/excelDocs/scarletAndViolet151/pokemon_data.xlsx
@@ -662,7 +662,7 @@
         <v>0.06</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>0.2</v>
+        <v>0.18</v>
       </c>
       <c r="F2" s="3">
         <f>IF(B2:B210="common", 4, IF(B2:B210="uncommon", 3, IF(B2:B210="rare", 0.792892156862745, 1)))</f>
@@ -677,20 +677,20 @@
         <v/>
       </c>
       <c r="I2" s="3" t="n">
-        <v>9.73</v>
+        <v>9.890000000000001</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>65.38</v>
+        <v>65.62</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>232.49</v>
+        <v>232.98</v>
       </c>
       <c r="L2" s="3" t="n">
-        <v>5.93</v>
+        <v>6.19</v>
       </c>
       <c r="M2" s="3" t="n"/>
       <c r="N2" s="3" t="n">
-        <v>372.1</v>
+        <v>372.92</v>
       </c>
       <c r="R2" s="3" t="n"/>
       <c r="S2" s="3" t="n"/>
@@ -728,10 +728,10 @@
         <v>21</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>0.22</v>
+        <v>0.21</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>0.64</v>
+        <v>0.59</v>
       </c>
       <c r="F3" s="3">
         <f>IF(B3:B211="common", 4, IF(B3:B211="uncommon", 3, IF(B3:B211="rare", 0.792892156862745, 1)))</f>
@@ -838,7 +838,7 @@
         <v>248</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>7.41</v>
+        <v>7.01</v>
       </c>
       <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="3">
@@ -892,7 +892,7 @@
         <v>225</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>36.43</v>
+        <v>36.5</v>
       </c>
       <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="3">
@@ -946,7 +946,7 @@
         <v>46</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>0.11</v>
+        <v>0.1</v>
       </c>
       <c r="E7" s="3" t="n">
         <v>0.58</v>
@@ -1002,10 +1002,10 @@
         <v>46</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>0.11</v>
+        <v>0.1</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>0.98</v>
+        <v>0.97</v>
       </c>
       <c r="F8" s="3">
         <f>IF(B8:B216="common", 4, IF(B8:B216="uncommon", 3, IF(B8:B216="rare", 0.792892156862745, 1)))</f>
@@ -1058,10 +1058,10 @@
         <v>46</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>0.08</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>0.62</v>
+        <v>0.59</v>
       </c>
       <c r="F9" s="3">
         <f>IF(B9:B217="common", 4, IF(B9:B217="uncommon", 3, IF(B9:B217="rare", 0.792892156862745, 1)))</f>
@@ -1114,7 +1114,7 @@
         <v>90</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.85</v>
       </c>
       <c r="E10" s="3" t="inlineStr"/>
       <c r="F10" s="3">
@@ -1168,7 +1168,7 @@
         <v>248</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>5.38</v>
+        <v>4.77</v>
       </c>
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="3">
@@ -1222,7 +1222,7 @@
         <v>0.06</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>0.16</v>
+        <v>0.14</v>
       </c>
       <c r="F12" s="3">
         <f>IF(B12:B220="common", 4, IF(B12:B220="uncommon", 3, IF(B12:B220="rare", 0.792892156862745, 1)))</f>
@@ -1272,10 +1272,10 @@
         <v>21</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>0.2</v>
+        <v>0.18</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>1.1</v>
+        <v>0.96</v>
       </c>
       <c r="F13" s="3">
         <f>IF(B13:B221="common", 4, IF(B13:B221="uncommon", 3, IF(B13:B221="rare", 0.792892156862745, 1)))</f>
@@ -1325,7 +1325,7 @@
         <v>154</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>4.61</v>
+        <v>4.45</v>
       </c>
       <c r="E14" s="3" t="inlineStr"/>
       <c r="F14" s="3">
@@ -1376,10 +1376,10 @@
         <v>21</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>0.15</v>
+        <v>0.14</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>0.76</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="F15" s="3">
         <f>IF(B15:B223="common", 4, IF(B15:B223="uncommon", 3, IF(B15:B223="rare", 0.792892156862745, 1)))</f>
@@ -1429,7 +1429,7 @@
         <v>46</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06</v>
       </c>
       <c r="E16" s="3" t="n">
         <v>0.11</v>
@@ -1485,7 +1485,7 @@
         <v>0.09</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>0.83</v>
+        <v>0.79</v>
       </c>
       <c r="F17" s="3">
         <f>IF(B17:B225="common", 4, IF(B17:B225="uncommon", 3, IF(B17:B225="rare", 0.792892156862745, 1)))</f>
@@ -1538,7 +1538,7 @@
         <v>0.11</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>0.47</v>
+        <v>0.38</v>
       </c>
       <c r="F18" s="3">
         <f>IF(B18:B226="common", 4, IF(B18:B226="uncommon", 3, IF(B18:B226="rare", 0.792892156862745, 1)))</f>
@@ -1588,7 +1588,7 @@
         <v>248</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>3.06</v>
+        <v>2.85</v>
       </c>
       <c r="E19" s="3" t="inlineStr"/>
       <c r="F19" s="3">
@@ -1639,7 +1639,7 @@
         <v>90</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.85</v>
       </c>
       <c r="E20" s="3" t="inlineStr"/>
       <c r="F20" s="3">
@@ -1690,7 +1690,7 @@
         <v>248</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>13.25</v>
+        <v>13.09</v>
       </c>
       <c r="E21" s="3" t="inlineStr"/>
       <c r="F21" s="3">
@@ -1741,7 +1741,7 @@
         <v>225</v>
       </c>
       <c r="D22" s="3" t="n">
-        <v>65.98</v>
+        <v>65.44</v>
       </c>
       <c r="E22" s="3" t="inlineStr"/>
       <c r="F22" s="3">
@@ -1792,10 +1792,10 @@
         <v>46</v>
       </c>
       <c r="D23" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.09</v>
       </c>
       <c r="E23" s="3" t="n">
-        <v>0.19</v>
+        <v>0.16</v>
       </c>
       <c r="F23" s="3">
         <f>IF(B23:B231="common", 4, IF(B23:B231="uncommon", 3, IF(B23:B231="rare", 0.792892156862745, 1)))</f>
@@ -1845,7 +1845,7 @@
         <v>188</v>
       </c>
       <c r="D24" s="3" t="n">
-        <v>33.97</v>
+        <v>34.54</v>
       </c>
       <c r="E24" s="3" t="inlineStr"/>
       <c r="F24" s="3">
@@ -1896,7 +1896,7 @@
         <v>33</v>
       </c>
       <c r="D25" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06</v>
       </c>
       <c r="E25" s="3" t="n">
         <v>0.14</v>
@@ -1949,10 +1949,10 @@
         <v>46</v>
       </c>
       <c r="D26" s="3" t="n">
-        <v>0.04</v>
+        <v>0.05</v>
       </c>
       <c r="E26" s="3" t="n">
-        <v>0.15</v>
+        <v>0.19</v>
       </c>
       <c r="F26" s="3">
         <f>IF(B26:B234="common", 4, IF(B26:B234="uncommon", 3, IF(B26:B234="rare", 0.792892156862745, 1)))</f>
@@ -2002,7 +2002,7 @@
         <v>188</v>
       </c>
       <c r="D27" s="3" t="n">
-        <v>7.77</v>
+        <v>7.19</v>
       </c>
       <c r="E27" s="3" t="inlineStr"/>
       <c r="F27" s="3">
@@ -2056,7 +2056,7 @@
         <v>0.18</v>
       </c>
       <c r="E28" s="3" t="n">
-        <v>0.91</v>
+        <v>0.87</v>
       </c>
       <c r="F28" s="3">
         <f>IF(B28:B236="common", 4, IF(B28:B236="uncommon", 3, IF(B28:B236="rare", 0.792892156862745, 1)))</f>
@@ -2106,7 +2106,7 @@
         <v>90</v>
       </c>
       <c r="D29" s="3" t="n">
-        <v>3.86</v>
+        <v>4.25</v>
       </c>
       <c r="E29" s="3" t="inlineStr"/>
       <c r="F29" s="3">
@@ -2157,7 +2157,7 @@
         <v>248</v>
       </c>
       <c r="D30" s="3" t="n">
-        <v>25.18</v>
+        <v>26.9</v>
       </c>
       <c r="E30" s="3" t="inlineStr"/>
       <c r="F30" s="3">
@@ -2208,7 +2208,7 @@
         <v>225</v>
       </c>
       <c r="D31" s="3" t="n">
-        <v>206.26</v>
+        <v>198.4</v>
       </c>
       <c r="E31" s="3" t="inlineStr"/>
       <c r="F31" s="3">
@@ -2259,10 +2259,10 @@
         <v>46</v>
       </c>
       <c r="D32" s="3" t="n">
-        <v>0.1</v>
+        <v>0.09</v>
       </c>
       <c r="E32" s="3" t="n">
-        <v>0.25</v>
+        <v>0.24</v>
       </c>
       <c r="F32" s="3">
         <f>IF(B32:B240="common", 4, IF(B32:B240="uncommon", 3, IF(B32:B240="rare", 0.792892156862745, 1)))</f>
@@ -2312,7 +2312,7 @@
         <v>188</v>
       </c>
       <c r="D33" s="3" t="n">
-        <v>42.53</v>
+        <v>42.66</v>
       </c>
       <c r="E33" s="3" t="inlineStr"/>
       <c r="F33" s="3">
@@ -2363,10 +2363,10 @@
         <v>33</v>
       </c>
       <c r="D34" s="3" t="n">
-        <v>0.1</v>
+        <v>0.08</v>
       </c>
       <c r="E34" s="3" t="n">
-        <v>0.21</v>
+        <v>0.2</v>
       </c>
       <c r="F34" s="3">
         <f>IF(B34:B242="common", 4, IF(B34:B242="uncommon", 3, IF(B34:B242="rare", 0.792892156862745, 1)))</f>
@@ -2416,7 +2416,7 @@
         <v>188</v>
       </c>
       <c r="D35" s="3" t="n">
-        <v>32.92</v>
+        <v>32.18</v>
       </c>
       <c r="E35" s="3" t="inlineStr"/>
       <c r="F35" s="3">
@@ -2467,10 +2467,10 @@
         <v>33</v>
       </c>
       <c r="D36" s="3" t="n">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="E36" s="3" t="n">
-        <v>0.19</v>
+        <v>0.23</v>
       </c>
       <c r="F36" s="3">
         <f>IF(B36:B244="common", 4, IF(B36:B244="uncommon", 3, IF(B36:B244="rare", 0.792892156862745, 1)))</f>
@@ -2520,7 +2520,7 @@
         <v>46</v>
       </c>
       <c r="D37" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06</v>
       </c>
       <c r="E37" s="3" t="n">
         <v>0.13</v>
@@ -2573,7 +2573,7 @@
         <v>33</v>
       </c>
       <c r="D38" s="3" t="n">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="E38" s="3" t="n">
         <v>0.18</v>
@@ -2626,10 +2626,10 @@
         <v>46</v>
       </c>
       <c r="D39" s="3" t="n">
-        <v>0.08</v>
+        <v>0.06</v>
       </c>
       <c r="E39" s="3" t="n">
-        <v>0.14</v>
+        <v>0.16</v>
       </c>
       <c r="F39" s="3">
         <f>IF(B39:B247="common", 4, IF(B39:B247="uncommon", 3, IF(B39:B247="rare", 0.792892156862745, 1)))</f>
@@ -2682,7 +2682,7 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="E40" s="3" t="n">
-        <v>0.62</v>
+        <v>0.66</v>
       </c>
       <c r="F40" s="3">
         <f>IF(B40:B248="common", 4, IF(B40:B248="uncommon", 3, IF(B40:B248="rare", 0.792892156862745, 1)))</f>
@@ -2735,7 +2735,7 @@
         <v>0.09</v>
       </c>
       <c r="E41" s="3" t="n">
-        <v>0.61</v>
+        <v>0.64</v>
       </c>
       <c r="F41" s="3">
         <f>IF(B41:B249="common", 4, IF(B41:B249="uncommon", 3, IF(B41:B249="rare", 0.792892156862745, 1)))</f>
@@ -2785,7 +2785,7 @@
         <v>248</v>
       </c>
       <c r="D42" s="3" t="n">
-        <v>3.18</v>
+        <v>3.26</v>
       </c>
       <c r="E42" s="3" t="inlineStr"/>
       <c r="F42" s="3">
@@ -2836,10 +2836,10 @@
         <v>33</v>
       </c>
       <c r="D43" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.09</v>
       </c>
       <c r="E43" s="3" t="n">
-        <v>0.16</v>
+        <v>0.14</v>
       </c>
       <c r="F43" s="3">
         <f>IF(B43:B251="common", 4, IF(B43:B251="uncommon", 3, IF(B43:B251="rare", 0.792892156862745, 1)))</f>
@@ -2889,7 +2889,7 @@
         <v>46</v>
       </c>
       <c r="D44" s="3" t="n">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="E44" s="3" t="n">
         <v>0.14</v>
@@ -2942,10 +2942,10 @@
         <v>21</v>
       </c>
       <c r="D45" s="3" t="n">
-        <v>0.28</v>
+        <v>0.32</v>
       </c>
       <c r="E45" s="3" t="n">
-        <v>0.71</v>
+        <v>0.72</v>
       </c>
       <c r="F45" s="3">
         <f>IF(B45:B253="common", 4, IF(B45:B253="uncommon", 3, IF(B45:B253="rare", 0.792892156862745, 1)))</f>
@@ -2995,7 +2995,7 @@
         <v>21</v>
       </c>
       <c r="D46" s="3" t="n">
-        <v>0.3</v>
+        <v>0.28</v>
       </c>
       <c r="E46" s="3" t="inlineStr"/>
       <c r="F46" s="3">
@@ -3046,10 +3046,10 @@
         <v>21</v>
       </c>
       <c r="D47" s="3" t="n">
-        <v>0.13</v>
+        <v>0.11</v>
       </c>
       <c r="E47" s="3" t="n">
-        <v>0.87</v>
+        <v>0.88</v>
       </c>
       <c r="F47" s="3">
         <f>IF(B47:B255="common", 4, IF(B47:B255="uncommon", 3, IF(B47:B255="rare", 0.792892156862745, 1)))</f>
@@ -3099,10 +3099,10 @@
         <v>46</v>
       </c>
       <c r="D48" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06</v>
       </c>
       <c r="E48" s="3" t="n">
-        <v>0.15</v>
+        <v>0.16</v>
       </c>
       <c r="F48" s="3">
         <f>IF(B48:B256="common", 4, IF(B48:B256="uncommon", 3, IF(B48:B256="rare", 0.792892156862745, 1)))</f>
@@ -3152,10 +3152,10 @@
         <v>33</v>
       </c>
       <c r="D49" s="3" t="n">
-        <v>0.13</v>
+        <v>0.11</v>
       </c>
       <c r="E49" s="3" t="n">
-        <v>1.75</v>
+        <v>1.67</v>
       </c>
       <c r="F49" s="3">
         <f>IF(B49:B257="common", 4, IF(B49:B257="uncommon", 3, IF(B49:B257="rare", 0.792892156862745, 1)))</f>
@@ -3205,7 +3205,7 @@
         <v>188</v>
       </c>
       <c r="D50" s="3" t="n">
-        <v>20.09</v>
+        <v>20.11</v>
       </c>
       <c r="E50" s="3" t="inlineStr"/>
       <c r="F50" s="3">
@@ -3256,10 +3256,10 @@
         <v>21</v>
       </c>
       <c r="D51" s="3" t="n">
-        <v>0.31</v>
+        <v>0.32</v>
       </c>
       <c r="E51" s="3" t="n">
-        <v>1.41</v>
+        <v>1.37</v>
       </c>
       <c r="F51" s="3">
         <f>IF(B51:B259="common", 4, IF(B51:B259="uncommon", 3, IF(B51:B259="rare", 0.792892156862745, 1)))</f>
@@ -3312,7 +3312,7 @@
         <v>0.1</v>
       </c>
       <c r="E52" s="3" t="n">
-        <v>0.2</v>
+        <v>0.19</v>
       </c>
       <c r="F52" s="3">
         <f>IF(B52:B260="common", 4, IF(B52:B260="uncommon", 3, IF(B52:B260="rare", 0.792892156862745, 1)))</f>
@@ -3362,10 +3362,10 @@
         <v>46</v>
       </c>
       <c r="D53" s="3" t="n">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="E53" s="3" t="n">
-        <v>0.12</v>
+        <v>0.13</v>
       </c>
       <c r="F53" s="3">
         <f>IF(B53:B261="common", 4, IF(B53:B261="uncommon", 3, IF(B53:B261="rare", 0.792892156862745, 1)))</f>
@@ -3415,10 +3415,10 @@
         <v>33</v>
       </c>
       <c r="D54" s="3" t="n">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="E54" s="3" t="n">
-        <v>0.14</v>
+        <v>0.2</v>
       </c>
       <c r="F54" s="3">
         <f>IF(B54:B262="common", 4, IF(B54:B262="uncommon", 3, IF(B54:B262="rare", 0.792892156862745, 1)))</f>
@@ -3471,7 +3471,7 @@
         <v>0.12</v>
       </c>
       <c r="E55" s="3" t="n">
-        <v>0.32</v>
+        <v>0.3</v>
       </c>
       <c r="F55" s="3">
         <f>IF(B55:B263="common", 4, IF(B55:B263="uncommon", 3, IF(B55:B263="rare", 0.792892156862745, 1)))</f>
@@ -3524,7 +3524,7 @@
         <v>0.06</v>
       </c>
       <c r="E56" s="3" t="n">
-        <v>0.15</v>
+        <v>0.16</v>
       </c>
       <c r="F56" s="3">
         <f>IF(B56:B264="common", 4, IF(B56:B264="uncommon", 3, IF(B56:B264="rare", 0.792892156862745, 1)))</f>
@@ -3627,10 +3627,10 @@
         <v>21</v>
       </c>
       <c r="D58" s="3" t="n">
-        <v>0.14</v>
+        <v>0.13</v>
       </c>
       <c r="E58" s="3" t="n">
-        <v>1.18</v>
+        <v>1.16</v>
       </c>
       <c r="F58" s="3">
         <f>IF(B58:B266="common", 4, IF(B58:B266="uncommon", 3, IF(B58:B266="rare", 0.792892156862745, 1)))</f>
@@ -3680,10 +3680,10 @@
         <v>33</v>
       </c>
       <c r="D59" s="3" t="n">
-        <v>0.21</v>
+        <v>0.14</v>
       </c>
       <c r="E59" s="3" t="n">
-        <v>1.28</v>
+        <v>1.14</v>
       </c>
       <c r="F59" s="3">
         <f>IF(B59:B267="common", 4, IF(B59:B267="uncommon", 3, IF(B59:B267="rare", 0.792892156862745, 1)))</f>
@@ -3786,7 +3786,7 @@
         <v>248</v>
       </c>
       <c r="D61" s="3" t="n">
-        <v>5.88</v>
+        <v>5.56</v>
       </c>
       <c r="E61" s="3" t="inlineStr"/>
       <c r="F61" s="3">
@@ -3837,7 +3837,7 @@
         <v>225</v>
       </c>
       <c r="D62" s="3" t="n">
-        <v>13.84</v>
+        <v>13.57</v>
       </c>
       <c r="E62" s="3" t="inlineStr"/>
       <c r="F62" s="3">
@@ -3888,10 +3888,10 @@
         <v>46</v>
       </c>
       <c r="D63" s="3" t="n">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="E63" s="3" t="n">
-        <v>0.12</v>
+        <v>0.13</v>
       </c>
       <c r="F63" s="3">
         <f>IF(B63:B271="common", 4, IF(B63:B271="uncommon", 3, IF(B63:B271="rare", 0.792892156862745, 1)))</f>
@@ -3941,10 +3941,10 @@
         <v>33</v>
       </c>
       <c r="D64" s="3" t="n">
-        <v>0.08</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="E64" s="3" t="n">
-        <v>1.55</v>
+        <v>1.5</v>
       </c>
       <c r="F64" s="3">
         <f>IF(B64:B272="common", 4, IF(B64:B272="uncommon", 3, IF(B64:B272="rare", 0.792892156862745, 1)))</f>
@@ -3997,7 +3997,7 @@
         <v>0.05</v>
       </c>
       <c r="E65" s="3" t="n">
-        <v>0.15</v>
+        <v>0.14</v>
       </c>
       <c r="F65" s="3">
         <f>IF(B65:B273="common", 4, IF(B65:B273="uncommon", 3, IF(B65:B273="rare", 0.792892156862745, 1)))</f>
@@ -4047,10 +4047,10 @@
         <v>33</v>
       </c>
       <c r="D66" s="3" t="n">
-        <v>0.08</v>
+        <v>0.06</v>
       </c>
       <c r="E66" s="3" t="n">
-        <v>0.11</v>
+        <v>0.12</v>
       </c>
       <c r="F66" s="3">
         <f>IF(B66:B274="common", 4, IF(B66:B274="uncommon", 3, IF(B66:B274="rare", 0.792892156862745, 1)))</f>
@@ -4100,10 +4100,10 @@
         <v>21</v>
       </c>
       <c r="D67" s="3" t="n">
-        <v>0.26</v>
+        <v>0.2</v>
       </c>
       <c r="E67" s="3" t="n">
-        <v>1.28</v>
+        <v>1.08</v>
       </c>
       <c r="F67" s="3">
         <f>IF(B67:B275="common", 4, IF(B67:B275="uncommon", 3, IF(B67:B275="rare", 0.792892156862745, 1)))</f>
@@ -4156,7 +4156,7 @@
         <v>0.08</v>
       </c>
       <c r="E68" s="3" t="n">
-        <v>0.17</v>
+        <v>0.18</v>
       </c>
       <c r="F68" s="3">
         <f>IF(B68:B276="common", 4, IF(B68:B276="uncommon", 3, IF(B68:B276="rare", 0.792892156862745, 1)))</f>
@@ -4206,10 +4206,10 @@
         <v>21</v>
       </c>
       <c r="D69" s="3" t="n">
-        <v>0.29</v>
+        <v>0.3</v>
       </c>
       <c r="E69" s="3" t="n">
-        <v>1.84</v>
+        <v>2</v>
       </c>
       <c r="F69" s="3">
         <f>IF(B69:B277="common", 4, IF(B69:B277="uncommon", 3, IF(B69:B277="rare", 0.792892156862745, 1)))</f>
@@ -4259,10 +4259,10 @@
         <v>46</v>
       </c>
       <c r="D70" s="3" t="n">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="E70" s="3" t="n">
-        <v>0.15</v>
+        <v>0.18</v>
       </c>
       <c r="F70" s="3">
         <f>IF(B70:B278="common", 4, IF(B70:B278="uncommon", 3, IF(B70:B278="rare", 0.792892156862745, 1)))</f>
@@ -4312,10 +4312,10 @@
         <v>33</v>
       </c>
       <c r="D71" s="3" t="n">
-        <v>0.13</v>
+        <v>0.12</v>
       </c>
       <c r="E71" s="3" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.85</v>
       </c>
       <c r="F71" s="3">
         <f>IF(B71:B279="common", 4, IF(B71:B279="uncommon", 3, IF(B71:B279="rare", 0.792892156862745, 1)))</f>
@@ -4365,7 +4365,7 @@
         <v>248</v>
       </c>
       <c r="D72" s="3" t="n">
-        <v>5.54</v>
+        <v>4.99</v>
       </c>
       <c r="E72" s="3" t="inlineStr"/>
       <c r="F72" s="3">
@@ -4416,7 +4416,7 @@
         <v>225</v>
       </c>
       <c r="D73" s="3" t="n">
-        <v>13.18</v>
+        <v>12.98</v>
       </c>
       <c r="E73" s="3" t="inlineStr"/>
       <c r="F73" s="3">
@@ -4467,10 +4467,10 @@
         <v>33</v>
       </c>
       <c r="D74" s="3" t="n">
-        <v>0.09</v>
+        <v>0.08</v>
       </c>
       <c r="E74" s="3" t="n">
-        <v>0.17</v>
+        <v>0.2</v>
       </c>
       <c r="F74" s="3">
         <f>IF(B74:B282="common", 4, IF(B74:B282="uncommon", 3, IF(B74:B282="rare", 0.792892156862745, 1)))</f>
@@ -4626,7 +4626,7 @@
         <v>33</v>
       </c>
       <c r="D77" s="3" t="n">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="E77" s="3" t="n">
         <v>0.16</v>
@@ -4679,7 +4679,7 @@
         <v>90</v>
       </c>
       <c r="D78" s="3" t="n">
-        <v>0.61</v>
+        <v>0.63</v>
       </c>
       <c r="E78" s="3" t="inlineStr"/>
       <c r="F78" s="3">
@@ -4730,7 +4730,7 @@
         <v>248</v>
       </c>
       <c r="D79" s="3" t="n">
-        <v>5.37</v>
+        <v>5.26</v>
       </c>
       <c r="E79" s="3" t="inlineStr"/>
       <c r="F79" s="3">
@@ -4784,7 +4784,7 @@
         <v>0.12</v>
       </c>
       <c r="E80" s="3" t="n">
-        <v>0.64</v>
+        <v>0.6</v>
       </c>
       <c r="F80" s="3">
         <f>IF(B80:B288="common", 4, IF(B80:B288="uncommon", 3, IF(B80:B288="rare", 0.792892156862745, 1)))</f>
@@ -4837,7 +4837,7 @@
         <v>0.06</v>
       </c>
       <c r="E81" s="3" t="n">
-        <v>0.13</v>
+        <v>0.16</v>
       </c>
       <c r="F81" s="3">
         <f>IF(B81:B289="common", 4, IF(B81:B289="uncommon", 3, IF(B81:B289="rare", 0.792892156862745, 1)))</f>
@@ -4887,10 +4887,10 @@
         <v>46</v>
       </c>
       <c r="D82" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06</v>
       </c>
       <c r="E82" s="3" t="n">
-        <v>0.15</v>
+        <v>0.17</v>
       </c>
       <c r="F82" s="3">
         <f>IF(B82:B290="common", 4, IF(B82:B290="uncommon", 3, IF(B82:B290="rare", 0.792892156862745, 1)))</f>
@@ -4943,7 +4943,7 @@
         <v>0.05</v>
       </c>
       <c r="E83" s="3" t="n">
-        <v>0.12</v>
+        <v>0.14</v>
       </c>
       <c r="F83" s="3">
         <f>IF(B83:B291="common", 4, IF(B83:B291="uncommon", 3, IF(B83:B291="rare", 0.792892156862745, 1)))</f>
@@ -4993,10 +4993,10 @@
         <v>21</v>
       </c>
       <c r="D84" s="3" t="n">
-        <v>0.16</v>
+        <v>0.15</v>
       </c>
       <c r="E84" s="3" t="n">
-        <v>0.89</v>
+        <v>0.93</v>
       </c>
       <c r="F84" s="3">
         <f>IF(B84:B292="common", 4, IF(B84:B292="uncommon", 3, IF(B84:B292="rare", 0.792892156862745, 1)))</f>
@@ -5046,10 +5046,10 @@
         <v>33</v>
       </c>
       <c r="D85" s="3" t="n">
-        <v>0.13</v>
+        <v>0.12</v>
       </c>
       <c r="E85" s="3" t="n">
-        <v>0.23</v>
+        <v>0.21</v>
       </c>
       <c r="F85" s="3">
         <f>IF(B85:B293="common", 4, IF(B85:B293="uncommon", 3, IF(B85:B293="rare", 0.792892156862745, 1)))</f>
@@ -5102,7 +5102,7 @@
         <v>0.11</v>
       </c>
       <c r="E86" s="3" t="n">
-        <v>1.24</v>
+        <v>1.2</v>
       </c>
       <c r="F86" s="3">
         <f>IF(B86:B294="common", 4, IF(B86:B294="uncommon", 3, IF(B86:B294="rare", 0.792892156862745, 1)))</f>
@@ -5152,10 +5152,10 @@
         <v>33</v>
       </c>
       <c r="D87" s="3" t="n">
-        <v>0.12</v>
+        <v>0.1</v>
       </c>
       <c r="E87" s="3" t="n">
-        <v>1.16</v>
+        <v>1.22</v>
       </c>
       <c r="F87" s="3">
         <f>IF(B87:B295="common", 4, IF(B87:B295="uncommon", 3, IF(B87:B295="rare", 0.792892156862745, 1)))</f>
@@ -5205,7 +5205,7 @@
         <v>46</v>
       </c>
       <c r="D88" s="3" t="n">
-        <v>0.06</v>
+        <v>0.04</v>
       </c>
       <c r="E88" s="3" t="n">
         <v>0.14</v>
@@ -5258,10 +5258,10 @@
         <v>33</v>
       </c>
       <c r="D89" s="3" t="n">
-        <v>0.08</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="E89" s="3" t="n">
-        <v>1.18</v>
+        <v>1.05</v>
       </c>
       <c r="F89" s="3">
         <f>IF(B89:B297="common", 4, IF(B89:B297="uncommon", 3, IF(B89:B297="rare", 0.792892156862745, 1)))</f>
@@ -5314,7 +5314,7 @@
         <v>0.1</v>
       </c>
       <c r="E90" s="3" t="n">
-        <v>0.33</v>
+        <v>0.28</v>
       </c>
       <c r="F90" s="3">
         <f>IF(B90:B298="common", 4, IF(B90:B298="uncommon", 3, IF(B90:B298="rare", 0.792892156862745, 1)))</f>
@@ -5364,7 +5364,7 @@
         <v>188</v>
       </c>
       <c r="D91" s="3" t="n">
-        <v>27.43</v>
+        <v>27.57</v>
       </c>
       <c r="E91" s="3" t="inlineStr"/>
       <c r="F91" s="3">
@@ -5415,10 +5415,10 @@
         <v>46</v>
       </c>
       <c r="D92" s="3" t="n">
-        <v>0.08</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="E92" s="3" t="n">
-        <v>0.16</v>
+        <v>0.2</v>
       </c>
       <c r="F92" s="3">
         <f>IF(B92:B300="common", 4, IF(B92:B300="uncommon", 3, IF(B92:B300="rare", 0.792892156862745, 1)))</f>
@@ -5468,10 +5468,10 @@
         <v>21</v>
       </c>
       <c r="D93" s="3" t="n">
-        <v>0.2</v>
+        <v>0.18</v>
       </c>
       <c r="E93" s="3" t="n">
-        <v>2.15</v>
+        <v>2.12</v>
       </c>
       <c r="F93" s="3">
         <f>IF(B93:B301="common", 4, IF(B93:B301="uncommon", 3, IF(B93:B301="rare", 0.792892156862745, 1)))</f>
@@ -5521,7 +5521,7 @@
         <v>90</v>
       </c>
       <c r="D94" s="3" t="n">
-        <v>1.06</v>
+        <v>0.82</v>
       </c>
       <c r="E94" s="3" t="inlineStr"/>
       <c r="F94" s="3">
@@ -5572,7 +5572,7 @@
         <v>248</v>
       </c>
       <c r="D95" s="3" t="n">
-        <v>4.34</v>
+        <v>4.23</v>
       </c>
       <c r="E95" s="3" t="inlineStr"/>
       <c r="F95" s="3">
@@ -5626,7 +5626,7 @@
         <v>0.08</v>
       </c>
       <c r="E96" s="3" t="n">
-        <v>1.3</v>
+        <v>1.26</v>
       </c>
       <c r="F96" s="3">
         <f>IF(B96:B304="common", 4, IF(B96:B304="uncommon", 3, IF(B96:B304="rare", 0.792892156862745, 1)))</f>
@@ -5676,10 +5676,10 @@
         <v>21</v>
       </c>
       <c r="D97" s="3" t="n">
-        <v>0.15</v>
+        <v>0.14</v>
       </c>
       <c r="E97" s="3" t="n">
-        <v>1.07</v>
+        <v>0.96</v>
       </c>
       <c r="F97" s="3">
         <f>IF(B97:B305="common", 4, IF(B97:B305="uncommon", 3, IF(B97:B305="rare", 0.792892156862745, 1)))</f>
@@ -5729,10 +5729,10 @@
         <v>33</v>
       </c>
       <c r="D98" s="3" t="n">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="E98" s="3" t="n">
-        <v>0.19</v>
+        <v>0.2</v>
       </c>
       <c r="F98" s="3">
         <f>IF(B98:B306="common", 4, IF(B98:B306="uncommon", 3, IF(B98:B306="rare", 0.792892156862745, 1)))</f>
@@ -5782,10 +5782,10 @@
         <v>46</v>
       </c>
       <c r="D99" s="3" t="n">
-        <v>0.09</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="E99" s="3" t="n">
-        <v>1.82</v>
+        <v>1.64</v>
       </c>
       <c r="F99" s="3">
         <f>IF(B99:B307="common", 4, IF(B99:B307="uncommon", 3, IF(B99:B307="rare", 0.792892156862745, 1)))</f>
@@ -5835,7 +5835,7 @@
         <v>90</v>
       </c>
       <c r="D100" s="3" t="n">
-        <v>0.7</v>
+        <v>0.65</v>
       </c>
       <c r="E100" s="3" t="inlineStr"/>
       <c r="F100" s="3">
@@ -5886,7 +5886,7 @@
         <v>248</v>
       </c>
       <c r="D101" s="3" t="n">
-        <v>4.81</v>
+        <v>4.89</v>
       </c>
       <c r="E101" s="3" t="inlineStr"/>
       <c r="F101" s="3">
@@ -5937,10 +5937,10 @@
         <v>33</v>
       </c>
       <c r="D102" s="3" t="n">
-        <v>0.05</v>
+        <v>0.06</v>
       </c>
       <c r="E102" s="3" t="n">
-        <v>1.26</v>
+        <v>1.41</v>
       </c>
       <c r="F102" s="3">
         <f>IF(B102:B310="common", 4, IF(B102:B310="uncommon", 3, IF(B102:B310="rare", 0.792892156862745, 1)))</f>
@@ -5990,10 +5990,10 @@
         <v>46</v>
       </c>
       <c r="D103" s="3" t="n">
-        <v>0.08</v>
+        <v>0.06</v>
       </c>
       <c r="E103" s="3" t="n">
-        <v>0.12</v>
+        <v>0.13</v>
       </c>
       <c r="F103" s="3">
         <f>IF(B103:B311="common", 4, IF(B103:B311="uncommon", 3, IF(B103:B311="rare", 0.792892156862745, 1)))</f>
@@ -6043,7 +6043,7 @@
         <v>46</v>
       </c>
       <c r="D104" s="3" t="n">
-        <v>0.04</v>
+        <v>0.05</v>
       </c>
       <c r="E104" s="3" t="n">
         <v>0.16</v>
@@ -6099,7 +6099,7 @@
         <v>0.09</v>
       </c>
       <c r="E105" s="3" t="n">
-        <v>1.49</v>
+        <v>1.28</v>
       </c>
       <c r="F105" s="3">
         <f>IF(B105:B313="common", 4, IF(B105:B313="uncommon", 3, IF(B105:B313="rare", 0.792892156862745, 1)))</f>
@@ -6149,10 +6149,10 @@
         <v>33</v>
       </c>
       <c r="D106" s="3" t="n">
-        <v>0.15</v>
+        <v>0.16</v>
       </c>
       <c r="E106" s="3" t="n">
-        <v>0.49</v>
+        <v>0.5</v>
       </c>
       <c r="F106" s="3">
         <f>IF(B106:B314="common", 4, IF(B106:B314="uncommon", 3, IF(B106:B314="rare", 0.792892156862745, 1)))</f>
@@ -6202,7 +6202,7 @@
         <v>46</v>
       </c>
       <c r="D107" s="3" t="n">
-        <v>0.1</v>
+        <v>0.09</v>
       </c>
       <c r="E107" s="3" t="n">
         <v>0.14</v>
@@ -6258,7 +6258,7 @@
         <v>0.18</v>
       </c>
       <c r="E108" s="3" t="n">
-        <v>0.68</v>
+        <v>0.65</v>
       </c>
       <c r="F108" s="3">
         <f>IF(B108:B316="common", 4, IF(B108:B316="uncommon", 3, IF(B108:B316="rare", 0.792892156862745, 1)))</f>
@@ -6308,7 +6308,7 @@
         <v>33</v>
       </c>
       <c r="D109" s="3" t="n">
-        <v>0.06</v>
+        <v>0.08</v>
       </c>
       <c r="E109" s="3" t="n">
         <v>0.17</v>
@@ -6361,7 +6361,7 @@
         <v>188</v>
       </c>
       <c r="D110" s="3" t="n">
-        <v>9.800000000000001</v>
+        <v>9.869999999999999</v>
       </c>
       <c r="E110" s="3" t="inlineStr"/>
       <c r="F110" s="3">
@@ -6415,7 +6415,7 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="E111" s="3" t="n">
-        <v>0.14</v>
+        <v>0.13</v>
       </c>
       <c r="F111" s="3">
         <f>IF(B111:B319="common", 4, IF(B111:B319="uncommon", 3, IF(B111:B319="rare", 0.792892156862745, 1)))</f>
@@ -6465,10 +6465,10 @@
         <v>46</v>
       </c>
       <c r="D112" s="3" t="n">
-        <v>0.09</v>
+        <v>0.08</v>
       </c>
       <c r="E112" s="3" t="n">
-        <v>0.16</v>
+        <v>0.19</v>
       </c>
       <c r="F112" s="3">
         <f>IF(B112:B320="common", 4, IF(B112:B320="uncommon", 3, IF(B112:B320="rare", 0.792892156862745, 1)))</f>
@@ -6518,10 +6518,10 @@
         <v>46</v>
       </c>
       <c r="D113" s="3" t="n">
-        <v>0.08</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="E113" s="3" t="n">
-        <v>1.06</v>
+        <v>0.96</v>
       </c>
       <c r="F113" s="3">
         <f>IF(B113:B321="common", 4, IF(B113:B321="uncommon", 3, IF(B113:B321="rare", 0.792892156862745, 1)))</f>
@@ -6571,10 +6571,10 @@
         <v>46</v>
       </c>
       <c r="D114" s="3" t="n">
-        <v>0.08</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="E114" s="3" t="n">
-        <v>0.14</v>
+        <v>0.13</v>
       </c>
       <c r="F114" s="3">
         <f>IF(B114:B322="common", 4, IF(B114:B322="uncommon", 3, IF(B114:B322="rare", 0.792892156862745, 1)))</f>
@@ -6627,7 +6627,7 @@
         <v>0.09</v>
       </c>
       <c r="E115" s="3" t="n">
-        <v>0.13</v>
+        <v>0.18</v>
       </c>
       <c r="F115" s="3">
         <f>IF(B115:B323="common", 4, IF(B115:B323="uncommon", 3, IF(B115:B323="rare", 0.792892156862745, 1)))</f>
@@ -6677,7 +6677,7 @@
         <v>46</v>
       </c>
       <c r="D116" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06</v>
       </c>
       <c r="E116" s="3" t="n">
         <v>0.12</v>
@@ -6730,10 +6730,10 @@
         <v>21</v>
       </c>
       <c r="D117" s="3" t="n">
-        <v>0.14</v>
+        <v>0.13</v>
       </c>
       <c r="E117" s="3" t="n">
-        <v>0.59</v>
+        <v>0.6</v>
       </c>
       <c r="F117" s="3">
         <f>IF(B117:B325="common", 4, IF(B117:B325="uncommon", 3, IF(B117:B325="rare", 0.792892156862745, 1)))</f>
@@ -6786,7 +6786,7 @@
         <v>0.08</v>
       </c>
       <c r="E118" s="3" t="n">
-        <v>0.18</v>
+        <v>0.17</v>
       </c>
       <c r="F118" s="3">
         <f>IF(B118:B326="common", 4, IF(B118:B326="uncommon", 3, IF(B118:B326="rare", 0.792892156862745, 1)))</f>
@@ -6839,7 +6839,7 @@
         <v>0.1</v>
       </c>
       <c r="E119" s="3" t="n">
-        <v>2.18</v>
+        <v>2.61</v>
       </c>
       <c r="F119" s="3">
         <f>IF(B119:B327="common", 4, IF(B119:B327="uncommon", 3, IF(B119:B327="rare", 0.792892156862745, 1)))</f>
@@ -6889,7 +6889,7 @@
         <v>90</v>
       </c>
       <c r="D120" s="3" t="n">
-        <v>6.41</v>
+        <v>6.32</v>
       </c>
       <c r="E120" s="3" t="inlineStr"/>
       <c r="F120" s="3">
@@ -6940,7 +6940,7 @@
         <v>248</v>
       </c>
       <c r="D121" s="3" t="n">
-        <v>18.51</v>
+        <v>17.12</v>
       </c>
       <c r="E121" s="3" t="inlineStr"/>
       <c r="F121" s="3">
@@ -6991,7 +6991,7 @@
         <v>154</v>
       </c>
       <c r="D122" s="3" t="n">
-        <v>12.65</v>
+        <v>12</v>
       </c>
       <c r="E122" s="3" t="inlineStr"/>
       <c r="F122" s="3">
@@ -7042,7 +7042,7 @@
         <v>90</v>
       </c>
       <c r="D123" s="3" t="n">
-        <v>10.27</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="E123" s="3" t="inlineStr"/>
       <c r="F123" s="3">
@@ -7093,10 +7093,10 @@
         <v>21</v>
       </c>
       <c r="D124" s="3" t="n">
-        <v>0.55</v>
+        <v>0.47</v>
       </c>
       <c r="E124" s="3" t="n">
-        <v>1.58</v>
+        <v>1.46</v>
       </c>
       <c r="F124" s="3">
         <f>IF(B124:B332="common", 4, IF(B124:B332="uncommon", 3, IF(B124:B332="rare", 0.792892156862745, 1)))</f>
@@ -7149,7 +7149,7 @@
         <v>0.24</v>
       </c>
       <c r="E125" s="3" t="n">
-        <v>0.74</v>
+        <v>0.63</v>
       </c>
       <c r="F125" s="3">
         <f>IF(B125:B333="common", 4, IF(B125:B333="uncommon", 3, IF(B125:B333="rare", 0.792892156862745, 1)))</f>
@@ -7199,10 +7199,10 @@
         <v>21</v>
       </c>
       <c r="D126" s="3" t="n">
-        <v>0.13</v>
+        <v>0.12</v>
       </c>
       <c r="E126" s="3" t="n">
-        <v>0.57</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="F126" s="3">
         <f>IF(B126:B334="common", 4, IF(B126:B334="uncommon", 3, IF(B126:B334="rare", 0.792892156862745, 1)))</f>
@@ -7252,7 +7252,7 @@
         <v>188</v>
       </c>
       <c r="D127" s="3" t="n">
-        <v>5.65</v>
+        <v>5.29</v>
       </c>
       <c r="E127" s="3" t="inlineStr"/>
       <c r="F127" s="3">
@@ -7303,10 +7303,10 @@
         <v>33</v>
       </c>
       <c r="D128" s="3" t="n">
-        <v>0.09</v>
+        <v>0.08</v>
       </c>
       <c r="E128" s="3" t="n">
-        <v>0.17</v>
+        <v>0.19</v>
       </c>
       <c r="F128" s="3">
         <f>IF(B128:B336="common", 4, IF(B128:B336="uncommon", 3, IF(B128:B336="rare", 0.792892156862745, 1)))</f>
@@ -7359,7 +7359,7 @@
         <v>0.16</v>
       </c>
       <c r="E129" s="3" t="n">
-        <v>0.76</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="F129" s="3">
         <f>IF(B129:B337="common", 4, IF(B129:B337="uncommon", 3, IF(B129:B337="rare", 0.792892156862745, 1)))</f>
@@ -7409,7 +7409,7 @@
         <v>188</v>
       </c>
       <c r="D130" s="3" t="n">
-        <v>9.49</v>
+        <v>9.109999999999999</v>
       </c>
       <c r="E130" s="3" t="inlineStr"/>
       <c r="F130" s="3">
@@ -7463,7 +7463,7 @@
         <v>0.09</v>
       </c>
       <c r="E131" s="3" t="n">
-        <v>0.17</v>
+        <v>0.19</v>
       </c>
       <c r="F131" s="3">
         <f>IF(B131:B339="common", 4, IF(B131:B339="uncommon", 3, IF(B131:B339="rare", 0.792892156862745, 1)))</f>
@@ -7513,10 +7513,10 @@
         <v>46</v>
       </c>
       <c r="D132" s="3" t="n">
-        <v>0.12</v>
+        <v>0.13</v>
       </c>
       <c r="E132" s="3" t="n">
-        <v>1.67</v>
+        <v>1.46</v>
       </c>
       <c r="F132" s="3">
         <f>IF(B132:B340="common", 4, IF(B132:B340="uncommon", 3, IF(B132:B340="rare", 0.792892156862745, 1)))</f>
@@ -7569,7 +7569,7 @@
         <v>0.1</v>
       </c>
       <c r="E133" s="3" t="n">
-        <v>1.19</v>
+        <v>1.2</v>
       </c>
       <c r="F133" s="3">
         <f>IF(B133:B341="common", 4, IF(B133:B341="uncommon", 3, IF(B133:B341="rare", 0.792892156862745, 1)))</f>
@@ -7675,7 +7675,7 @@
         <v>0.05</v>
       </c>
       <c r="E135" s="3" t="n">
-        <v>0.17</v>
+        <v>0.16</v>
       </c>
       <c r="F135" s="3">
         <f>IF(B135:B343="common", 4, IF(B135:B343="uncommon", 3, IF(B135:B343="rare", 0.792892156862745, 1)))</f>
@@ -7725,7 +7725,7 @@
         <v>90</v>
       </c>
       <c r="D136" s="3" t="n">
-        <v>1.13</v>
+        <v>1.02</v>
       </c>
       <c r="E136" s="3" t="inlineStr"/>
       <c r="F136" s="3">
@@ -7776,7 +7776,7 @@
         <v>248</v>
       </c>
       <c r="D137" s="3" t="n">
-        <v>7.37</v>
+        <v>7.43</v>
       </c>
       <c r="E137" s="3" t="inlineStr"/>
       <c r="F137" s="3">
@@ -7827,7 +7827,7 @@
         <v>46</v>
       </c>
       <c r="D138" s="3" t="n">
-        <v>0.08</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="E138" s="3" t="n">
         <v>0.14</v>
@@ -7883,7 +7883,7 @@
         <v>0.09</v>
       </c>
       <c r="E139" s="3" t="n">
-        <v>1.84</v>
+        <v>1.69</v>
       </c>
       <c r="F139" s="3">
         <f>IF(B139:B347="common", 4, IF(B139:B347="uncommon", 3, IF(B139:B347="rare", 0.792892156862745, 1)))</f>
@@ -7933,7 +7933,7 @@
         <v>188</v>
       </c>
       <c r="D140" s="3" t="n">
-        <v>5.82</v>
+        <v>5.73</v>
       </c>
       <c r="E140" s="3" t="inlineStr"/>
       <c r="F140" s="3">
@@ -7984,10 +7984,10 @@
         <v>21</v>
       </c>
       <c r="D141" s="3" t="n">
-        <v>0.15</v>
+        <v>0.13</v>
       </c>
       <c r="E141" s="3" t="n">
-        <v>0.68</v>
+        <v>0.57</v>
       </c>
       <c r="F141" s="3">
         <f>IF(B141:B349="common", 4, IF(B141:B349="uncommon", 3, IF(B141:B349="rare", 0.792892156862745, 1)))</f>
@@ -8037,10 +8037,10 @@
         <v>33</v>
       </c>
       <c r="D142" s="3" t="n">
-        <v>0.09</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="E142" s="3" t="n">
-        <v>1.46</v>
+        <v>1.45</v>
       </c>
       <c r="F142" s="3">
         <f>IF(B142:B350="common", 4, IF(B142:B350="uncommon", 3, IF(B142:B350="rare", 0.792892156862745, 1)))</f>
@@ -8093,7 +8093,7 @@
         <v>0.05</v>
       </c>
       <c r="E143" s="3" t="n">
-        <v>0.13</v>
+        <v>0.15</v>
       </c>
       <c r="F143" s="3">
         <f>IF(B143:B351="common", 4, IF(B143:B351="uncommon", 3, IF(B143:B351="rare", 0.792892156862745, 1)))</f>
@@ -8146,7 +8146,7 @@
         <v>0.06</v>
       </c>
       <c r="E144" s="3" t="n">
-        <v>0.15</v>
+        <v>0.16</v>
       </c>
       <c r="F144" s="3">
         <f>IF(B144:B352="common", 4, IF(B144:B352="uncommon", 3, IF(B144:B352="rare", 0.792892156862745, 1)))</f>
@@ -8196,10 +8196,10 @@
         <v>33</v>
       </c>
       <c r="D145" s="3" t="n">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="E145" s="3" t="n">
-        <v>0.14</v>
+        <v>0.13</v>
       </c>
       <c r="F145" s="3">
         <f>IF(B145:B353="common", 4, IF(B145:B353="uncommon", 3, IF(B145:B353="rare", 0.792892156862745, 1)))</f>
@@ -8249,10 +8249,10 @@
         <v>33</v>
       </c>
       <c r="D146" s="3" t="n">
-        <v>0.09</v>
+        <v>0.08</v>
       </c>
       <c r="E146" s="3" t="n">
-        <v>0.19</v>
+        <v>0.18</v>
       </c>
       <c r="F146" s="3">
         <f>IF(B146:B354="common", 4, IF(B146:B354="uncommon", 3, IF(B146:B354="rare", 0.792892156862745, 1)))</f>
@@ -8302,10 +8302,10 @@
         <v>46</v>
       </c>
       <c r="D147" s="3" t="n">
-        <v>0.15</v>
+        <v>0.16</v>
       </c>
       <c r="E147" s="3" t="n">
-        <v>2.07</v>
+        <v>2.4</v>
       </c>
       <c r="F147" s="3">
         <f>IF(B147:B355="common", 4, IF(B147:B355="uncommon", 3, IF(B147:B355="rare", 0.792892156862745, 1)))</f>
@@ -8358,7 +8358,7 @@
         <v>0.1</v>
       </c>
       <c r="E148" s="3" t="n">
-        <v>0.23</v>
+        <v>0.28</v>
       </c>
       <c r="F148" s="3">
         <f>IF(B148:B356="common", 4, IF(B148:B356="uncommon", 3, IF(B148:B356="rare", 0.792892156862745, 1)))</f>
@@ -8408,10 +8408,10 @@
         <v>46</v>
       </c>
       <c r="D149" s="3" t="n">
-        <v>0.12</v>
+        <v>0.09</v>
       </c>
       <c r="E149" s="3" t="n">
-        <v>0.23</v>
+        <v>0.22</v>
       </c>
       <c r="F149" s="3">
         <f>IF(B149:B357="common", 4, IF(B149:B357="uncommon", 3, IF(B149:B357="rare", 0.792892156862745, 1)))</f>
@@ -8461,7 +8461,7 @@
         <v>188</v>
       </c>
       <c r="D150" s="3" t="n">
-        <v>24.97</v>
+        <v>24.78</v>
       </c>
       <c r="E150" s="3" t="inlineStr"/>
       <c r="F150" s="3">
@@ -8512,10 +8512,10 @@
         <v>33</v>
       </c>
       <c r="D151" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06</v>
       </c>
       <c r="E151" s="3" t="n">
-        <v>1.54</v>
+        <v>1.42</v>
       </c>
       <c r="F151" s="3">
         <f>IF(B151:B359="common", 4, IF(B151:B359="uncommon", 3, IF(B151:B359="rare", 0.792892156862745, 1)))</f>
@@ -8618,10 +8618,10 @@
         <v>46</v>
       </c>
       <c r="D153" s="3" t="n">
-        <v>0.13</v>
+        <v>0.12</v>
       </c>
       <c r="E153" s="3" t="n">
-        <v>1.85</v>
+        <v>1.79</v>
       </c>
       <c r="F153" s="3">
         <f>IF(B153:B361="common", 4, IF(B153:B361="uncommon", 3, IF(B153:B361="rare", 0.792892156862745, 1)))</f>
@@ -8671,7 +8671,7 @@
         <v>188</v>
       </c>
       <c r="D154" s="3" t="n">
-        <v>17.04</v>
+        <v>16.93</v>
       </c>
       <c r="E154" s="3" t="inlineStr"/>
       <c r="F154" s="3">
@@ -8722,10 +8722,10 @@
         <v>33</v>
       </c>
       <c r="D155" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06</v>
       </c>
       <c r="E155" s="3" t="n">
-        <v>0.16</v>
+        <v>0.17</v>
       </c>
       <c r="F155" s="3">
         <f>IF(B155:B363="common", 4, IF(B155:B363="uncommon", 3, IF(B155:B363="rare", 0.792892156862745, 1)))</f>
@@ -8778,7 +8778,7 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="E156" s="3" t="n">
-        <v>0.14</v>
+        <v>0.12</v>
       </c>
       <c r="F156" s="3">
         <f>IF(B156:B364="common", 4, IF(B156:B364="uncommon", 3, IF(B156:B364="rare", 0.792892156862745, 1)))</f>
@@ -8831,7 +8831,7 @@
         <v>0.06</v>
       </c>
       <c r="E157" s="3" t="n">
-        <v>0.13</v>
+        <v>0.12</v>
       </c>
       <c r="F157" s="3">
         <f>IF(B157:B365="common", 4, IF(B157:B365="uncommon", 3, IF(B157:B365="rare", 0.792892156862745, 1)))</f>
@@ -8881,7 +8881,7 @@
         <v>33</v>
       </c>
       <c r="D158" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06</v>
       </c>
       <c r="E158" s="3" t="n">
         <v>0.16</v>
@@ -8934,10 +8934,10 @@
         <v>33</v>
       </c>
       <c r="D159" s="3" t="n">
-        <v>0.12</v>
+        <v>0.13</v>
       </c>
       <c r="E159" s="3" t="n">
-        <v>0.77</v>
+        <v>0.8</v>
       </c>
       <c r="F159" s="3">
         <f>IF(B159:B367="common", 4, IF(B159:B367="uncommon", 3, IF(B159:B367="rare", 0.792892156862745, 1)))</f>
@@ -8987,10 +8987,10 @@
         <v>46</v>
       </c>
       <c r="D160" s="3" t="n">
-        <v>0.08</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="E160" s="3" t="n">
-        <v>0.2</v>
+        <v>0.19</v>
       </c>
       <c r="F160" s="3">
         <f>IF(B160:B368="common", 4, IF(B160:B368="uncommon", 3, IF(B160:B368="rare", 0.792892156862745, 1)))</f>
@@ -9040,7 +9040,7 @@
         <v>188</v>
       </c>
       <c r="D161" s="3" t="n">
-        <v>18.79</v>
+        <v>18.6</v>
       </c>
       <c r="E161" s="3" t="inlineStr"/>
       <c r="F161" s="3">
@@ -9091,10 +9091,10 @@
         <v>21</v>
       </c>
       <c r="D162" s="3" t="n">
-        <v>0.13</v>
+        <v>0.12</v>
       </c>
       <c r="E162" s="3" t="n">
-        <v>1.19</v>
+        <v>1.21</v>
       </c>
       <c r="F162" s="3">
         <f>IF(B162:B370="common", 4, IF(B162:B370="uncommon", 3, IF(B162:B370="rare", 0.792892156862745, 1)))</f>
@@ -9144,10 +9144,10 @@
         <v>33</v>
       </c>
       <c r="D163" s="3" t="n">
-        <v>0.08</v>
+        <v>0.09</v>
       </c>
       <c r="E163" s="3" t="n">
-        <v>0.14</v>
+        <v>0.13</v>
       </c>
       <c r="F163" s="3">
         <f>IF(B163:B371="common", 4, IF(B163:B371="uncommon", 3, IF(B163:B371="rare", 0.792892156862745, 1)))</f>
@@ -9197,10 +9197,10 @@
         <v>33</v>
       </c>
       <c r="D164" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06</v>
       </c>
       <c r="E164" s="3" t="n">
-        <v>0.15</v>
+        <v>0.14</v>
       </c>
       <c r="F164" s="3">
         <f>IF(B164:B372="common", 4, IF(B164:B372="uncommon", 3, IF(B164:B372="rare", 0.792892156862745, 1)))</f>
@@ -9253,7 +9253,7 @@
         <v>0.05</v>
       </c>
       <c r="E165" s="3" t="n">
-        <v>0.1</v>
+        <v>0.16</v>
       </c>
       <c r="F165" s="3">
         <f>IF(B165:B373="common", 4, IF(B165:B373="uncommon", 3, IF(B165:B373="rare", 0.792892156862745, 1)))</f>
@@ -9303,10 +9303,10 @@
         <v>33</v>
       </c>
       <c r="D166" s="3" t="n">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="E166" s="3" t="n">
-        <v>0.15</v>
+        <v>0.19</v>
       </c>
       <c r="F166" s="3">
         <f>IF(B166:B374="common", 4, IF(B166:B374="uncommon", 3, IF(B166:B374="rare", 0.792892156862745, 1)))</f>
@@ -9356,10 +9356,10 @@
         <v>46</v>
       </c>
       <c r="D167" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06</v>
       </c>
       <c r="E167" s="3" t="n">
-        <v>0.13</v>
+        <v>0.12</v>
       </c>
       <c r="F167" s="3">
         <f>IF(B167:B375="common", 4, IF(B167:B375="uncommon", 3, IF(B167:B375="rare", 0.792892156862745, 1)))</f>
@@ -9409,10 +9409,10 @@
         <v>33</v>
       </c>
       <c r="D168" s="3" t="n">
-        <v>0.12</v>
+        <v>0.11</v>
       </c>
       <c r="E168" s="3" t="n">
-        <v>0.98</v>
+        <v>0.9</v>
       </c>
       <c r="F168" s="3">
         <f>IF(B168:B376="common", 4, IF(B168:B376="uncommon", 3, IF(B168:B376="rare", 0.792892156862745, 1)))</f>
@@ -9462,7 +9462,7 @@
         <v>46</v>
       </c>
       <c r="D169" s="3" t="n">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="E169" s="3" t="n">
         <v>0.17</v>
@@ -9518,7 +9518,7 @@
         <v>0.05</v>
       </c>
       <c r="E170" s="3" t="n">
-        <v>0.16</v>
+        <v>0.15</v>
       </c>
       <c r="F170" s="3">
         <f>IF(B170:B378="common", 4, IF(B170:B378="uncommon", 3, IF(B170:B378="rare", 0.792892156862745, 1)))</f>
@@ -9568,10 +9568,10 @@
         <v>33</v>
       </c>
       <c r="D171" s="3" t="n">
-        <v>0.09</v>
+        <v>0.08</v>
       </c>
       <c r="E171" s="3" t="n">
-        <v>2.65</v>
+        <v>2.37</v>
       </c>
       <c r="F171" s="3">
         <f>IF(B171:B379="common", 4, IF(B171:B379="uncommon", 3, IF(B171:B379="rare", 0.792892156862745, 1)))</f>
@@ -9621,10 +9621,10 @@
         <v>33</v>
       </c>
       <c r="D172" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06</v>
       </c>
       <c r="E172" s="3" t="n">
-        <v>0.15</v>
+        <v>0.18</v>
       </c>
       <c r="F172" s="3">
         <f>IF(B172:B380="common", 4, IF(B172:B380="uncommon", 3, IF(B172:B380="rare", 0.792892156862745, 1)))</f>
@@ -9674,10 +9674,10 @@
         <v>33</v>
       </c>
       <c r="D173" s="3" t="n">
-        <v>0.1</v>
+        <v>0.08</v>
       </c>
       <c r="E173" s="3" t="n">
-        <v>0.99</v>
+        <v>0.97</v>
       </c>
       <c r="F173" s="3">
         <f>IF(B173:B381="common", 4, IF(B173:B381="uncommon", 3, IF(B173:B381="rare", 0.792892156862745, 1)))</f>
@@ -9780,10 +9780,10 @@
         <v>46</v>
       </c>
       <c r="D175" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06</v>
       </c>
       <c r="E175" s="3" t="n">
-        <v>0.17</v>
+        <v>0.13</v>
       </c>
       <c r="F175" s="3">
         <f>IF(B175:B383="common", 4, IF(B175:B383="uncommon", 3, IF(B175:B383="rare", 0.792892156862745, 1)))</f>
@@ -9833,10 +9833,10 @@
         <v>33</v>
       </c>
       <c r="D176" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.05</v>
       </c>
       <c r="E176" s="3" t="n">
-        <v>0.17</v>
+        <v>0.15</v>
       </c>
       <c r="F176" s="3">
         <f>IF(B176:B384="common", 4, IF(B176:B384="uncommon", 3, IF(B176:B384="rare", 0.792892156862745, 1)))</f>
@@ -9886,10 +9886,10 @@
         <v>46</v>
       </c>
       <c r="D177" s="3" t="n">
-        <v>0.08</v>
+        <v>0.06</v>
       </c>
       <c r="E177" s="3" t="n">
-        <v>0.13</v>
+        <v>0.17</v>
       </c>
       <c r="F177" s="3">
         <f>IF(B177:B385="common", 4, IF(B177:B385="uncommon", 3, IF(B177:B385="rare", 0.792892156862745, 1)))</f>
@@ -9939,10 +9939,10 @@
         <v>33</v>
       </c>
       <c r="D178" s="3" t="n">
-        <v>0.13</v>
+        <v>0.12</v>
       </c>
       <c r="E178" s="3" t="n">
-        <v>1.22</v>
+        <v>1.18</v>
       </c>
       <c r="F178" s="3">
         <f>IF(B178:B386="common", 4, IF(B178:B386="uncommon", 3, IF(B178:B386="rare", 0.792892156862745, 1)))</f>
@@ -9992,10 +9992,10 @@
         <v>46</v>
       </c>
       <c r="D179" s="3" t="n">
-        <v>0.08</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="E179" s="3" t="n">
-        <v>0.83</v>
+        <v>1.07</v>
       </c>
       <c r="F179" s="3">
         <f>IF(B179:B387="common", 4, IF(B179:B387="uncommon", 3, IF(B179:B387="rare", 0.792892156862745, 1)))</f>
@@ -10045,7 +10045,7 @@
         <v>46</v>
       </c>
       <c r="D180" s="3" t="n">
-        <v>0.1</v>
+        <v>0.11</v>
       </c>
       <c r="E180" s="3" t="n">
         <v>0.18</v>
@@ -10098,7 +10098,7 @@
         <v>188</v>
       </c>
       <c r="D181" s="3" t="n">
-        <v>40</v>
+        <v>38.56</v>
       </c>
       <c r="E181" s="3" t="inlineStr"/>
       <c r="F181" s="3">
@@ -10152,7 +10152,7 @@
         <v>0.16</v>
       </c>
       <c r="E182" s="3" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.57</v>
       </c>
       <c r="F182" s="3">
         <f>IF(B182:B390="common", 4, IF(B182:B390="uncommon", 3, IF(B182:B390="rare", 0.792892156862745, 1)))</f>
@@ -10202,10 +10202,10 @@
         <v>46</v>
       </c>
       <c r="D183" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06</v>
       </c>
       <c r="E183" s="3" t="n">
-        <v>0.14</v>
+        <v>0.18</v>
       </c>
       <c r="F183" s="3">
         <f>IF(B183:B391="common", 4, IF(B183:B391="uncommon", 3, IF(B183:B391="rare", 0.792892156862745, 1)))</f>
@@ -10255,7 +10255,7 @@
         <v>154</v>
       </c>
       <c r="D184" s="3" t="n">
-        <v>2.85</v>
+        <v>2.19</v>
       </c>
       <c r="E184" s="3" t="inlineStr"/>
       <c r="F184" s="3">
@@ -10306,10 +10306,10 @@
         <v>46</v>
       </c>
       <c r="D185" s="3" t="n">
-        <v>0.05</v>
+        <v>0.06</v>
       </c>
       <c r="E185" s="3" t="n">
-        <v>0.14</v>
+        <v>0.17</v>
       </c>
       <c r="F185" s="3">
         <f>IF(B185:B393="common", 4, IF(B185:B393="uncommon", 3, IF(B185:B393="rare", 0.792892156862745, 1)))</f>
@@ -10359,7 +10359,7 @@
         <v>188</v>
       </c>
       <c r="D186" s="3" t="n">
-        <v>6.7</v>
+        <v>6.47</v>
       </c>
       <c r="E186" s="3" t="inlineStr"/>
       <c r="F186" s="3">
@@ -10413,7 +10413,7 @@
         <v>0.1</v>
       </c>
       <c r="E187" s="3" t="n">
-        <v>0.87</v>
+        <v>0.85</v>
       </c>
       <c r="F187" s="3">
         <f>IF(B187:B395="common", 4, IF(B187:B395="uncommon", 3, IF(B187:B395="rare", 0.792892156862745, 1)))</f>
@@ -10466,7 +10466,7 @@
         <v>0.06</v>
       </c>
       <c r="E188" s="3" t="n">
-        <v>0.11</v>
+        <v>0.15</v>
       </c>
       <c r="F188" s="3">
         <f>IF(B188:B396="common", 4, IF(B188:B396="uncommon", 3, IF(B188:B396="rare", 0.792892156862745, 1)))</f>
@@ -10516,10 +10516,10 @@
         <v>33</v>
       </c>
       <c r="D189" s="3" t="n">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="E189" s="3" t="n">
-        <v>0.14</v>
+        <v>0.17</v>
       </c>
       <c r="F189" s="3">
         <f>IF(B189:B397="common", 4, IF(B189:B397="uncommon", 3, IF(B189:B397="rare", 0.792892156862745, 1)))</f>
@@ -10569,10 +10569,10 @@
         <v>21</v>
       </c>
       <c r="D190" s="3" t="n">
-        <v>0.21</v>
+        <v>0.22</v>
       </c>
       <c r="E190" s="3" t="n">
-        <v>1.46</v>
+        <v>1.31</v>
       </c>
       <c r="F190" s="3">
         <f>IF(B190:B398="common", 4, IF(B190:B398="uncommon", 3, IF(B190:B398="rare", 0.792892156862745, 1)))</f>
@@ -10622,10 +10622,10 @@
         <v>33</v>
       </c>
       <c r="D191" s="3" t="n">
-        <v>0.09</v>
+        <v>0.08</v>
       </c>
       <c r="E191" s="3" t="n">
-        <v>0.17</v>
+        <v>0.2</v>
       </c>
       <c r="F191" s="3">
         <f>IF(B191:B399="common", 4, IF(B191:B399="uncommon", 3, IF(B191:B399="rare", 0.792892156862745, 1)))</f>
@@ -10675,10 +10675,10 @@
         <v>46</v>
       </c>
       <c r="D192" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06</v>
       </c>
       <c r="E192" s="3" t="n">
-        <v>0.13</v>
+        <v>0.17</v>
       </c>
       <c r="F192" s="3">
         <f>IF(B192:B400="common", 4, IF(B192:B400="uncommon", 3, IF(B192:B400="rare", 0.792892156862745, 1)))</f>
@@ -10728,7 +10728,7 @@
         <v>90</v>
       </c>
       <c r="D193" s="3" t="n">
-        <v>0.55</v>
+        <v>0.73</v>
       </c>
       <c r="E193" s="3" t="inlineStr"/>
       <c r="F193" s="3">
@@ -10779,7 +10779,7 @@
         <v>248</v>
       </c>
       <c r="D194" s="3" t="n">
-        <v>9.69</v>
+        <v>9.470000000000001</v>
       </c>
       <c r="E194" s="3" t="inlineStr"/>
       <c r="F194" s="3">
@@ -10830,7 +10830,7 @@
         <v>225</v>
       </c>
       <c r="D195" s="3" t="n">
-        <v>57.96</v>
+        <v>57.55</v>
       </c>
       <c r="E195" s="3" t="inlineStr"/>
       <c r="F195" s="3">
@@ -10934,7 +10934,7 @@
         <v>21</v>
       </c>
       <c r="D197" s="3" t="n">
-        <v>0.19</v>
+        <v>0.2</v>
       </c>
       <c r="E197" s="3" t="n">
         <v>0.77</v>
@@ -10990,7 +10990,7 @@
         <v>0.06</v>
       </c>
       <c r="E198" s="3" t="n">
-        <v>0.14</v>
+        <v>0.13</v>
       </c>
       <c r="F198" s="3">
         <f>IF(B198:B406="common", 4, IF(B198:B406="uncommon", 3, IF(B198:B406="rare", 0.792892156862745, 1)))</f>
@@ -11040,10 +11040,10 @@
         <v>46</v>
       </c>
       <c r="D199" s="3" t="n">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="E199" s="3" t="n">
-        <v>0.16</v>
+        <v>0.19</v>
       </c>
       <c r="F199" s="3">
         <f>IF(B199:B407="common", 4, IF(B199:B407="uncommon", 3, IF(B199:B407="rare", 0.792892156862745, 1)))</f>
@@ -11096,7 +11096,7 @@
         <v>0.1</v>
       </c>
       <c r="E200" s="3" t="n">
-        <v>0.27</v>
+        <v>0.25</v>
       </c>
       <c r="F200" s="3">
         <f>IF(B200:B408="common", 4, IF(B200:B408="uncommon", 3, IF(B200:B408="rare", 0.792892156862745, 1)))</f>
@@ -11146,7 +11146,7 @@
         <v>188</v>
       </c>
       <c r="D201" s="3" t="n">
-        <v>24.22</v>
+        <v>23.06</v>
       </c>
       <c r="E201" s="3" t="inlineStr"/>
       <c r="F201" s="3">
@@ -11250,10 +11250,10 @@
         <v>46</v>
       </c>
       <c r="D203" s="3" t="n">
-        <v>0.11</v>
+        <v>0.1</v>
       </c>
       <c r="E203" s="3" t="n">
-        <v>1.46</v>
+        <v>1.47</v>
       </c>
       <c r="F203" s="3">
         <f>IF(B203:B411="common", 4, IF(B203:B411="uncommon", 3, IF(B203:B411="rare", 0.792892156862745, 1)))</f>
@@ -11306,7 +11306,7 @@
         <v>0.13</v>
       </c>
       <c r="E204" s="3" t="n">
-        <v>0.75</v>
+        <v>0.74</v>
       </c>
       <c r="F204" s="3">
         <f>IF(B204:B412="common", 4, IF(B204:B412="uncommon", 3, IF(B204:B412="rare", 0.792892156862745, 1)))</f>
@@ -11356,7 +11356,7 @@
         <v>90</v>
       </c>
       <c r="D205" s="3" t="n">
-        <v>0.64</v>
+        <v>0.74</v>
       </c>
       <c r="E205" s="3" t="inlineStr"/>
       <c r="F205" s="3">
@@ -11407,7 +11407,7 @@
         <v>248</v>
       </c>
       <c r="D206" s="3" t="n">
-        <v>6.9</v>
+        <v>6.27</v>
       </c>
       <c r="E206" s="3" t="inlineStr"/>
       <c r="F206" s="3">
@@ -11458,7 +11458,7 @@
         <v>90</v>
       </c>
       <c r="D207" s="3" t="n">
-        <v>0.76</v>
+        <v>0.8</v>
       </c>
       <c r="E207" s="3" t="inlineStr"/>
       <c r="F207" s="3">
@@ -11509,7 +11509,7 @@
         <v>248</v>
       </c>
       <c r="D208" s="3" t="n">
-        <v>7.15</v>
+        <v>7.23</v>
       </c>
       <c r="E208" s="3" t="inlineStr"/>
       <c r="F208" s="3">
@@ -11560,7 +11560,7 @@
         <v>225</v>
       </c>
       <c r="D209" s="3" t="n">
-        <v>46.15</v>
+        <v>47.08</v>
       </c>
       <c r="E209" s="3" t="inlineStr"/>
       <c r="F209" s="3">
@@ -18298,7 +18298,7 @@
         </is>
       </c>
       <c r="B2" s="13" t="n">
-        <v>0.4304347826086957</v>
+        <v>0.4008695652173913</v>
       </c>
     </row>
     <row r="3">
@@ -18308,7 +18308,7 @@
         </is>
       </c>
       <c r="B3" s="13" t="n">
-        <v>0.4881818181818181</v>
+        <v>0.4536363636363635</v>
       </c>
     </row>
     <row r="4">
@@ -18318,7 +18318,7 @@
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>0.2016211484593838</v>
+        <v>0.1925595238095238</v>
       </c>
     </row>
     <row r="5">
@@ -18328,7 +18328,7 @@
         </is>
       </c>
       <c r="B5" s="13" t="n">
-        <v>5.329323789133571</v>
+        <v>5.212912706255096</v>
       </c>
     </row>
     <row r="6">
@@ -18368,7 +18368,7 @@
         </is>
       </c>
       <c r="B9" s="13" t="n">
-        <v>1.740372340425532</v>
+        <v>1.716223404255319</v>
       </c>
     </row>
     <row r="10">
@@ -18378,7 +18378,7 @@
         </is>
       </c>
       <c r="B10" s="13" t="n">
-        <v>1.954666666666667</v>
+        <v>1.917866666666667</v>
       </c>
     </row>
     <row r="11">
@@ -18388,7 +18388,7 @@
         </is>
       </c>
       <c r="B11" s="13" t="n">
-        <v>0.3157777777777778</v>
+        <v>0.3143333333333334</v>
       </c>
     </row>
     <row r="12">
@@ -18398,7 +18398,7 @@
         </is>
       </c>
       <c r="B12" s="13" t="n">
-        <v>0.1305844155844156</v>
+        <v>0.121038961038961</v>
       </c>
     </row>
     <row r="13">
@@ -18408,7 +18408,7 @@
         </is>
       </c>
       <c r="B13" s="13" t="n">
-        <v>0.5363709677419355</v>
+        <v>0.5255241935483871</v>
       </c>
     </row>
     <row r="14">
@@ -18438,7 +18438,7 @@
         </is>
       </c>
       <c r="B16" s="13" t="n">
-        <v>4.677772168196328</v>
+        <v>4.594986558842668</v>
       </c>
     </row>
     <row r="17">
@@ -18448,7 +18448,7 @@
         </is>
       </c>
       <c r="B17" s="13" t="n">
-        <v>11.12733370657979</v>
+        <v>10.85496471776104</v>
       </c>
     </row>
     <row r="18">
@@ -18458,7 +18458,7 @@
         </is>
       </c>
       <c r="B18" s="13" t="n">
-        <v>1.397333706579793</v>
+        <v>0.9649647177610419</v>
       </c>
     </row>
     <row r="19">
@@ -18468,7 +18468,7 @@
         </is>
       </c>
       <c r="B19" s="14" t="n">
-        <v>1.14361086398559</v>
+        <v>1.097569738904049</v>
       </c>
     </row>
     <row r="20">
@@ -18478,7 +18478,7 @@
         </is>
       </c>
       <c r="B20" s="15" t="n">
-        <v>0.1436108639855902</v>
+        <v>0.09756973890404863</v>
       </c>
     </row>
     <row r="21">

</xml_diff>